<commit_message>
📥 WeTravel: Reporting_Payments_WeTravel-539682-1778780011.xlsx (2026-05-14)
</commit_message>
<xml_diff>
--- a/reportes/Reporting_Payments_WeTravel.xlsx
+++ b/reportes/Reporting_Payments_WeTravel.xlsx
@@ -82,7 +82,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y23"/>
+  <dimension ref="A1:Y30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="29.4" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -104,8 +104,8 @@
     <col width="32.199999999999996" min="17" max="17" bestFit="1" customWidth="1"/>
     <col width="31.900000000000002" min="18" max="18" bestFit="1" customWidth="1"/>
     <col width="41.800000000000004" min="19" max="19" bestFit="1" customWidth="1"/>
-    <col width="135.3" min="20" max="20" bestFit="1" customWidth="1"/>
-    <col width="125.4" min="21" max="21" bestFit="1" customWidth="1"/>
+    <col width="255" min="20" max="20" bestFit="1" customWidth="1"/>
+    <col width="223.3" min="21" max="21" bestFit="1" customWidth="1"/>
     <col width="77.0" min="22" max="22" bestFit="1" customWidth="1"/>
     <col width="14.0" min="23" max="23" bestFit="1" customWidth="1"/>
     <col width="23.799999999999997" min="24" max="24" bestFit="1" customWidth="1"/>
@@ -242,21 +242,21 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:41</t>
+          <t>2026/05/13 04:18:31</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:43</t>
+          <t>2026/05/13 04:18:33</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>822740352219193810944</t>
+          <t>822743406261352546304</t>
         </is>
       </c>
       <c r="D2" s="0" t="n">
-        <v>81000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
@@ -280,7 +280,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="J2" s="0" t="n">
@@ -290,46 +290,46 @@
         <v>0.0</v>
       </c>
       <c r="L2" s="0" t="n">
-        <v>81000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M2" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N2" s="0" t="n">
-        <v>81000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O2" s="0" t="n">
-        <v>2754.0</v>
+        <v>433.5</v>
       </c>
       <c r="P2" s="0" t="n">
-        <v>814.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <v>77432.0</v>
+        <v>12185.0</v>
       </c>
       <c r="R2" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="V2" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W2" s="0"/>
@@ -347,21 +347,21 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:11</t>
+          <t>2026/05/13 03:36:03</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:12</t>
+          <t>2026/05/13 03:36:05</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>822740218587619794944</t>
+          <t>822743384884528578560</t>
         </is>
       </c>
       <c r="D3" s="0" t="n">
-        <v>25500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
@@ -385,7 +385,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>6624</t>
+          <t>7758</t>
         </is>
       </c>
       <c r="J3" s="0" t="n">
@@ -395,46 +395,46 @@
         <v>0.0</v>
       </c>
       <c r="L3" s="0" t="n">
-        <v>25500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M3" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N3" s="0" t="n">
-        <v>25500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O3" s="0" t="n">
-        <v>739.5</v>
+        <v>369.75</v>
       </c>
       <c r="P3" s="0" t="n">
-        <v>259.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q3" s="0" t="n">
-        <v>24501.5</v>
+        <v>12248.75</v>
       </c>
       <c r="R3" s="0" t="inlineStr">
         <is>
-          <t>MELB PEREZ SALDANA</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t>MELBA ASTRID PEREZ SALDAÑA</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="V3" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W3" s="0"/>
@@ -452,17 +452,17 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:10</t>
+          <t>2026/05/12 21:17:39</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:12</t>
+          <t>2026/05/12 21:17:41</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>822740202977192058880</t>
+          <t>822743194435830431744</t>
         </is>
       </c>
       <c r="D4" s="0" t="n">
@@ -557,17 +557,17 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:20</t>
+          <t>2026/05/12 19:10:30</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:22</t>
+          <t>2026/05/12 19:11:16</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>822738944267014664192</t>
+          <t>822743130440389902336</t>
         </is>
       </c>
       <c r="D5" s="0" t="n">
@@ -590,12 +590,12 @@
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t>6156</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J5" s="0" t="n">
@@ -624,27 +624,27 @@
       </c>
       <c r="R5" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas, Denisse Olivo</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V5" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W5" s="0"/>
@@ -662,21 +662,21 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/06 23:07:12</t>
+          <t>2026/05/12 18:19:51</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/06 23:07:12</t>
+          <t>2026/05/12 18:19:53</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>822738900913572839424</t>
+          <t>822743104942704197632</t>
         </is>
       </c>
       <c r="D6" s="0" t="n">
-        <v>20500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
@@ -690,15 +690,19 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t>transferencia</t>
-        </is>
-      </c>
-      <c r="I6" s="0"/>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>1709</t>
+        </is>
+      </c>
       <c r="J6" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -706,41 +710,41 @@
         <v>0.0</v>
       </c>
       <c r="L6" s="0" t="n">
-        <v>0.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M6" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N6" s="0" t="n">
-        <v>0.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O6" s="0" t="n">
-        <v>0.0</v>
+        <v>1305.0</v>
       </c>
       <c r="P6" s="0" t="n">
-        <v>0.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q6" s="0" t="n">
-        <v>0.0</v>
+        <v>43241.0</v>
       </c>
       <c r="R6" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>RAFAEL BELTRAN LOPEZ</t>
         </is>
       </c>
       <c r="S6" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>rbeltran1976@hotmail.com</t>
         </is>
       </c>
       <c r="T6" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com</t>
+          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
         </is>
       </c>
       <c r="U6" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern, María Patricia García Kern</t>
+          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
         </is>
       </c>
       <c r="V6" s="0" t="inlineStr">
@@ -763,21 +767,21 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:40</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:42</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>822735991480689651712</t>
+          <t>822742523051869483008</t>
         </is>
       </c>
       <c r="D7" s="0" t="n">
-        <v>45000.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
@@ -791,19 +795,15 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
-        </is>
-      </c>
-      <c r="I7" s="0" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
-      </c>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I7" s="0"/>
       <c r="J7" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -811,46 +811,46 @@
         <v>0.0</v>
       </c>
       <c r="L7" s="0" t="n">
-        <v>45000.0</v>
+        <v>0.0</v>
       </c>
       <c r="M7" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N7" s="0" t="n">
-        <v>45000.0</v>
+        <v>0.0</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>1530.0</v>
+        <v>0.0</v>
       </c>
       <c r="P7" s="0" t="n">
-        <v>454.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q7" s="0" t="n">
-        <v>43016.0</v>
+        <v>0.0</v>
       </c>
       <c r="R7" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V7" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W7" s="0"/>
@@ -868,17 +868,17 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:35</t>
+          <t>2026/05/11 22:22:09</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:36</t>
+          <t>2026/05/11 22:22:12</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>822733043006520176640</t>
+          <t>822742502121738878976</t>
         </is>
       </c>
       <c r="D8" s="0" t="n">
@@ -906,7 +906,7 @@
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>5558</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="J8" s="0" t="n">
@@ -935,27 +935,27 @@
       </c>
       <c r="R8" s="0" t="inlineStr">
         <is>
-          <t>IGNACIO PORTILLA</t>
+          <t>Macarena Olavarri</t>
         </is>
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t>mx.portilla@gmail.com</t>
+          <t>macaolavarri@gmail.com</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
+          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t>VALERIA PORTILLA, Natalia Portilla</t>
+          <t>Macarena Olavarri, Isabel Fernández</t>
         </is>
       </c>
       <c r="V8" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W8" s="0"/>
@@ -973,21 +973,21 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:10:30</t>
+          <t>2026/05/08 23:10:41</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:11:05</t>
+          <t>2026/05/08 23:10:43</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>822732983572553019392</t>
+          <t>822740352219193810944</t>
         </is>
       </c>
       <c r="D9" s="0" t="n">
-        <v>18000.0</v>
+        <v>81000.0</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
@@ -1006,12 +1006,12 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="J9" s="0" t="n">
@@ -1021,46 +1021,46 @@
         <v>0.0</v>
       </c>
       <c r="L9" s="0" t="n">
-        <v>18000.0</v>
+        <v>81000.0</v>
       </c>
       <c r="M9" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N9" s="0" t="n">
-        <v>18000.0</v>
+        <v>81000.0</v>
       </c>
       <c r="O9" s="0" t="n">
-        <v>522.0</v>
+        <v>2754.0</v>
       </c>
       <c r="P9" s="0" t="n">
-        <v>184.0</v>
+        <v>814.0</v>
       </c>
       <c r="Q9" s="0" t="n">
-        <v>17294.0</v>
+        <v>77432.0</v>
       </c>
       <c r="R9" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>Judith Escobar Torres</t>
         </is>
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>judith.escobar@gmail.com</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
         </is>
       </c>
       <c r="V9" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W9" s="0"/>
@@ -1078,21 +1078,21 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:49</t>
+          <t>2026/05/08 18:45:11</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:51</t>
+          <t>2026/05/08 18:45:12</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>822728072370714607616</t>
+          <t>822740218587619794944</t>
         </is>
       </c>
       <c r="D10" s="0" t="n">
-        <v>9833.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>2071</t>
+          <t>6624</t>
         </is>
       </c>
       <c r="J10" s="0" t="n">
@@ -1126,46 +1126,46 @@
         <v>0.0</v>
       </c>
       <c r="L10" s="0" t="n">
-        <v>9833.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M10" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N10" s="0" t="n">
-        <v>9833.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O10" s="0" t="n">
-        <v>285.16</v>
+        <v>739.5</v>
       </c>
       <c r="P10" s="0" t="n">
-        <v>102.33</v>
+        <v>259.0</v>
       </c>
       <c r="Q10" s="0" t="n">
-        <v>9445.51</v>
+        <v>24501.5</v>
       </c>
       <c r="R10" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>MELB PEREZ SALDANA</t>
         </is>
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>MELBA ASTRID PEREZ SALDAÑA</t>
         </is>
       </c>
       <c r="V10" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W10" s="0"/>
@@ -1183,17 +1183,17 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:44</t>
+          <t>2026/05/08 18:14:10</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:46</t>
+          <t>2026/05/08 18:14:12</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>822728021498622136320</t>
+          <t>822740202977192058880</t>
         </is>
       </c>
       <c r="D11" s="0" t="n">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>9925</t>
         </is>
       </c>
       <c r="J11" s="0" t="n">
@@ -1250,27 +1250,27 @@
       </c>
       <c r="R11" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S11" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T11" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U11" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V11" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W11" s="0"/>
@@ -1288,17 +1288,17 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:01</t>
+          <t>2026/05/07 00:33:20</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:03</t>
+          <t>2026/05/07 00:33:22</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>822727454901268389888</t>
+          <t>822738944267014664192</t>
         </is>
       </c>
       <c r="D12" s="0" t="n">
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>6156</t>
         </is>
       </c>
       <c r="J12" s="0" t="n">
@@ -1355,27 +1355,27 @@
       </c>
       <c r="R12" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>Alejandra Serpas</t>
         </is>
       </c>
       <c r="S12" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="T12" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="U12" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>Alejandra Serpas, Denisse Olivo</t>
         </is>
       </c>
       <c r="V12" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W12" s="0"/>
@@ -1393,25 +1393,25 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:12</t>
+          <t>2026/05/06 23:07:12</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:13</t>
+          <t>2026/05/11 23:05:58</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>822727364900010598400</t>
+          <t>822738900913572839424</t>
         </is>
       </c>
       <c r="D13" s="0" t="n">
-        <v>22500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Successful</t>
+          <t>Refunded</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
@@ -1421,61 +1421,57 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I13" s="0" t="inlineStr">
-        <is>
-          <t>7852</t>
-        </is>
-      </c>
+          <t>transferencia</t>
+        </is>
+      </c>
+      <c r="I13" s="0"/>
       <c r="J13" s="0" t="n">
-        <v>0.0</v>
+        <v>20500.0</v>
       </c>
       <c r="K13" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L13" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M13" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N13" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O13" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P13" s="0" t="n">
-        <v>229.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q13" s="0" t="n">
-        <v>21618.5</v>
+        <v>0.0</v>
       </c>
       <c r="R13" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S13" s="0" t="inlineStr">
         <is>
-          <t>ricardocb23@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T13" s="0" t="inlineStr">
         <is>
-          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U13" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V13" s="0" t="inlineStr">
@@ -1498,21 +1494,21 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:19</t>
+          <t>2026/05/02 22:46:40</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:21</t>
+          <t>2026/05/02 22:46:42</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>822726495229304659968</t>
+          <t>822735991480689651712</t>
         </is>
       </c>
       <c r="D14" s="0" t="n">
-        <v>14750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
@@ -1526,7 +1522,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -1536,7 +1532,7 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="J14" s="0" t="n">
@@ -1546,46 +1542,46 @@
         <v>0.0</v>
       </c>
       <c r="L14" s="0" t="n">
-        <v>14750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M14" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N14" s="0" t="n">
-        <v>14750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O14" s="0" t="n">
-        <v>427.75</v>
+        <v>1530.0</v>
       </c>
       <c r="P14" s="0" t="n">
-        <v>151.5</v>
+        <v>454.0</v>
       </c>
       <c r="Q14" s="0" t="n">
-        <v>14170.75</v>
+        <v>43016.0</v>
       </c>
       <c r="R14" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>ALEJANDRO CANALES MORALES</t>
         </is>
       </c>
       <c r="S14" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="T14" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="U14" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
         </is>
       </c>
       <c r="V14" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W14" s="0"/>
@@ -1603,21 +1599,21 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:21</t>
+          <t>2026/04/28 21:08:35</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:23</t>
+          <t>2026/04/28 21:08:36</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>822725726179188305920</t>
+          <t>822733043006520176640</t>
         </is>
       </c>
       <c r="D15" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
@@ -1636,12 +1632,12 @@
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
-          <t>9962</t>
+          <t>5558</t>
         </is>
       </c>
       <c r="J15" s="0" t="n">
@@ -1651,46 +1647,46 @@
         <v>0.0</v>
       </c>
       <c r="L15" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M15" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N15" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O15" s="0" t="n">
-        <v>739.5</v>
+        <v>652.5</v>
       </c>
       <c r="P15" s="0" t="n">
-        <v>259.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q15" s="0" t="n">
-        <v>24501.5</v>
+        <v>21618.5</v>
       </c>
       <c r="R15" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon Mendez</t>
+          <t>IGNACIO PORTILLA</t>
         </is>
       </c>
       <c r="S15" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>mx.portilla@gmail.com</t>
         </is>
       </c>
       <c r="T15" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
         </is>
       </c>
       <c r="U15" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon</t>
+          <t>VALERIA PORTILLA, Natalia Portilla</t>
         </is>
       </c>
       <c r="V15" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W15" s="0"/>
@@ -1708,21 +1704,21 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:42</t>
+          <t>2026/04/28 19:10:30</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:44</t>
+          <t>2026/04/28 19:11:05</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>822724934643911520256</t>
+          <t>822732983572553019392</t>
         </is>
       </c>
       <c r="D16" s="0" t="n">
-        <v>70500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -1741,12 +1737,12 @@
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J16" s="0" t="n">
@@ -1756,41 +1752,41 @@
         <v>0.0</v>
       </c>
       <c r="L16" s="0" t="n">
-        <v>70500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="M16" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N16" s="0" t="n">
-        <v>70500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="O16" s="0" t="n">
-        <v>2397.0</v>
+        <v>522.0</v>
       </c>
       <c r="P16" s="0" t="n">
-        <v>709.0</v>
+        <v>184.0</v>
       </c>
       <c r="Q16" s="0" t="n">
-        <v>67394.0</v>
+        <v>17294.0</v>
       </c>
       <c r="R16" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S16" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T16" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U16" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V16" s="0" t="inlineStr">
@@ -1813,21 +1809,21 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:28</t>
+          <t>2026/04/22 00:32:49</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:30</t>
+          <t>2026/04/22 00:32:51</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>822722199504844500992</t>
+          <t>822728072370714607616</t>
         </is>
       </c>
       <c r="D17" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
@@ -1851,7 +1847,7 @@
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>4291</t>
+          <t>2071</t>
         </is>
       </c>
       <c r="J17" s="0" t="n">
@@ -1861,46 +1857,46 @@
         <v>0.0</v>
       </c>
       <c r="L17" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M17" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N17" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O17" s="0" t="n">
-        <v>1305.0</v>
+        <v>285.16</v>
       </c>
       <c r="P17" s="0" t="n">
-        <v>454.0</v>
+        <v>102.33</v>
       </c>
       <c r="Q17" s="0" t="n">
-        <v>43241.0</v>
+        <v>9445.51</v>
       </c>
       <c r="R17" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="S17" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="T17" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="U17" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="V17" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W17" s="0"/>
@@ -1918,21 +1914,21 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:45</t>
+          <t>2026/04/21 22:51:44</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:47</t>
+          <t>2026/04/21 22:51:46</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>822722120121735725056</t>
+          <t>822728021498622136320</t>
         </is>
       </c>
       <c r="D18" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -1951,12 +1947,12 @@
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J18" s="0" t="n">
@@ -1966,46 +1962,46 @@
         <v>0.0</v>
       </c>
       <c r="L18" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M18" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N18" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O18" s="0" t="n">
-        <v>1530.0</v>
+        <v>652.5</v>
       </c>
       <c r="P18" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q18" s="0" t="n">
-        <v>43016.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R18" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S18" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T18" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U18" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac, Gabriela Vazquez</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V18" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W18" s="0"/>
@@ -2023,21 +2019,21 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:14</t>
+          <t>2026/04/21 04:06:01</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:16</t>
+          <t>2026/04/21 04:06:03</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>822718782367677300736</t>
+          <t>822727454901268389888</t>
         </is>
       </c>
       <c r="D19" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
@@ -2051,7 +2047,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -2061,7 +2057,7 @@
       </c>
       <c r="I19" s="0" t="inlineStr">
         <is>
-          <t>7348</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J19" s="0" t="n">
@@ -2071,46 +2067,46 @@
         <v>0.0</v>
       </c>
       <c r="L19" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M19" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N19" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O19" s="0" t="n">
-        <v>1305.0</v>
+        <v>652.5</v>
       </c>
       <c r="P19" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q19" s="0" t="n">
-        <v>43241.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R19" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera Lima</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S19" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T19" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U19" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V19" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W19" s="0"/>
@@ -2128,21 +2124,21 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:52</t>
+          <t>2026/04/21 01:07:12</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:54</t>
+          <t>2026/04/21 01:07:13</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>822717931075648110592</t>
+          <t>822727364900010598400</t>
         </is>
       </c>
       <c r="D20" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
@@ -2161,12 +2157,12 @@
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>7852</t>
         </is>
       </c>
       <c r="J20" s="0" t="n">
@@ -2176,46 +2172,46 @@
         <v>0.0</v>
       </c>
       <c r="L20" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M20" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N20" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O20" s="0" t="n">
-        <v>1530.0</v>
+        <v>652.5</v>
       </c>
       <c r="P20" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q20" s="0" t="n">
-        <v>43016.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R20" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+          <t>RICARDO CAMACHO BOFILL</t>
         </is>
       </c>
       <c r="S20" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com</t>
+          <t>ricardocb23@gmail.com</t>
         </is>
       </c>
       <c r="T20" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
         </is>
       </c>
       <c r="U20" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
         </is>
       </c>
       <c r="V20" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W20" s="0"/>
@@ -2233,21 +2229,21 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:06</t>
+          <t>2026/04/19 20:19:19</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:09</t>
+          <t>2026/04/19 20:19:21</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>822717887408069685248</t>
+          <t>822726495229304659968</t>
         </is>
       </c>
       <c r="D21" s="0" t="n">
-        <v>31500.0</v>
+        <v>14750.0</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
@@ -2261,7 +2257,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>apple_pay</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -2271,7 +2267,7 @@
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t>4006</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="J21" s="0" t="n">
@@ -2281,46 +2277,46 @@
         <v>0.0</v>
       </c>
       <c r="L21" s="0" t="n">
-        <v>31500.0</v>
+        <v>14750.0</v>
       </c>
       <c r="M21" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N21" s="0" t="n">
-        <v>31500.0</v>
+        <v>14750.0</v>
       </c>
       <c r="O21" s="0" t="n">
-        <v>1071.0</v>
+        <v>427.75</v>
       </c>
       <c r="P21" s="0" t="n">
-        <v>319.0</v>
+        <v>151.5</v>
       </c>
       <c r="Q21" s="0" t="n">
-        <v>30110.0</v>
+        <v>14170.75</v>
       </c>
       <c r="R21" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="S21" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="T21" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="U21" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago, Michelle Ralph</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="V21" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W21" s="0"/>
@@ -2338,17 +2334,17 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:57</t>
+          <t>2026/04/18 18:51:21</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:59</t>
+          <t>2026/04/18 18:51:23</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>822717804781623066624</t>
+          <t>822725726179188305920</t>
         </is>
       </c>
       <c r="D22" s="0" t="n">
@@ -2376,7 +2372,7 @@
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t>3513</t>
+          <t>9962</t>
         </is>
       </c>
       <c r="J22" s="0" t="n">
@@ -2405,22 +2401,22 @@
       </c>
       <c r="R22" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>Jonatan Oregon Mendez</t>
         </is>
       </c>
       <c r="S22" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="T22" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="U22" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>Jonatan Oregon</t>
         </is>
       </c>
       <c r="V22" s="0" t="inlineStr">
@@ -2443,21 +2439,21 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:51</t>
+          <t>2026/04/17 16:38:42</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:53</t>
+          <t>2026/04/17 16:38:44</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>822717250585584762880</t>
+          <t>822724934643911520256</t>
         </is>
       </c>
       <c r="D23" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -2481,7 +2477,7 @@
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J23" s="0" t="n">
@@ -2491,46 +2487,46 @@
         <v>0.0</v>
       </c>
       <c r="L23" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="M23" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N23" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="O23" s="0" t="n">
-        <v>1530.0</v>
+        <v>2397.0</v>
       </c>
       <c r="P23" s="0" t="n">
-        <v>454.0</v>
+        <v>709.0</v>
       </c>
       <c r="Q23" s="0" t="n">
-        <v>43016.0</v>
+        <v>67394.0</v>
       </c>
       <c r="R23" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion</t>
+          <t>Marcela Alvarez Campos</t>
         </is>
       </c>
       <c r="S23" s="0" t="inlineStr">
         <is>
-          <t>sofiacarrioncobian@hotmail.com</t>
+          <t>marcela.ac@me.com</t>
         </is>
       </c>
       <c r="T23" s="0" t="inlineStr">
         <is>
-          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
         </is>
       </c>
       <c r="U23" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion, Ana María Carrion</t>
+          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
         </is>
       </c>
       <c r="V23" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W23" s="0"/>
@@ -2540,6 +2536,741 @@
         </is>
       </c>
       <c r="Y23" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 22:04:28</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 22:04:30</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>822722199504844500992</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I24" s="0" t="inlineStr">
+        <is>
+          <t>4291</t>
+        </is>
+      </c>
+      <c r="J24" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K24" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L24" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M24" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N24" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O24" s="0" t="n">
+        <v>1305.0</v>
+      </c>
+      <c r="P24" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q24" s="0" t="n">
+        <v>43241.0</v>
+      </c>
+      <c r="R24" s="0" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="S24" s="0" t="inlineStr">
+        <is>
+          <t>mendoza.carlos.a@gmail.com</t>
+        </is>
+      </c>
+      <c r="T24" s="0" t="inlineStr">
+        <is>
+          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
+        </is>
+      </c>
+      <c r="U24" s="0" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
+        </is>
+      </c>
+      <c r="V24" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+        </is>
+      </c>
+      <c r="W24" s="0"/>
+      <c r="X24" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y24" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 19:26:45</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 19:26:47</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>822722120121735725056</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H25" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I25" s="0" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+      <c r="J25" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K25" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L25" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M25" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N25" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O25" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P25" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q25" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R25" s="0" t="inlineStr">
+        <is>
+          <t>Ana paula Isaac</t>
+        </is>
+      </c>
+      <c r="S25" s="0" t="inlineStr">
+        <is>
+          <t>anapauisaac@gmail.com</t>
+        </is>
+      </c>
+      <c r="T25" s="0" t="inlineStr">
+        <is>
+          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
+        </is>
+      </c>
+      <c r="U25" s="0" t="inlineStr">
+        <is>
+          <t>Ana paula Isaac, Gabriela Vazquez</t>
+        </is>
+      </c>
+      <c r="V25" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W25" s="0"/>
+      <c r="X25" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y25" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/09 04:55:14</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/09 04:55:16</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>822718782367677300736</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>apple_pay</t>
+        </is>
+      </c>
+      <c r="H26" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I26" s="0" t="inlineStr">
+        <is>
+          <t>7348</t>
+        </is>
+      </c>
+      <c r="J26" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K26" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L26" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M26" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N26" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O26" s="0" t="n">
+        <v>1305.0</v>
+      </c>
+      <c r="P26" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q26" s="0" t="n">
+        <v>43241.0</v>
+      </c>
+      <c r="R26" s="0" t="inlineStr">
+        <is>
+          <t>Francisco Javier Vera Lima</t>
+        </is>
+      </c>
+      <c r="S26" s="0" t="inlineStr">
+        <is>
+          <t>fjvera@vmodal.mx</t>
+        </is>
+      </c>
+      <c r="T26" s="0" t="inlineStr">
+        <is>
+          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+        </is>
+      </c>
+      <c r="U26" s="0" t="inlineStr">
+        <is>
+          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
+        </is>
+      </c>
+      <c r="V26" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W26" s="0"/>
+      <c r="X26" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y26" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:52</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:54</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>822717931075648110592</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H27" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I27" s="0" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="J27" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K27" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L27" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M27" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N27" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O27" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P27" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q27" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R27" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+        </is>
+      </c>
+      <c r="S27" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T27" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+        </is>
+      </c>
+      <c r="U27" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+        </is>
+      </c>
+      <c r="V27" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W27" s="0"/>
+      <c r="X27" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y27" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:06</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:09</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>822717887408069685248</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H28" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I28" s="0" t="inlineStr">
+        <is>
+          <t>4006</t>
+        </is>
+      </c>
+      <c r="J28" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K28" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L28" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="M28" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N28" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="O28" s="0" t="n">
+        <v>1071.0</v>
+      </c>
+      <c r="P28" s="0" t="n">
+        <v>319.0</v>
+      </c>
+      <c r="Q28" s="0" t="n">
+        <v>30110.0</v>
+      </c>
+      <c r="R28" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago</t>
+        </is>
+      </c>
+      <c r="S28" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com</t>
+        </is>
+      </c>
+      <c r="T28" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+        </is>
+      </c>
+      <c r="U28" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago, Michelle Ralph</t>
+        </is>
+      </c>
+      <c r="V28" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W28" s="0"/>
+      <c r="X28" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y28" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:57</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:59</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>822717804781623066624</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H29" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I29" s="0" t="inlineStr">
+        <is>
+          <t>3513</t>
+        </is>
+      </c>
+      <c r="J29" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K29" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L29" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="M29" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N29" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="O29" s="0" t="n">
+        <v>739.5</v>
+      </c>
+      <c r="P29" s="0" t="n">
+        <v>259.0</v>
+      </c>
+      <c r="Q29" s="0" t="n">
+        <v>24501.5</v>
+      </c>
+      <c r="R29" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="S29" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="T29" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="U29" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="V29" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W29" s="0"/>
+      <c r="X29" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y29" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:51</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:53</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>822717250585584762880</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H30" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I30" s="0" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="J30" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K30" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L30" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M30" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N30" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O30" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P30" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q30" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R30" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion</t>
+        </is>
+      </c>
+      <c r="S30" s="0" t="inlineStr">
+        <is>
+          <t>sofiacarrioncobian@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T30" s="0" t="inlineStr">
+        <is>
+          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+        </is>
+      </c>
+      <c r="U30" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion, Ana María Carrion</t>
+        </is>
+      </c>
+      <c r="V30" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W30" s="0"/>
+      <c r="X30" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y30" s="0" t="inlineStr">
         <is>
           <t>daniel@akampa.mx</t>
         </is>

</xml_diff>

<commit_message>
📥 WeTravel: Reporting_Payments_WeTravel-539682-1778866763.xlsx (2026-05-15)
</commit_message>
<xml_diff>
--- a/reportes/Reporting_Payments_WeTravel.xlsx
+++ b/reportes/Reporting_Payments_WeTravel.xlsx
@@ -82,7 +82,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y30"/>
+  <dimension ref="A1:Y32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="29.4" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -242,21 +242,21 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:31</t>
+          <t>2026/05/15 17:24:50</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:33</t>
+          <t>2026/05/15 17:24:53</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>822743406261352546304</t>
+          <t>822745251580101009408</t>
         </is>
       </c>
       <c r="D2" s="0" t="n">
-        <v>12750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
@@ -275,12 +275,12 @@
       </c>
       <c r="H2" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>1009</t>
+          <t>3097</t>
         </is>
       </c>
       <c r="J2" s="0" t="n">
@@ -290,46 +290,46 @@
         <v>0.0</v>
       </c>
       <c r="L2" s="0" t="n">
-        <v>12750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M2" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N2" s="0" t="n">
-        <v>12750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O2" s="0" t="n">
-        <v>433.5</v>
+        <v>652.5</v>
       </c>
       <c r="P2" s="0" t="n">
-        <v>131.5</v>
+        <v>229.0</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <v>12185.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R2" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Marihel Arias</t>
         </is>
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>marihel_arias@hotmail.com</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Marihel Arias, Alondra Arias</t>
         </is>
       </c>
       <c r="V2" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W2" s="0"/>
@@ -347,21 +347,21 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:03</t>
+          <t>2026/05/14 21:47:03</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:05</t>
+          <t>2026/05/14 21:47:05</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>822743384884528578560</t>
+          <t>822744658783664881664</t>
         </is>
       </c>
       <c r="D3" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
@@ -380,12 +380,12 @@
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>7758</t>
+          <t>1003</t>
         </is>
       </c>
       <c r="J3" s="0" t="n">
@@ -395,41 +395,41 @@
         <v>0.0</v>
       </c>
       <c r="L3" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M3" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N3" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O3" s="0" t="n">
-        <v>369.75</v>
+        <v>1530.0</v>
       </c>
       <c r="P3" s="0" t="n">
-        <v>131.5</v>
+        <v>454.0</v>
       </c>
       <c r="Q3" s="0" t="n">
-        <v>12248.75</v>
+        <v>43016.0</v>
       </c>
       <c r="R3" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>FERNANDO FONSECA</t>
         </is>
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>fonsecaf88@gmail.com, fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>FERNANDO FONSECA, Matias fonseca</t>
         </is>
       </c>
       <c r="V3" s="0" t="inlineStr">
@@ -452,21 +452,21 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:39</t>
+          <t>2026/05/13 04:18:31</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:41</t>
+          <t>2026/05/13 04:18:33</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>822743194435830431744</t>
+          <t>822743406261352546304</t>
         </is>
       </c>
       <c r="D4" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
@@ -485,12 +485,12 @@
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>9925</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="J4" s="0" t="n">
@@ -500,46 +500,46 @@
         <v>0.0</v>
       </c>
       <c r="L4" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M4" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N4" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O4" s="0" t="n">
-        <v>652.5</v>
+        <v>433.5</v>
       </c>
       <c r="P4" s="0" t="n">
-        <v>229.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q4" s="0" t="n">
-        <v>21618.5</v>
+        <v>12185.0</v>
       </c>
       <c r="R4" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="S4" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="T4" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="U4" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="V4" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W4" s="0"/>
@@ -557,21 +557,21 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:10:30</t>
+          <t>2026/05/13 03:36:03</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:11:16</t>
+          <t>2026/05/13 03:36:05</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>822743130440389902336</t>
+          <t>822743384884528578560</t>
         </is>
       </c>
       <c r="D5" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>7758</t>
         </is>
       </c>
       <c r="J5" s="0" t="n">
@@ -605,46 +605,46 @@
         <v>0.0</v>
       </c>
       <c r="L5" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M5" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N5" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O5" s="0" t="n">
-        <v>652.5</v>
+        <v>369.75</v>
       </c>
       <c r="P5" s="0" t="n">
-        <v>229.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q5" s="0" t="n">
-        <v>21618.5</v>
+        <v>12248.75</v>
       </c>
       <c r="R5" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="V5" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W5" s="0"/>
@@ -662,21 +662,21 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:51</t>
+          <t>2026/05/12 21:17:39</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:53</t>
+          <t>2026/05/12 21:17:41</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>822743104942704197632</t>
+          <t>822743194435830431744</t>
         </is>
       </c>
       <c r="D6" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t>1709</t>
+          <t>9925</t>
         </is>
       </c>
       <c r="J6" s="0" t="n">
@@ -710,46 +710,46 @@
         <v>0.0</v>
       </c>
       <c r="L6" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M6" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N6" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O6" s="0" t="n">
-        <v>1305.0</v>
+        <v>652.5</v>
       </c>
       <c r="P6" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q6" s="0" t="n">
-        <v>43241.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R6" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S6" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T6" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U6" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V6" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W6" s="0"/>
@@ -767,21 +767,21 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/12 19:10:30</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/12 19:11:16</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>822742523051869483008</t>
+          <t>822743130440389902336</t>
         </is>
       </c>
       <c r="D7" s="0" t="n">
-        <v>20500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
@@ -795,15 +795,19 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="I7" s="0"/>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I7" s="0" t="inlineStr">
+        <is>
+          <t>7580</t>
+        </is>
+      </c>
       <c r="J7" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -811,46 +815,46 @@
         <v>0.0</v>
       </c>
       <c r="L7" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M7" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N7" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>0.0</v>
+        <v>652.5</v>
       </c>
       <c r="P7" s="0" t="n">
-        <v>0.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q7" s="0" t="n">
-        <v>0.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R7" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V7" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W7" s="0"/>
@@ -868,21 +872,21 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:09</t>
+          <t>2026/05/12 18:19:51</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:12</t>
+          <t>2026/05/12 18:19:53</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>822742502121738878976</t>
+          <t>822743104942704197632</t>
         </is>
       </c>
       <c r="D8" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
@@ -901,12 +905,12 @@
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>1775</t>
+          <t>1709</t>
         </is>
       </c>
       <c r="J8" s="0" t="n">
@@ -916,46 +920,46 @@
         <v>0.0</v>
       </c>
       <c r="L8" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M8" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N8" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O8" s="0" t="n">
-        <v>652.5</v>
+        <v>1305.0</v>
       </c>
       <c r="P8" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q8" s="0" t="n">
-        <v>21618.5</v>
+        <v>43241.0</v>
       </c>
       <c r="R8" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri</t>
+          <t>RAFAEL BELTRAN LOPEZ</t>
         </is>
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com</t>
+          <t>rbeltran1976@hotmail.com</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
+          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri, Isabel Fernández</t>
+          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
         </is>
       </c>
       <c r="V8" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W8" s="0"/>
@@ -973,21 +977,21 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:41</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:43</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>822740352219193810944</t>
+          <t>822742523051869483008</t>
         </is>
       </c>
       <c r="D9" s="0" t="n">
-        <v>81000.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
@@ -1001,19 +1005,15 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
-        </is>
-      </c>
-      <c r="I9" s="0" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I9" s="0"/>
       <c r="J9" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1021,46 +1021,46 @@
         <v>0.0</v>
       </c>
       <c r="L9" s="0" t="n">
-        <v>81000.0</v>
+        <v>0.0</v>
       </c>
       <c r="M9" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N9" s="0" t="n">
-        <v>81000.0</v>
+        <v>0.0</v>
       </c>
       <c r="O9" s="0" t="n">
-        <v>2754.0</v>
+        <v>0.0</v>
       </c>
       <c r="P9" s="0" t="n">
-        <v>814.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q9" s="0" t="n">
-        <v>77432.0</v>
+        <v>0.0</v>
       </c>
       <c r="R9" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V9" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W9" s="0"/>
@@ -1078,21 +1078,21 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:11</t>
+          <t>2026/05/11 22:22:09</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:12</t>
+          <t>2026/05/11 22:22:12</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>822740218587619794944</t>
+          <t>822742502121738878976</t>
         </is>
       </c>
       <c r="D10" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
@@ -1111,12 +1111,12 @@
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>6624</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="J10" s="0" t="n">
@@ -1126,46 +1126,46 @@
         <v>0.0</v>
       </c>
       <c r="L10" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M10" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N10" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O10" s="0" t="n">
-        <v>739.5</v>
+        <v>652.5</v>
       </c>
       <c r="P10" s="0" t="n">
-        <v>259.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q10" s="0" t="n">
-        <v>24501.5</v>
+        <v>21618.5</v>
       </c>
       <c r="R10" s="0" t="inlineStr">
         <is>
-          <t>MELB PEREZ SALDANA</t>
+          <t>Macarena Olavarri</t>
         </is>
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>macaolavarri@gmail.com</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t>MELBA ASTRID PEREZ SALDAÑA</t>
+          <t>Macarena Olavarri, Isabel Fernández</t>
         </is>
       </c>
       <c r="V10" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W10" s="0"/>
@@ -1183,21 +1183,21 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:10</t>
+          <t>2026/05/08 23:10:41</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:12</t>
+          <t>2026/05/08 23:10:43</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>822740202977192058880</t>
+          <t>822740352219193810944</t>
         </is>
       </c>
       <c r="D11" s="0" t="n">
-        <v>22500.0</v>
+        <v>81000.0</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
@@ -1216,12 +1216,12 @@
       </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>9925</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="J11" s="0" t="n">
@@ -1231,46 +1231,46 @@
         <v>0.0</v>
       </c>
       <c r="L11" s="0" t="n">
-        <v>22500.0</v>
+        <v>81000.0</v>
       </c>
       <c r="M11" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N11" s="0" t="n">
-        <v>22500.0</v>
+        <v>81000.0</v>
       </c>
       <c r="O11" s="0" t="n">
-        <v>652.5</v>
+        <v>2754.0</v>
       </c>
       <c r="P11" s="0" t="n">
-        <v>229.0</v>
+        <v>814.0</v>
       </c>
       <c r="Q11" s="0" t="n">
-        <v>21618.5</v>
+        <v>77432.0</v>
       </c>
       <c r="R11" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>Judith Escobar Torres</t>
         </is>
       </c>
       <c r="S11" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>judith.escobar@gmail.com</t>
         </is>
       </c>
       <c r="T11" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
         </is>
       </c>
       <c r="U11" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
         </is>
       </c>
       <c r="V11" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W11" s="0"/>
@@ -1288,21 +1288,21 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:20</t>
+          <t>2026/05/08 18:45:11</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:22</t>
+          <t>2026/05/08 18:45:12</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>822738944267014664192</t>
+          <t>822740218587619794944</t>
         </is>
       </c>
       <c r="D12" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>6156</t>
+          <t>6624</t>
         </is>
       </c>
       <c r="J12" s="0" t="n">
@@ -1336,46 +1336,46 @@
         <v>0.0</v>
       </c>
       <c r="L12" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M12" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N12" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O12" s="0" t="n">
-        <v>652.5</v>
+        <v>739.5</v>
       </c>
       <c r="P12" s="0" t="n">
-        <v>229.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q12" s="0" t="n">
-        <v>21618.5</v>
+        <v>24501.5</v>
       </c>
       <c r="R12" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas</t>
+          <t>MELB PEREZ SALDANA</t>
         </is>
       </c>
       <c r="S12" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="T12" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="U12" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas, Denisse Olivo</t>
+          <t>MELBA ASTRID PEREZ SALDAÑA</t>
         </is>
       </c>
       <c r="V12" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W12" s="0"/>
@@ -1393,25 +1393,25 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/06 23:07:12</t>
+          <t>2026/05/08 18:14:10</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:05:58</t>
+          <t>2026/05/08 18:14:12</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>822738900913572839424</t>
+          <t>822740202977192058880</t>
         </is>
       </c>
       <c r="D13" s="0" t="n">
-        <v>20500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Refunded</t>
+          <t>Successful</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
@@ -1421,62 +1421,66 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>transferencia</t>
-        </is>
-      </c>
-      <c r="I13" s="0"/>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>9925</t>
+        </is>
+      </c>
       <c r="J13" s="0" t="n">
-        <v>20500.0</v>
+        <v>0.0</v>
       </c>
       <c r="K13" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L13" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M13" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N13" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O13" s="0" t="n">
-        <v>0.0</v>
+        <v>652.5</v>
       </c>
       <c r="P13" s="0" t="n">
-        <v>0.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q13" s="0" t="n">
-        <v>0.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R13" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S13" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T13" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U13" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V13" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W13" s="0"/>
@@ -1494,21 +1498,21 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:40</t>
+          <t>2026/05/07 00:33:20</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:42</t>
+          <t>2026/05/07 00:33:22</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>822735991480689651712</t>
+          <t>822738944267014664192</t>
         </is>
       </c>
       <c r="D14" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
@@ -1527,12 +1531,12 @@
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t>2003</t>
+          <t>6156</t>
         </is>
       </c>
       <c r="J14" s="0" t="n">
@@ -1542,41 +1546,41 @@
         <v>0.0</v>
       </c>
       <c r="L14" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M14" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N14" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O14" s="0" t="n">
-        <v>1530.0</v>
+        <v>652.5</v>
       </c>
       <c r="P14" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q14" s="0" t="n">
-        <v>43016.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R14" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES</t>
+          <t>Alejandra Serpas</t>
         </is>
       </c>
       <c r="S14" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com</t>
+          <t>denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="T14" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
+          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="U14" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
+          <t>Alejandra Serpas, Denisse Olivo</t>
         </is>
       </c>
       <c r="V14" s="0" t="inlineStr">
@@ -1599,25 +1603,25 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:35</t>
+          <t>2026/05/06 23:07:12</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:36</t>
+          <t>2026/05/11 23:05:58</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>822733043006520176640</t>
+          <t>822738900913572839424</t>
         </is>
       </c>
       <c r="D15" s="0" t="n">
-        <v>22500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Successful</t>
+          <t>Refunded</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
@@ -1627,61 +1631,57 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
-        </is>
-      </c>
-      <c r="I15" s="0" t="inlineStr">
-        <is>
-          <t>5558</t>
-        </is>
-      </c>
+          <t>transferencia</t>
+        </is>
+      </c>
+      <c r="I15" s="0"/>
       <c r="J15" s="0" t="n">
-        <v>0.0</v>
+        <v>20500.0</v>
       </c>
       <c r="K15" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L15" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M15" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N15" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O15" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P15" s="0" t="n">
-        <v>229.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q15" s="0" t="n">
-        <v>21618.5</v>
+        <v>0.0</v>
       </c>
       <c r="R15" s="0" t="inlineStr">
         <is>
-          <t>IGNACIO PORTILLA</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S15" s="0" t="inlineStr">
         <is>
-          <t>mx.portilla@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T15" s="0" t="inlineStr">
         <is>
-          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U15" s="0" t="inlineStr">
         <is>
-          <t>VALERIA PORTILLA, Natalia Portilla</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V15" s="0" t="inlineStr">
@@ -1704,21 +1704,21 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:10:30</t>
+          <t>2026/05/02 22:46:40</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:11:05</t>
+          <t>2026/05/02 22:46:42</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>822732983572553019392</t>
+          <t>822735991480689651712</t>
         </is>
       </c>
       <c r="D16" s="0" t="n">
-        <v>18000.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="J16" s="0" t="n">
@@ -1752,46 +1752,46 @@
         <v>0.0</v>
       </c>
       <c r="L16" s="0" t="n">
-        <v>18000.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M16" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N16" s="0" t="n">
-        <v>18000.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O16" s="0" t="n">
-        <v>522.0</v>
+        <v>1530.0</v>
       </c>
       <c r="P16" s="0" t="n">
-        <v>184.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q16" s="0" t="n">
-        <v>17294.0</v>
+        <v>43016.0</v>
       </c>
       <c r="R16" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>ALEJANDRO CANALES MORALES</t>
         </is>
       </c>
       <c r="S16" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="T16" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="U16" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
         </is>
       </c>
       <c r="V16" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W16" s="0"/>
@@ -1809,21 +1809,21 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:49</t>
+          <t>2026/04/28 21:08:35</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:51</t>
+          <t>2026/04/28 21:08:36</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>822728072370714607616</t>
+          <t>822733043006520176640</t>
         </is>
       </c>
       <c r="D17" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
@@ -1842,12 +1842,12 @@
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>2071</t>
+          <t>5558</t>
         </is>
       </c>
       <c r="J17" s="0" t="n">
@@ -1857,46 +1857,46 @@
         <v>0.0</v>
       </c>
       <c r="L17" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M17" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N17" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O17" s="0" t="n">
-        <v>285.16</v>
+        <v>652.5</v>
       </c>
       <c r="P17" s="0" t="n">
-        <v>102.33</v>
+        <v>229.0</v>
       </c>
       <c r="Q17" s="0" t="n">
-        <v>9445.51</v>
+        <v>21618.5</v>
       </c>
       <c r="R17" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>IGNACIO PORTILLA</t>
         </is>
       </c>
       <c r="S17" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>mx.portilla@gmail.com</t>
         </is>
       </c>
       <c r="T17" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
         </is>
       </c>
       <c r="U17" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>VALERIA PORTILLA, Natalia Portilla</t>
         </is>
       </c>
       <c r="V17" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W17" s="0"/>
@@ -1914,21 +1914,21 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:44</t>
+          <t>2026/04/28 19:10:30</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:46</t>
+          <t>2026/04/28 19:11:05</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>822728021498622136320</t>
+          <t>822732983572553019392</t>
         </is>
       </c>
       <c r="D18" s="0" t="n">
-        <v>22500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -1962,22 +1962,22 @@
         <v>0.0</v>
       </c>
       <c r="L18" s="0" t="n">
-        <v>22500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="M18" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N18" s="0" t="n">
-        <v>22500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="O18" s="0" t="n">
-        <v>652.5</v>
+        <v>522.0</v>
       </c>
       <c r="P18" s="0" t="n">
-        <v>229.0</v>
+        <v>184.0</v>
       </c>
       <c r="Q18" s="0" t="n">
-        <v>21618.5</v>
+        <v>17294.0</v>
       </c>
       <c r="R18" s="0" t="inlineStr">
         <is>
@@ -2019,21 +2019,21 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:01</t>
+          <t>2026/04/22 00:32:49</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:03</t>
+          <t>2026/04/22 00:32:51</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>822727454901268389888</t>
+          <t>822728072370714607616</t>
         </is>
       </c>
       <c r="D19" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="I19" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>2071</t>
         </is>
       </c>
       <c r="J19" s="0" t="n">
@@ -2067,46 +2067,46 @@
         <v>0.0</v>
       </c>
       <c r="L19" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M19" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N19" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O19" s="0" t="n">
-        <v>652.5</v>
+        <v>285.16</v>
       </c>
       <c r="P19" s="0" t="n">
-        <v>229.0</v>
+        <v>102.33</v>
       </c>
       <c r="Q19" s="0" t="n">
-        <v>21618.5</v>
+        <v>9445.51</v>
       </c>
       <c r="R19" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="S19" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="T19" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="U19" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="V19" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W19" s="0"/>
@@ -2124,17 +2124,17 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:12</t>
+          <t>2026/04/21 22:51:44</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:13</t>
+          <t>2026/04/21 22:51:46</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>822727364900010598400</t>
+          <t>822728021498622136320</t>
         </is>
       </c>
       <c r="D20" s="0" t="n">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>7852</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J20" s="0" t="n">
@@ -2191,22 +2191,22 @@
       </c>
       <c r="R20" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S20" s="0" t="inlineStr">
         <is>
-          <t>ricardocb23@gmail.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T20" s="0" t="inlineStr">
         <is>
-          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U20" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V20" s="0" t="inlineStr">
@@ -2229,21 +2229,21 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:19</t>
+          <t>2026/04/21 04:06:01</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:21</t>
+          <t>2026/04/21 04:06:03</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>822726495229304659968</t>
+          <t>822727454901268389888</t>
         </is>
       </c>
       <c r="D21" s="0" t="n">
-        <v>14750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
@@ -2257,17 +2257,17 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J21" s="0" t="n">
@@ -2277,46 +2277,46 @@
         <v>0.0</v>
       </c>
       <c r="L21" s="0" t="n">
-        <v>14750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M21" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N21" s="0" t="n">
-        <v>14750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O21" s="0" t="n">
-        <v>427.75</v>
+        <v>652.5</v>
       </c>
       <c r="P21" s="0" t="n">
-        <v>151.5</v>
+        <v>229.0</v>
       </c>
       <c r="Q21" s="0" t="n">
-        <v>14170.75</v>
+        <v>21618.5</v>
       </c>
       <c r="R21" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S21" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T21" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U21" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V21" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W21" s="0"/>
@@ -2334,21 +2334,21 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:21</t>
+          <t>2026/04/21 01:07:12</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:23</t>
+          <t>2026/04/21 01:07:13</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>822725726179188305920</t>
+          <t>822727364900010598400</t>
         </is>
       </c>
       <c r="D22" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t>9962</t>
+          <t>7852</t>
         </is>
       </c>
       <c r="J22" s="0" t="n">
@@ -2382,46 +2382,46 @@
         <v>0.0</v>
       </c>
       <c r="L22" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M22" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N22" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O22" s="0" t="n">
-        <v>739.5</v>
+        <v>652.5</v>
       </c>
       <c r="P22" s="0" t="n">
-        <v>259.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q22" s="0" t="n">
-        <v>24501.5</v>
+        <v>21618.5</v>
       </c>
       <c r="R22" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon Mendez</t>
+          <t>RICARDO CAMACHO BOFILL</t>
         </is>
       </c>
       <c r="S22" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>ricardocb23@gmail.com</t>
         </is>
       </c>
       <c r="T22" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
         </is>
       </c>
       <c r="U22" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon</t>
+          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
         </is>
       </c>
       <c r="V22" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W22" s="0"/>
@@ -2439,21 +2439,21 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:42</t>
+          <t>2026/04/19 20:19:19</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:44</t>
+          <t>2026/04/19 20:19:21</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>822724934643911520256</t>
+          <t>822726495229304659968</t>
         </is>
       </c>
       <c r="D23" s="0" t="n">
-        <v>70500.0</v>
+        <v>14750.0</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>apple_pay</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="J23" s="0" t="n">
@@ -2487,46 +2487,46 @@
         <v>0.0</v>
       </c>
       <c r="L23" s="0" t="n">
-        <v>70500.0</v>
+        <v>14750.0</v>
       </c>
       <c r="M23" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N23" s="0" t="n">
-        <v>70500.0</v>
+        <v>14750.0</v>
       </c>
       <c r="O23" s="0" t="n">
-        <v>2397.0</v>
+        <v>427.75</v>
       </c>
       <c r="P23" s="0" t="n">
-        <v>709.0</v>
+        <v>151.5</v>
       </c>
       <c r="Q23" s="0" t="n">
-        <v>67394.0</v>
+        <v>14170.75</v>
       </c>
       <c r="R23" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="S23" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="T23" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="U23" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="V23" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W23" s="0"/>
@@ -2544,21 +2544,21 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:28</t>
+          <t>2026/04/18 18:51:21</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:30</t>
+          <t>2026/04/18 18:51:23</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>822722199504844500992</t>
+          <t>822725726179188305920</t>
         </is>
       </c>
       <c r="D24" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t>4291</t>
+          <t>9962</t>
         </is>
       </c>
       <c r="J24" s="0" t="n">
@@ -2592,46 +2592,46 @@
         <v>0.0</v>
       </c>
       <c r="L24" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M24" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N24" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O24" s="0" t="n">
-        <v>1305.0</v>
+        <v>739.5</v>
       </c>
       <c r="P24" s="0" t="n">
-        <v>454.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q24" s="0" t="n">
-        <v>43241.0</v>
+        <v>24501.5</v>
       </c>
       <c r="R24" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza</t>
+          <t>Jonatan Oregon Mendez</t>
         </is>
       </c>
       <c r="S24" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="T24" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="U24" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
+          <t>Jonatan Oregon</t>
         </is>
       </c>
       <c r="V24" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W24" s="0"/>
@@ -2649,21 +2649,21 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:45</t>
+          <t>2026/04/17 16:38:42</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:47</t>
+          <t>2026/04/17 16:38:44</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>822722120121735725056</t>
+          <t>822724934643911520256</t>
         </is>
       </c>
       <c r="D25" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J25" s="0" t="n">
@@ -2697,46 +2697,46 @@
         <v>0.0</v>
       </c>
       <c r="L25" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="M25" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N25" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="O25" s="0" t="n">
-        <v>1530.0</v>
+        <v>2397.0</v>
       </c>
       <c r="P25" s="0" t="n">
-        <v>454.0</v>
+        <v>709.0</v>
       </c>
       <c r="Q25" s="0" t="n">
-        <v>43016.0</v>
+        <v>67394.0</v>
       </c>
       <c r="R25" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac</t>
+          <t>Marcela Alvarez Campos</t>
         </is>
       </c>
       <c r="S25" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com</t>
+          <t>marcela.ac@me.com</t>
         </is>
       </c>
       <c r="T25" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
+          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
         </is>
       </c>
       <c r="U25" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac, Gabriela Vazquez</t>
+          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
         </is>
       </c>
       <c r="V25" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W25" s="0"/>
@@ -2754,17 +2754,17 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:14</t>
+          <t>2026/04/13 22:04:28</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:16</t>
+          <t>2026/04/13 22:04:30</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>822718782367677300736</t>
+          <t>822722199504844500992</t>
         </is>
       </c>
       <c r="D26" s="0" t="n">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t>7348</t>
+          <t>4291</t>
         </is>
       </c>
       <c r="J26" s="0" t="n">
@@ -2821,27 +2821,27 @@
       </c>
       <c r="R26" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera Lima</t>
+          <t>Carlos Mendoza</t>
         </is>
       </c>
       <c r="S26" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx</t>
+          <t>mendoza.carlos.a@gmail.com</t>
         </is>
       </c>
       <c r="T26" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
         </is>
       </c>
       <c r="U26" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
+          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
         </is>
       </c>
       <c r="V26" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W26" s="0"/>
@@ -2859,17 +2859,17 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:52</t>
+          <t>2026/04/13 19:26:45</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:54</t>
+          <t>2026/04/13 19:26:47</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>822717931075648110592</t>
+          <t>822722120121735725056</t>
         </is>
       </c>
       <c r="D27" s="0" t="n">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="I27" s="0" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="J27" s="0" t="n">
@@ -2926,22 +2926,22 @@
       </c>
       <c r="R27" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+          <t>Ana paula Isaac</t>
         </is>
       </c>
       <c r="S27" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com</t>
+          <t>anapauisaac@gmail.com</t>
         </is>
       </c>
       <c r="T27" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
         </is>
       </c>
       <c r="U27" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+          <t>Ana paula Isaac, Gabriela Vazquez</t>
         </is>
       </c>
       <c r="V27" s="0" t="inlineStr">
@@ -2964,21 +2964,21 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:06</t>
+          <t>2026/04/09 04:55:14</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:09</t>
+          <t>2026/04/09 04:55:16</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>822717887408069685248</t>
+          <t>822718782367677300736</t>
         </is>
       </c>
       <c r="D28" s="0" t="n">
-        <v>31500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
@@ -2992,17 +2992,17 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>apple_pay</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I28" s="0" t="inlineStr">
         <is>
-          <t>4006</t>
+          <t>7348</t>
         </is>
       </c>
       <c r="J28" s="0" t="n">
@@ -3012,41 +3012,41 @@
         <v>0.0</v>
       </c>
       <c r="L28" s="0" t="n">
-        <v>31500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M28" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N28" s="0" t="n">
-        <v>31500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O28" s="0" t="n">
-        <v>1071.0</v>
+        <v>1305.0</v>
       </c>
       <c r="P28" s="0" t="n">
-        <v>319.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q28" s="0" t="n">
-        <v>30110.0</v>
+        <v>43241.0</v>
       </c>
       <c r="R28" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago</t>
+          <t>Francisco Javier Vera Lima</t>
         </is>
       </c>
       <c r="S28" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com</t>
+          <t>fjvera@vmodal.mx</t>
         </is>
       </c>
       <c r="T28" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
         </is>
       </c>
       <c r="U28" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago, Michelle Ralph</t>
+          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
         </is>
       </c>
       <c r="V28" s="0" t="inlineStr">
@@ -3069,21 +3069,21 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:57</t>
+          <t>2026/04/08 00:43:52</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:59</t>
+          <t>2026/04/08 00:43:54</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>822717804781623066624</t>
+          <t>822717931075648110592</t>
         </is>
       </c>
       <c r="D29" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -3102,12 +3102,12 @@
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t>3513</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="J29" s="0" t="n">
@@ -3117,46 +3117,46 @@
         <v>0.0</v>
       </c>
       <c r="L29" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M29" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N29" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O29" s="0" t="n">
-        <v>739.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P29" s="0" t="n">
-        <v>259.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q29" s="0" t="n">
-        <v>24501.5</v>
+        <v>43016.0</v>
       </c>
       <c r="R29" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
         </is>
       </c>
       <c r="S29" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>mardoqueorq@hotmail.com</t>
         </is>
       </c>
       <c r="T29" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
         </is>
       </c>
       <c r="U29" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
         </is>
       </c>
       <c r="V29" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W29" s="0"/>
@@ -3174,21 +3174,21 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:51</t>
+          <t>2026/04/07 23:17:06</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:53</t>
+          <t>2026/04/07 23:17:09</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>822717250585584762880</t>
+          <t>822717887408069685248</t>
         </is>
       </c>
       <c r="D30" s="0" t="n">
-        <v>45000.0</v>
+        <v>31500.0</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>4006</t>
         </is>
       </c>
       <c r="J30" s="0" t="n">
@@ -3222,46 +3222,46 @@
         <v>0.0</v>
       </c>
       <c r="L30" s="0" t="n">
-        <v>45000.0</v>
+        <v>31500.0</v>
       </c>
       <c r="M30" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N30" s="0" t="n">
-        <v>45000.0</v>
+        <v>31500.0</v>
       </c>
       <c r="O30" s="0" t="n">
-        <v>1530.0</v>
+        <v>1071.0</v>
       </c>
       <c r="P30" s="0" t="n">
-        <v>454.0</v>
+        <v>319.0</v>
       </c>
       <c r="Q30" s="0" t="n">
-        <v>43016.0</v>
+        <v>30110.0</v>
       </c>
       <c r="R30" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion</t>
+          <t>Eduardo Zago</t>
         </is>
       </c>
       <c r="S30" s="0" t="inlineStr">
         <is>
-          <t>sofiacarrioncobian@hotmail.com</t>
+          <t>eddiezago500@gmail.com</t>
         </is>
       </c>
       <c r="T30" s="0" t="inlineStr">
         <is>
-          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
         </is>
       </c>
       <c r="U30" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion, Ana María Carrion</t>
+          <t>Eduardo Zago, Michelle Ralph</t>
         </is>
       </c>
       <c r="V30" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W30" s="0"/>
@@ -3271,6 +3271,216 @@
         </is>
       </c>
       <c r="Y30" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:57</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:59</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>822717804781623066624</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H31" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I31" s="0" t="inlineStr">
+        <is>
+          <t>3513</t>
+        </is>
+      </c>
+      <c r="J31" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K31" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L31" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="M31" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N31" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="O31" s="0" t="n">
+        <v>739.5</v>
+      </c>
+      <c r="P31" s="0" t="n">
+        <v>259.0</v>
+      </c>
+      <c r="Q31" s="0" t="n">
+        <v>24501.5</v>
+      </c>
+      <c r="R31" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="S31" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="T31" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="U31" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="V31" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W31" s="0"/>
+      <c r="X31" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y31" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:51</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:53</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>822717250585584762880</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H32" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I32" s="0" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="J32" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K32" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L32" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M32" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N32" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O32" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P32" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q32" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R32" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion</t>
+        </is>
+      </c>
+      <c r="S32" s="0" t="inlineStr">
+        <is>
+          <t>sofiacarrioncobian@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T32" s="0" t="inlineStr">
+        <is>
+          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+        </is>
+      </c>
+      <c r="U32" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion, Ana María Carrion</t>
+        </is>
+      </c>
+      <c r="V32" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W32" s="0"/>
+      <c r="X32" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y32" s="0" t="inlineStr">
         <is>
           <t>daniel@akampa.mx</t>
         </is>

</xml_diff>

<commit_message>
📥 WeTravel: Reporting_Payments_WeTravel-539682-1779077848.xlsx (2026-05-18)
</commit_message>
<xml_diff>
--- a/reportes/Reporting_Payments_WeTravel.xlsx
+++ b/reportes/Reporting_Payments_WeTravel.xlsx
@@ -82,7 +82,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y32"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="29.4" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -242,17 +242,17 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/15 17:24:50</t>
+          <t>2026/05/18 01:01:03</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/15 17:24:53</t>
+          <t>2026/05/18 01:01:18</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>822745251580101009408</t>
+          <t>822746930752535928832</t>
         </is>
       </c>
       <c r="D2" s="0" t="n">
@@ -275,12 +275,12 @@
       </c>
       <c r="H2" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>3097</t>
+          <t>6353</t>
         </is>
       </c>
       <c r="J2" s="0" t="n">
@@ -299,37 +299,37 @@
         <v>22500.0</v>
       </c>
       <c r="O2" s="0" t="n">
-        <v>652.5</v>
+        <v>337.5</v>
       </c>
       <c r="P2" s="0" t="n">
         <v>229.0</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <v>21618.5</v>
+        <v>21933.5</v>
       </c>
       <c r="R2" s="0" t="inlineStr">
         <is>
-          <t>Marihel Arias</t>
+          <t>Sasha Porteny</t>
         </is>
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t>marihel_arias@hotmail.com</t>
+          <t>sashaglatt@gmail.com</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
+          <t>sashaglatt@gmail.com, trietedouard@gmail.com</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
         <is>
-          <t>Marihel Arias, Alondra Arias</t>
+          <t>Sasha Glatt Porteny, Edouard Triet</t>
         </is>
       </c>
       <c r="V2" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W2" s="0"/>
@@ -347,17 +347,17 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/14 21:47:03</t>
+          <t>2026/05/17 15:13:36</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/14 21:47:05</t>
+          <t>2026/05/17 15:13:38</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>822744658783664881664</t>
+          <t>822746635081215909888</t>
         </is>
       </c>
       <c r="D3" s="0" t="n">
@@ -385,7 +385,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="J3" s="0" t="n">
@@ -414,22 +414,22 @@
       </c>
       <c r="R3" s="0" t="inlineStr">
         <is>
-          <t>FERNANDO FONSECA</t>
+          <t>SIMON NATHAN GITTLER</t>
         </is>
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t>fonsecaf88@gmail.com</t>
+          <t>simon.gitt@gmail.com</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t>fonsecaf88@gmail.com, fonsecaf88@gmail.com</t>
+          <t>simon.gitt@gmail.com, halina@hadasa.com.mx</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t>FERNANDO FONSECA, Matias fonseca</t>
+          <t>SIMON NATHAN GITTLER SALOMON, Halina Unikel</t>
         </is>
       </c>
       <c r="V3" s="0" t="inlineStr">
@@ -452,21 +452,21 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:31</t>
+          <t>2026/05/17 03:20:35</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:33</t>
+          <t>2026/05/17 03:20:37</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>822743406261352546304</t>
+          <t>822746276208009285632</t>
         </is>
       </c>
       <c r="D4" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
@@ -500,46 +500,46 @@
         <v>0.0</v>
       </c>
       <c r="L4" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M4" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N4" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O4" s="0" t="n">
-        <v>433.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P4" s="0" t="n">
-        <v>131.5</v>
+        <v>454.0</v>
       </c>
       <c r="Q4" s="0" t="n">
-        <v>12185.0</v>
+        <v>43016.0</v>
       </c>
       <c r="R4" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Mauricio Schiavon magaña</t>
         </is>
       </c>
       <c r="S4" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>mschiavon@me.com</t>
         </is>
       </c>
       <c r="T4" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>mschiavon@me.com, mschiavon@me.com</t>
         </is>
       </c>
       <c r="U4" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Mauricio Esteban Schiavon Magaña, Mauricio Esteban Schiavon Magaña</t>
         </is>
       </c>
       <c r="V4" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W4" s="0"/>
@@ -557,21 +557,21 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:03</t>
+          <t>2026/05/16 16:30:32</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:05</t>
+          <t>2026/05/16 23:29:12</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>822743384884528578560</t>
+          <t>822745949026787532800</t>
         </is>
       </c>
       <c r="D5" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
@@ -585,19 +585,15 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>spei</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I5" s="0" t="inlineStr">
-        <is>
-          <t>7758</t>
-        </is>
-      </c>
+          <t>SPEI</t>
+        </is>
+      </c>
+      <c r="I5" s="0"/>
       <c r="J5" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -605,41 +601,41 @@
         <v>0.0</v>
       </c>
       <c r="L5" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M5" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N5" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O5" s="0" t="n">
-        <v>369.75</v>
+        <v>0.0</v>
       </c>
       <c r="P5" s="0" t="n">
-        <v>131.5</v>
+        <v>454.0</v>
       </c>
       <c r="Q5" s="0" t="n">
-        <v>12248.75</v>
+        <v>44546.0</v>
       </c>
       <c r="R5" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>Miguel Ángel Garcia</t>
         </is>
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>miguel@garcia.mx</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>Miguel@garcia.mx, Paonany8@gmail.com</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>Miguel Ángel Garcia, María Elena Sánche</t>
         </is>
       </c>
       <c r="V5" s="0" t="inlineStr">
@@ -662,17 +658,17 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:39</t>
+          <t>2026/05/15 17:24:50</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:41</t>
+          <t>2026/05/15 17:24:53</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>822743194435830431744</t>
+          <t>822745251580101009408</t>
         </is>
       </c>
       <c r="D6" s="0" t="n">
@@ -695,12 +691,12 @@
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t>9925</t>
+          <t>3097</t>
         </is>
       </c>
       <c r="J6" s="0" t="n">
@@ -729,27 +725,27 @@
       </c>
       <c r="R6" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>Marihel Arias</t>
         </is>
       </c>
       <c r="S6" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>marihel_arias@hotmail.com</t>
         </is>
       </c>
       <c r="T6" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
         </is>
       </c>
       <c r="U6" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>Marihel Arias, Alondra Arias</t>
         </is>
       </c>
       <c r="V6" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W6" s="0"/>
@@ -767,21 +763,21 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:10:30</t>
+          <t>2026/05/14 21:47:03</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:11:16</t>
+          <t>2026/05/14 21:47:05</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>822743130440389902336</t>
+          <t>822744658783664881664</t>
         </is>
       </c>
       <c r="D7" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
@@ -800,12 +796,12 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>1003</t>
         </is>
       </c>
       <c r="J7" s="0" t="n">
@@ -815,46 +811,46 @@
         <v>0.0</v>
       </c>
       <c r="L7" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M7" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N7" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>652.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P7" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q7" s="0" t="n">
-        <v>21618.5</v>
+        <v>43016.0</v>
       </c>
       <c r="R7" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>FERNANDO FONSECA</t>
         </is>
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>fonsecaf88@gmail.com, fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>FERNANDO FONSECA, Matias fonseca</t>
         </is>
       </c>
       <c r="V7" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W7" s="0"/>
@@ -872,21 +868,21 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:51</t>
+          <t>2026/05/13 04:18:31</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:53</t>
+          <t>2026/05/13 04:18:33</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>822743104942704197632</t>
+          <t>822743406261352546304</t>
         </is>
       </c>
       <c r="D8" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
@@ -905,12 +901,12 @@
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>1709</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="J8" s="0" t="n">
@@ -920,41 +916,41 @@
         <v>0.0</v>
       </c>
       <c r="L8" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M8" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N8" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O8" s="0" t="n">
-        <v>1305.0</v>
+        <v>433.5</v>
       </c>
       <c r="P8" s="0" t="n">
-        <v>454.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q8" s="0" t="n">
-        <v>43241.0</v>
+        <v>12185.0</v>
       </c>
       <c r="R8" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="V8" s="0" t="inlineStr">
@@ -977,21 +973,21 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/13 03:36:03</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/13 03:36:05</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>822742523051869483008</t>
+          <t>822743384884528578560</t>
         </is>
       </c>
       <c r="D9" s="0" t="n">
-        <v>20500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
@@ -1005,15 +1001,19 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="I9" s="0"/>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>7758</t>
+        </is>
+      </c>
       <c r="J9" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1021,46 +1021,46 @@
         <v>0.0</v>
       </c>
       <c r="L9" s="0" t="n">
-        <v>0.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M9" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N9" s="0" t="n">
-        <v>0.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O9" s="0" t="n">
-        <v>0.0</v>
+        <v>369.75</v>
       </c>
       <c r="P9" s="0" t="n">
-        <v>0.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q9" s="0" t="n">
-        <v>0.0</v>
+        <v>12248.75</v>
       </c>
       <c r="R9" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="V9" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W9" s="0"/>
@@ -1078,17 +1078,17 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:09</t>
+          <t>2026/05/12 21:17:39</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:12</t>
+          <t>2026/05/12 21:17:41</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>822742502121738878976</t>
+          <t>822743194435830431744</t>
         </is>
       </c>
       <c r="D10" s="0" t="n">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>1775</t>
+          <t>9925</t>
         </is>
       </c>
       <c r="J10" s="0" t="n">
@@ -1145,22 +1145,22 @@
       </c>
       <c r="R10" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri, Isabel Fernández</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V10" s="0" t="inlineStr">
@@ -1183,21 +1183,21 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:41</t>
+          <t>2026/05/12 19:10:30</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:43</t>
+          <t>2026/05/12 19:11:16</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>822740352219193810944</t>
+          <t>822743130440389902336</t>
         </is>
       </c>
       <c r="D11" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
@@ -1216,12 +1216,12 @@
       </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J11" s="0" t="n">
@@ -1231,46 +1231,46 @@
         <v>0.0</v>
       </c>
       <c r="L11" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M11" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N11" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O11" s="0" t="n">
-        <v>2754.0</v>
+        <v>652.5</v>
       </c>
       <c r="P11" s="0" t="n">
-        <v>814.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q11" s="0" t="n">
-        <v>77432.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R11" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S11" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T11" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U11" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V11" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W11" s="0"/>
@@ -1288,21 +1288,21 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:11</t>
+          <t>2026/05/12 18:19:51</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:12</t>
+          <t>2026/05/12 18:19:53</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>822740218587619794944</t>
+          <t>822743104942704197632</t>
         </is>
       </c>
       <c r="D12" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>6624</t>
+          <t>1709</t>
         </is>
       </c>
       <c r="J12" s="0" t="n">
@@ -1336,41 +1336,41 @@
         <v>0.0</v>
       </c>
       <c r="L12" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M12" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N12" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O12" s="0" t="n">
-        <v>739.5</v>
+        <v>1305.0</v>
       </c>
       <c r="P12" s="0" t="n">
-        <v>259.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q12" s="0" t="n">
-        <v>24501.5</v>
+        <v>43241.0</v>
       </c>
       <c r="R12" s="0" t="inlineStr">
         <is>
-          <t>MELB PEREZ SALDANA</t>
+          <t>RAFAEL BELTRAN LOPEZ</t>
         </is>
       </c>
       <c r="S12" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>rbeltran1976@hotmail.com</t>
         </is>
       </c>
       <c r="T12" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
         </is>
       </c>
       <c r="U12" s="0" t="inlineStr">
         <is>
-          <t>MELBA ASTRID PEREZ SALDAÑA</t>
+          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
         </is>
       </c>
       <c r="V12" s="0" t="inlineStr">
@@ -1393,21 +1393,21 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:10</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:12</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>822740202977192058880</t>
+          <t>822742523051869483008</t>
         </is>
       </c>
       <c r="D13" s="0" t="n">
-        <v>22500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
@@ -1421,19 +1421,15 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I13" s="0" t="inlineStr">
-        <is>
-          <t>9925</t>
-        </is>
-      </c>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I13" s="0"/>
       <c r="J13" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1441,46 +1437,46 @@
         <v>0.0</v>
       </c>
       <c r="L13" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M13" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N13" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O13" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P13" s="0" t="n">
-        <v>229.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q13" s="0" t="n">
-        <v>21618.5</v>
+        <v>0.0</v>
       </c>
       <c r="R13" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S13" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T13" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U13" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V13" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W13" s="0"/>
@@ -1498,17 +1494,17 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:20</t>
+          <t>2026/05/11 22:22:09</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:22</t>
+          <t>2026/05/11 22:22:12</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>822738944267014664192</t>
+          <t>822742502121738878976</t>
         </is>
       </c>
       <c r="D14" s="0" t="n">
@@ -1536,7 +1532,7 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t>6156</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="J14" s="0" t="n">
@@ -1565,27 +1561,27 @@
       </c>
       <c r="R14" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas</t>
+          <t>Macarena Olavarri</t>
         </is>
       </c>
       <c r="S14" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel</t>
+          <t>macaolavarri@gmail.com</t>
         </is>
       </c>
       <c r="T14" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
+          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
         </is>
       </c>
       <c r="U14" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas, Denisse Olivo</t>
+          <t>Macarena Olavarri, Isabel Fernández</t>
         </is>
       </c>
       <c r="V14" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W14" s="0"/>
@@ -1603,25 +1599,25 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>2026/05/06 23:07:12</t>
+          <t>2026/05/08 23:10:41</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:05:58</t>
+          <t>2026/05/08 23:10:43</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>822738900913572839424</t>
+          <t>822740352219193810944</t>
         </is>
       </c>
       <c r="D15" s="0" t="n">
-        <v>20500.0</v>
+        <v>81000.0</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Refunded</t>
+          <t>Successful</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
@@ -1631,62 +1627,66 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>transferencia</t>
-        </is>
-      </c>
-      <c r="I15" s="0"/>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I15" s="0" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
       <c r="J15" s="0" t="n">
-        <v>20500.0</v>
+        <v>0.0</v>
       </c>
       <c r="K15" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L15" s="0" t="n">
-        <v>0.0</v>
+        <v>81000.0</v>
       </c>
       <c r="M15" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N15" s="0" t="n">
-        <v>0.0</v>
+        <v>81000.0</v>
       </c>
       <c r="O15" s="0" t="n">
-        <v>0.0</v>
+        <v>2754.0</v>
       </c>
       <c r="P15" s="0" t="n">
-        <v>0.0</v>
+        <v>814.0</v>
       </c>
       <c r="Q15" s="0" t="n">
-        <v>0.0</v>
+        <v>77432.0</v>
       </c>
       <c r="R15" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Judith Escobar Torres</t>
         </is>
       </c>
       <c r="S15" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>judith.escobar@gmail.com</t>
         </is>
       </c>
       <c r="T15" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
         </is>
       </c>
       <c r="U15" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
         </is>
       </c>
       <c r="V15" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W15" s="0"/>
@@ -1704,21 +1704,21 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:40</t>
+          <t>2026/05/08 18:45:11</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:42</t>
+          <t>2026/05/08 18:45:12</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>822735991480689651712</t>
+          <t>822740218587619794944</t>
         </is>
       </c>
       <c r="D16" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t>2003</t>
+          <t>6624</t>
         </is>
       </c>
       <c r="J16" s="0" t="n">
@@ -1752,46 +1752,46 @@
         <v>0.0</v>
       </c>
       <c r="L16" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M16" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N16" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O16" s="0" t="n">
-        <v>1530.0</v>
+        <v>739.5</v>
       </c>
       <c r="P16" s="0" t="n">
-        <v>454.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q16" s="0" t="n">
-        <v>43016.0</v>
+        <v>24501.5</v>
       </c>
       <c r="R16" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES</t>
+          <t>MELB PEREZ SALDANA</t>
         </is>
       </c>
       <c r="S16" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="T16" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="U16" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
+          <t>MELBA ASTRID PEREZ SALDAÑA</t>
         </is>
       </c>
       <c r="V16" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W16" s="0"/>
@@ -1809,17 +1809,17 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:35</t>
+          <t>2026/05/08 18:14:10</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:36</t>
+          <t>2026/05/08 18:14:12</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>822733043006520176640</t>
+          <t>822740202977192058880</t>
         </is>
       </c>
       <c r="D17" s="0" t="n">
@@ -1842,12 +1842,12 @@
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>5558</t>
+          <t>9925</t>
         </is>
       </c>
       <c r="J17" s="0" t="n">
@@ -1876,27 +1876,27 @@
       </c>
       <c r="R17" s="0" t="inlineStr">
         <is>
-          <t>IGNACIO PORTILLA</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S17" s="0" t="inlineStr">
         <is>
-          <t>mx.portilla@gmail.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T17" s="0" t="inlineStr">
         <is>
-          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U17" s="0" t="inlineStr">
         <is>
-          <t>VALERIA PORTILLA, Natalia Portilla</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V17" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W17" s="0"/>
@@ -1914,21 +1914,21 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:10:30</t>
+          <t>2026/05/07 00:33:20</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:11:05</t>
+          <t>2026/05/07 00:33:22</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>822732983572553019392</t>
+          <t>822738944267014664192</t>
         </is>
       </c>
       <c r="D18" s="0" t="n">
-        <v>18000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -1947,12 +1947,12 @@
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>6156</t>
         </is>
       </c>
       <c r="J18" s="0" t="n">
@@ -1962,46 +1962,46 @@
         <v>0.0</v>
       </c>
       <c r="L18" s="0" t="n">
-        <v>18000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M18" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N18" s="0" t="n">
-        <v>18000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O18" s="0" t="n">
-        <v>522.0</v>
+        <v>652.5</v>
       </c>
       <c r="P18" s="0" t="n">
-        <v>184.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q18" s="0" t="n">
-        <v>17294.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R18" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>Alejandra Serpas</t>
         </is>
       </c>
       <c r="S18" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="T18" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="U18" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>Alejandra Serpas, Denisse Olivo</t>
         </is>
       </c>
       <c r="V18" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W18" s="0"/>
@@ -2019,25 +2019,25 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:49</t>
+          <t>2026/05/06 23:07:12</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:51</t>
+          <t>2026/05/11 23:05:58</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>822728072370714607616</t>
+          <t>822738900913572839424</t>
         </is>
       </c>
       <c r="D19" s="0" t="n">
-        <v>9833.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Successful</t>
+          <t>Refunded</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
@@ -2047,66 +2047,62 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I19" s="0" t="inlineStr">
-        <is>
-          <t>2071</t>
-        </is>
-      </c>
+          <t>transferencia</t>
+        </is>
+      </c>
+      <c r="I19" s="0"/>
       <c r="J19" s="0" t="n">
-        <v>0.0</v>
+        <v>20500.0</v>
       </c>
       <c r="K19" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L19" s="0" t="n">
-        <v>9833.0</v>
+        <v>0.0</v>
       </c>
       <c r="M19" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N19" s="0" t="n">
-        <v>9833.0</v>
+        <v>0.0</v>
       </c>
       <c r="O19" s="0" t="n">
-        <v>285.16</v>
+        <v>0.0</v>
       </c>
       <c r="P19" s="0" t="n">
-        <v>102.33</v>
+        <v>0.0</v>
       </c>
       <c r="Q19" s="0" t="n">
-        <v>9445.51</v>
+        <v>0.0</v>
       </c>
       <c r="R19" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S19" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T19" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U19" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V19" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W19" s="0"/>
@@ -2124,21 +2120,21 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:44</t>
+          <t>2026/05/02 22:46:40</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:46</t>
+          <t>2026/05/02 22:46:42</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>822728021498622136320</t>
+          <t>822735991480689651712</t>
         </is>
       </c>
       <c r="D20" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
@@ -2157,12 +2153,12 @@
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="J20" s="0" t="n">
@@ -2172,46 +2168,46 @@
         <v>0.0</v>
       </c>
       <c r="L20" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M20" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N20" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O20" s="0" t="n">
-        <v>652.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P20" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q20" s="0" t="n">
-        <v>21618.5</v>
+        <v>43016.0</v>
       </c>
       <c r="R20" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>ALEJANDRO CANALES MORALES</t>
         </is>
       </c>
       <c r="S20" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="T20" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="U20" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
         </is>
       </c>
       <c r="V20" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W20" s="0"/>
@@ -2229,17 +2225,17 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:01</t>
+          <t>2026/04/28 21:08:35</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:03</t>
+          <t>2026/04/28 21:08:36</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>822727454901268389888</t>
+          <t>822733043006520176640</t>
         </is>
       </c>
       <c r="D21" s="0" t="n">
@@ -2262,12 +2258,12 @@
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>5558</t>
         </is>
       </c>
       <c r="J21" s="0" t="n">
@@ -2296,27 +2292,27 @@
       </c>
       <c r="R21" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>IGNACIO PORTILLA</t>
         </is>
       </c>
       <c r="S21" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>mx.portilla@gmail.com</t>
         </is>
       </c>
       <c r="T21" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
         </is>
       </c>
       <c r="U21" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>VALERIA PORTILLA, Natalia Portilla</t>
         </is>
       </c>
       <c r="V21" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W21" s="0"/>
@@ -2334,21 +2330,21 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:12</t>
+          <t>2026/04/28 19:10:30</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:13</t>
+          <t>2026/04/28 19:11:05</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>822727364900010598400</t>
+          <t>822732983572553019392</t>
         </is>
       </c>
       <c r="D22" s="0" t="n">
-        <v>22500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -2372,7 +2368,7 @@
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t>7852</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J22" s="0" t="n">
@@ -2382,41 +2378,41 @@
         <v>0.0</v>
       </c>
       <c r="L22" s="0" t="n">
-        <v>22500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="M22" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N22" s="0" t="n">
-        <v>22500.0</v>
+        <v>18000.0</v>
       </c>
       <c r="O22" s="0" t="n">
-        <v>652.5</v>
+        <v>522.0</v>
       </c>
       <c r="P22" s="0" t="n">
-        <v>229.0</v>
+        <v>184.0</v>
       </c>
       <c r="Q22" s="0" t="n">
-        <v>21618.5</v>
+        <v>17294.0</v>
       </c>
       <c r="R22" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S22" s="0" t="inlineStr">
         <is>
-          <t>ricardocb23@gmail.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T22" s="0" t="inlineStr">
         <is>
-          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U22" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V22" s="0" t="inlineStr">
@@ -2439,21 +2435,21 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:19</t>
+          <t>2026/04/22 00:32:49</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:21</t>
+          <t>2026/04/22 00:32:51</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>822726495229304659968</t>
+          <t>822728072370714607616</t>
         </is>
       </c>
       <c r="D23" s="0" t="n">
-        <v>14750.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -2467,17 +2463,17 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>2071</t>
         </is>
       </c>
       <c r="J23" s="0" t="n">
@@ -2487,41 +2483,41 @@
         <v>0.0</v>
       </c>
       <c r="L23" s="0" t="n">
-        <v>14750.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M23" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N23" s="0" t="n">
-        <v>14750.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O23" s="0" t="n">
-        <v>427.75</v>
+        <v>285.16</v>
       </c>
       <c r="P23" s="0" t="n">
-        <v>151.5</v>
+        <v>102.33</v>
       </c>
       <c r="Q23" s="0" t="n">
-        <v>14170.75</v>
+        <v>9445.51</v>
       </c>
       <c r="R23" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="S23" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="T23" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="U23" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="V23" s="0" t="inlineStr">
@@ -2544,21 +2540,21 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:21</t>
+          <t>2026/04/21 22:51:44</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:23</t>
+          <t>2026/04/21 22:51:46</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>822725726179188305920</t>
+          <t>822728021498622136320</t>
         </is>
       </c>
       <c r="D24" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -2582,7 +2578,7 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t>9962</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J24" s="0" t="n">
@@ -2592,46 +2588,46 @@
         <v>0.0</v>
       </c>
       <c r="L24" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M24" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N24" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O24" s="0" t="n">
-        <v>739.5</v>
+        <v>652.5</v>
       </c>
       <c r="P24" s="0" t="n">
-        <v>259.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q24" s="0" t="n">
-        <v>24501.5</v>
+        <v>21618.5</v>
       </c>
       <c r="R24" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon Mendez</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S24" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T24" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U24" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V24" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W24" s="0"/>
@@ -2649,21 +2645,21 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:42</t>
+          <t>2026/04/21 04:06:01</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:44</t>
+          <t>2026/04/21 04:06:03</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>822724934643911520256</t>
+          <t>822727454901268389888</t>
         </is>
       </c>
       <c r="D25" s="0" t="n">
-        <v>70500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -2682,12 +2678,12 @@
       </c>
       <c r="H25" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J25" s="0" t="n">
@@ -2697,46 +2693,46 @@
         <v>0.0</v>
       </c>
       <c r="L25" s="0" t="n">
-        <v>70500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M25" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N25" s="0" t="n">
-        <v>70500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O25" s="0" t="n">
-        <v>2397.0</v>
+        <v>652.5</v>
       </c>
       <c r="P25" s="0" t="n">
-        <v>709.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q25" s="0" t="n">
-        <v>67394.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R25" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S25" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T25" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U25" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V25" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W25" s="0"/>
@@ -2754,21 +2750,21 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:28</t>
+          <t>2026/04/21 01:07:12</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:30</t>
+          <t>2026/04/21 01:07:13</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>822722199504844500992</t>
+          <t>822727364900010598400</t>
         </is>
       </c>
       <c r="D26" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -2792,7 +2788,7 @@
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t>4291</t>
+          <t>7852</t>
         </is>
       </c>
       <c r="J26" s="0" t="n">
@@ -2802,41 +2798,41 @@
         <v>0.0</v>
       </c>
       <c r="L26" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M26" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N26" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O26" s="0" t="n">
-        <v>1305.0</v>
+        <v>652.5</v>
       </c>
       <c r="P26" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q26" s="0" t="n">
-        <v>43241.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R26" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza</t>
+          <t>RICARDO CAMACHO BOFILL</t>
         </is>
       </c>
       <c r="S26" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com</t>
+          <t>ricardocb23@gmail.com</t>
         </is>
       </c>
       <c r="T26" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
+          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
         </is>
       </c>
       <c r="U26" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
+          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
         </is>
       </c>
       <c r="V26" s="0" t="inlineStr">
@@ -2859,21 +2855,21 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:45</t>
+          <t>2026/04/19 20:19:19</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:47</t>
+          <t>2026/04/19 20:19:21</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>822722120121735725056</t>
+          <t>822726495229304659968</t>
         </is>
       </c>
       <c r="D27" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -2887,7 +2883,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>apple_pay</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -2897,7 +2893,7 @@
       </c>
       <c r="I27" s="0" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="J27" s="0" t="n">
@@ -2907,46 +2903,46 @@
         <v>0.0</v>
       </c>
       <c r="L27" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="M27" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N27" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="O27" s="0" t="n">
-        <v>1530.0</v>
+        <v>427.75</v>
       </c>
       <c r="P27" s="0" t="n">
-        <v>454.0</v>
+        <v>151.5</v>
       </c>
       <c r="Q27" s="0" t="n">
-        <v>43016.0</v>
+        <v>14170.75</v>
       </c>
       <c r="R27" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="S27" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="T27" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="U27" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac, Gabriela Vazquez</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="V27" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W27" s="0"/>
@@ -2964,21 +2960,21 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:14</t>
+          <t>2026/04/18 18:51:21</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:16</t>
+          <t>2026/04/18 18:51:23</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>822718782367677300736</t>
+          <t>822725726179188305920</t>
         </is>
       </c>
       <c r="D28" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
@@ -2992,7 +2988,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -3002,7 +2998,7 @@
       </c>
       <c r="I28" s="0" t="inlineStr">
         <is>
-          <t>7348</t>
+          <t>9962</t>
         </is>
       </c>
       <c r="J28" s="0" t="n">
@@ -3012,41 +3008,41 @@
         <v>0.0</v>
       </c>
       <c r="L28" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M28" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N28" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O28" s="0" t="n">
-        <v>1305.0</v>
+        <v>739.5</v>
       </c>
       <c r="P28" s="0" t="n">
-        <v>454.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q28" s="0" t="n">
-        <v>43241.0</v>
+        <v>24501.5</v>
       </c>
       <c r="R28" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera Lima</t>
+          <t>Jonatan Oregon Mendez</t>
         </is>
       </c>
       <c r="S28" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="T28" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="U28" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
+          <t>Jonatan Oregon</t>
         </is>
       </c>
       <c r="V28" s="0" t="inlineStr">
@@ -3069,21 +3065,21 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:52</t>
+          <t>2026/04/17 16:38:42</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:54</t>
+          <t>2026/04/17 16:38:44</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>822717931075648110592</t>
+          <t>822724934643911520256</t>
         </is>
       </c>
       <c r="D29" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -3107,7 +3103,7 @@
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J29" s="0" t="n">
@@ -3117,46 +3113,46 @@
         <v>0.0</v>
       </c>
       <c r="L29" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="M29" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N29" s="0" t="n">
-        <v>45000.0</v>
+        <v>70500.0</v>
       </c>
       <c r="O29" s="0" t="n">
-        <v>1530.0</v>
+        <v>2397.0</v>
       </c>
       <c r="P29" s="0" t="n">
-        <v>454.0</v>
+        <v>709.0</v>
       </c>
       <c r="Q29" s="0" t="n">
-        <v>43016.0</v>
+        <v>67394.0</v>
       </c>
       <c r="R29" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+          <t>Marcela Alvarez Campos</t>
         </is>
       </c>
       <c r="S29" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com</t>
+          <t>marcela.ac@me.com</t>
         </is>
       </c>
       <c r="T29" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
         </is>
       </c>
       <c r="U29" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
         </is>
       </c>
       <c r="V29" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W29" s="0"/>
@@ -3174,21 +3170,21 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:06</t>
+          <t>2026/04/13 22:04:28</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:09</t>
+          <t>2026/04/13 22:04:30</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>822717887408069685248</t>
+          <t>822722199504844500992</t>
         </is>
       </c>
       <c r="D30" s="0" t="n">
-        <v>31500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -3207,12 +3203,12 @@
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t>4006</t>
+          <t>4291</t>
         </is>
       </c>
       <c r="J30" s="0" t="n">
@@ -3222,46 +3218,46 @@
         <v>0.0</v>
       </c>
       <c r="L30" s="0" t="n">
-        <v>31500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M30" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N30" s="0" t="n">
-        <v>31500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O30" s="0" t="n">
-        <v>1071.0</v>
+        <v>1305.0</v>
       </c>
       <c r="P30" s="0" t="n">
-        <v>319.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q30" s="0" t="n">
-        <v>30110.0</v>
+        <v>43241.0</v>
       </c>
       <c r="R30" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago</t>
+          <t>Carlos Mendoza</t>
         </is>
       </c>
       <c r="S30" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com</t>
+          <t>mendoza.carlos.a@gmail.com</t>
         </is>
       </c>
       <c r="T30" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
         </is>
       </c>
       <c r="U30" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago, Michelle Ralph</t>
+          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
         </is>
       </c>
       <c r="V30" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W30" s="0"/>
@@ -3279,21 +3275,21 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:57</t>
+          <t>2026/04/13 19:26:45</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:59</t>
+          <t>2026/04/13 19:26:47</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>822717804781623066624</t>
+          <t>822722120121735725056</t>
         </is>
       </c>
       <c r="D31" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
@@ -3312,12 +3308,12 @@
       </c>
       <c r="H31" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I31" s="0" t="inlineStr">
         <is>
-          <t>3513</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="J31" s="0" t="n">
@@ -3327,46 +3323,46 @@
         <v>0.0</v>
       </c>
       <c r="L31" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M31" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N31" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O31" s="0" t="n">
-        <v>739.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P31" s="0" t="n">
-        <v>259.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q31" s="0" t="n">
-        <v>24501.5</v>
+        <v>43016.0</v>
       </c>
       <c r="R31" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>Ana paula Isaac</t>
         </is>
       </c>
       <c r="S31" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>anapauisaac@gmail.com</t>
         </is>
       </c>
       <c r="T31" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
         </is>
       </c>
       <c r="U31" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>Ana paula Isaac, Gabriela Vazquez</t>
         </is>
       </c>
       <c r="V31" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W31" s="0"/>
@@ -3384,17 +3380,17 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:51</t>
+          <t>2026/04/09 04:55:14</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:53</t>
+          <t>2026/04/09 04:55:16</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>822717250585584762880</t>
+          <t>822718782367677300736</t>
         </is>
       </c>
       <c r="D32" s="0" t="n">
@@ -3412,17 +3408,17 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>apple_pay</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>7348</t>
         </is>
       </c>
       <c r="J32" s="0" t="n">
@@ -3441,37 +3437,37 @@
         <v>45000.0</v>
       </c>
       <c r="O32" s="0" t="n">
-        <v>1530.0</v>
+        <v>1305.0</v>
       </c>
       <c r="P32" s="0" t="n">
         <v>454.0</v>
       </c>
       <c r="Q32" s="0" t="n">
-        <v>43016.0</v>
+        <v>43241.0</v>
       </c>
       <c r="R32" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion</t>
+          <t>Francisco Javier Vera Lima</t>
         </is>
       </c>
       <c r="S32" s="0" t="inlineStr">
         <is>
-          <t>sofiacarrioncobian@hotmail.com</t>
+          <t>fjvera@vmodal.mx</t>
         </is>
       </c>
       <c r="T32" s="0" t="inlineStr">
         <is>
-          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
         </is>
       </c>
       <c r="U32" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion, Ana María Carrion</t>
+          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
         </is>
       </c>
       <c r="V32" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W32" s="0"/>
@@ -3481,6 +3477,426 @@
         </is>
       </c>
       <c r="Y32" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:52</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:54</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>822717931075648110592</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H33" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I33" s="0" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="J33" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K33" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L33" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M33" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N33" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O33" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P33" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q33" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R33" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+        </is>
+      </c>
+      <c r="S33" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T33" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+        </is>
+      </c>
+      <c r="U33" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+        </is>
+      </c>
+      <c r="V33" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W33" s="0"/>
+      <c r="X33" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y33" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:06</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:09</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>822717887408069685248</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I34" s="0" t="inlineStr">
+        <is>
+          <t>4006</t>
+        </is>
+      </c>
+      <c r="J34" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K34" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L34" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="M34" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N34" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="O34" s="0" t="n">
+        <v>1071.0</v>
+      </c>
+      <c r="P34" s="0" t="n">
+        <v>319.0</v>
+      </c>
+      <c r="Q34" s="0" t="n">
+        <v>30110.0</v>
+      </c>
+      <c r="R34" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago</t>
+        </is>
+      </c>
+      <c r="S34" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com</t>
+        </is>
+      </c>
+      <c r="T34" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+        </is>
+      </c>
+      <c r="U34" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago, Michelle Ralph</t>
+        </is>
+      </c>
+      <c r="V34" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W34" s="0"/>
+      <c r="X34" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y34" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:57</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:59</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>822717804781623066624</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I35" s="0" t="inlineStr">
+        <is>
+          <t>3513</t>
+        </is>
+      </c>
+      <c r="J35" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K35" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L35" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="M35" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N35" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="O35" s="0" t="n">
+        <v>739.5</v>
+      </c>
+      <c r="P35" s="0" t="n">
+        <v>259.0</v>
+      </c>
+      <c r="Q35" s="0" t="n">
+        <v>24501.5</v>
+      </c>
+      <c r="R35" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="S35" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="T35" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="U35" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="V35" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W35" s="0"/>
+      <c r="X35" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y35" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:51</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:53</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>822717250585584762880</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F36" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H36" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I36" s="0" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="J36" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K36" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L36" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M36" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N36" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O36" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P36" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q36" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R36" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion</t>
+        </is>
+      </c>
+      <c r="S36" s="0" t="inlineStr">
+        <is>
+          <t>sofiacarrioncobian@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T36" s="0" t="inlineStr">
+        <is>
+          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+        </is>
+      </c>
+      <c r="U36" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion, Ana María Carrion</t>
+        </is>
+      </c>
+      <c r="V36" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W36" s="0"/>
+      <c r="X36" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y36" s="0" t="inlineStr">
         <is>
           <t>daniel@akampa.mx</t>
         </is>

</xml_diff>

<commit_message>
📥 WeTravel: Reporting_Payments_WeTravel-539682-1779387048.xlsx (2026-05-21)
</commit_message>
<xml_diff>
--- a/reportes/Reporting_Payments_WeTravel.xlsx
+++ b/reportes/Reporting_Payments_WeTravel.xlsx
@@ -82,7 +82,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y36"/>
+  <dimension ref="A1:Y45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="29.4" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -242,21 +242,21 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 01:01:03</t>
+          <t>2026/05/21 17:22:39</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 01:01:18</t>
+          <t>2026/05/21 17:22:42</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>822746930752535928832</t>
+          <t>822749599136998244352</t>
         </is>
       </c>
       <c r="D2" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
@@ -275,12 +275,12 @@
       </c>
       <c r="H2" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>6353</t>
+          <t>2500</t>
         </is>
       </c>
       <c r="J2" s="0" t="n">
@@ -290,46 +290,46 @@
         <v>0.0</v>
       </c>
       <c r="L2" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M2" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N2" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O2" s="0" t="n">
-        <v>337.5</v>
+        <v>285.16</v>
       </c>
       <c r="P2" s="0" t="n">
-        <v>229.0</v>
+        <v>102.33</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <v>21933.5</v>
+        <v>9445.51</v>
       </c>
       <c r="R2" s="0" t="inlineStr">
         <is>
-          <t>Sasha Porteny</t>
+          <t>Leah Pages</t>
         </is>
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t>sashaglatt@gmail.com</t>
+          <t>pagesnava.leah@gmail.com</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t>sashaglatt@gmail.com, trietedouard@gmail.com</t>
+          <t>Pagesnava.leah@gmail.com</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
         <is>
-          <t>Sasha Glatt Porteny, Edouard Triet</t>
+          <t>Leah Pages</t>
         </is>
       </c>
       <c r="V2" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W2" s="0"/>
@@ -347,21 +347,21 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 15:13:36</t>
+          <t>2026/05/20 23:14:50</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 15:13:38</t>
+          <t>2026/05/20 23:14:51</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>822746635081215909888</t>
+          <t>822749051616429613056</t>
         </is>
       </c>
       <c r="D3" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
@@ -385,7 +385,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J3" s="0" t="n">
@@ -395,46 +395,46 @@
         <v>0.0</v>
       </c>
       <c r="L3" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M3" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N3" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O3" s="0" t="n">
-        <v>1530.0</v>
+        <v>867.0</v>
       </c>
       <c r="P3" s="0" t="n">
-        <v>454.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q3" s="0" t="n">
-        <v>43016.0</v>
+        <v>24374.0</v>
       </c>
       <c r="R3" s="0" t="inlineStr">
         <is>
-          <t>SIMON NATHAN GITTLER</t>
+          <t>Rodrigo Aviles</t>
         </is>
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t>simon.gitt@gmail.com</t>
+          <t>avilo26@hotmail.com</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t>simon.gitt@gmail.com, halina@hadasa.com.mx</t>
+          <t>avilo26@hotmail.com</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t>SIMON NATHAN GITTLER SALOMON, Halina Unikel</t>
+          <t>Rodrigo Aviles</t>
         </is>
       </c>
       <c r="V3" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W3" s="0"/>
@@ -452,21 +452,21 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 03:20:35</t>
+          <t>2026/05/20 17:53:15</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 03:20:37</t>
+          <t>2026/05/20 17:53:18</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>822746276208009285632</t>
+          <t>822748889761073610752</t>
         </is>
       </c>
       <c r="D4" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
@@ -485,12 +485,12 @@
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>1009</t>
+          <t>3493</t>
         </is>
       </c>
       <c r="J4" s="0" t="n">
@@ -500,46 +500,46 @@
         <v>0.0</v>
       </c>
       <c r="L4" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M4" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N4" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O4" s="0" t="n">
-        <v>1530.0</v>
+        <v>285.16</v>
       </c>
       <c r="P4" s="0" t="n">
-        <v>454.0</v>
+        <v>102.33</v>
       </c>
       <c r="Q4" s="0" t="n">
-        <v>43016.0</v>
+        <v>9445.51</v>
       </c>
       <c r="R4" s="0" t="inlineStr">
         <is>
-          <t>Mauricio Schiavon magaña</t>
+          <t>Liliana Osuna Domínguez</t>
         </is>
       </c>
       <c r="S4" s="0" t="inlineStr">
         <is>
-          <t>mschiavon@me.com</t>
+          <t>lilianaeod@gmail.com</t>
         </is>
       </c>
       <c r="T4" s="0" t="inlineStr">
         <is>
-          <t>mschiavon@me.com, mschiavon@me.com</t>
+          <t>Lilianaeod@gmail.com</t>
         </is>
       </c>
       <c r="U4" s="0" t="inlineStr">
         <is>
-          <t>Mauricio Esteban Schiavon Magaña, Mauricio Esteban Schiavon Magaña</t>
+          <t>Liliana Osuna Domínguez</t>
         </is>
       </c>
       <c r="V4" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W4" s="0"/>
@@ -557,21 +557,21 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/16 16:30:32</t>
+          <t>2026/05/20 17:09:53</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/16 23:29:12</t>
+          <t>2026/05/20 17:09:55</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>822745949026787532800</t>
+          <t>822748867929998106624</t>
         </is>
       </c>
       <c r="D5" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
@@ -585,15 +585,19 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>spei</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t>SPEI</t>
-        </is>
-      </c>
-      <c r="I5" s="0"/>
+          <t>mastercard</t>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>8841</t>
+        </is>
+      </c>
       <c r="J5" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -601,41 +605,41 @@
         <v>0.0</v>
       </c>
       <c r="L5" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M5" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N5" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O5" s="0" t="n">
-        <v>0.0</v>
+        <v>369.75</v>
       </c>
       <c r="P5" s="0" t="n">
-        <v>454.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q5" s="0" t="n">
-        <v>44546.0</v>
+        <v>12248.75</v>
       </c>
       <c r="R5" s="0" t="inlineStr">
         <is>
-          <t>Miguel Ángel Garcia</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t>miguel@garcia.mx</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t>Miguel@garcia.mx, Paonany8@gmail.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t>Miguel Ángel Garcia, María Elena Sánche</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="V5" s="0" t="inlineStr">
@@ -658,17 +662,17 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/15 17:24:50</t>
+          <t>2026/05/18 19:10:35</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/15 17:24:53</t>
+          <t>2026/05/18 19:11:23</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>822745251580101009408</t>
+          <t>822747479128876781568</t>
         </is>
       </c>
       <c r="D6" s="0" t="n">
@@ -763,21 +767,21 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/14 21:47:03</t>
+          <t>2026/05/18 19:10:33</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/14 21:47:05</t>
+          <t>2026/05/18 19:11:20</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>822744658783664881664</t>
+          <t>822747479118273585152</t>
         </is>
       </c>
       <c r="D7" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
@@ -801,7 +805,7 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="J7" s="0" t="n">
@@ -811,46 +815,46 @@
         <v>0.0</v>
       </c>
       <c r="L7" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M7" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N7" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>1530.0</v>
+        <v>433.5</v>
       </c>
       <c r="P7" s="0" t="n">
-        <v>454.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q7" s="0" t="n">
-        <v>43016.0</v>
+        <v>12185.0</v>
       </c>
       <c r="R7" s="0" t="inlineStr">
         <is>
-          <t>FERNANDO FONSECA</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t>fonsecaf88@gmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t>fonsecaf88@gmail.com, fonsecaf88@gmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
         <is>
-          <t>FERNANDO FONSECA, Matias fonseca</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="V7" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W7" s="0"/>
@@ -868,21 +872,21 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:31</t>
+          <t>2026/05/18 19:10:32</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:33</t>
+          <t>2026/05/18 19:11:18</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>822743406261352546304</t>
+          <t>822747479109650092032</t>
         </is>
       </c>
       <c r="D8" s="0" t="n">
-        <v>12750.0</v>
+        <v>18000.0</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
@@ -901,12 +905,12 @@
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>1009</t>
+          <t>6156</t>
         </is>
       </c>
       <c r="J8" s="0" t="n">
@@ -916,46 +920,46 @@
         <v>0.0</v>
       </c>
       <c r="L8" s="0" t="n">
-        <v>12750.0</v>
+        <v>18000.0</v>
       </c>
       <c r="M8" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N8" s="0" t="n">
-        <v>12750.0</v>
+        <v>18000.0</v>
       </c>
       <c r="O8" s="0" t="n">
-        <v>433.5</v>
+        <v>522.0</v>
       </c>
       <c r="P8" s="0" t="n">
-        <v>131.5</v>
+        <v>184.0</v>
       </c>
       <c r="Q8" s="0" t="n">
-        <v>12185.0</v>
+        <v>17294.0</v>
       </c>
       <c r="R8" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Alejandra Serpas</t>
         </is>
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Alejandra Serpas, Denisse Olivo</t>
         </is>
       </c>
       <c r="V8" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W8" s="0"/>
@@ -973,21 +977,21 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:03</t>
+          <t>2026/05/18 19:10:31</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:05</t>
+          <t>2026/05/18 19:11:14</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>822743384884528578560</t>
+          <t>822747479096832299008</t>
         </is>
       </c>
       <c r="D9" s="0" t="n">
-        <v>12750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
@@ -1006,12 +1010,12 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>7758</t>
+          <t>5558</t>
         </is>
       </c>
       <c r="J9" s="0" t="n">
@@ -1021,46 +1025,46 @@
         <v>0.0</v>
       </c>
       <c r="L9" s="0" t="n">
-        <v>12750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M9" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N9" s="0" t="n">
-        <v>12750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O9" s="0" t="n">
-        <v>369.75</v>
+        <v>652.5</v>
       </c>
       <c r="P9" s="0" t="n">
-        <v>131.5</v>
+        <v>229.0</v>
       </c>
       <c r="Q9" s="0" t="n">
-        <v>12248.75</v>
+        <v>21618.5</v>
       </c>
       <c r="R9" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>IGNACIO PORTILLA</t>
         </is>
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>mx.portilla@gmail.com</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>VALERIA PORTILLA, Natalia Portilla</t>
         </is>
       </c>
       <c r="V9" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W9" s="0"/>
@@ -1078,21 +1082,21 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:39</t>
+          <t>2026/05/18 16:14:03</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:41</t>
+          <t>2026/05/18 16:14:03</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>822743194435830431744</t>
+          <t>822747390277042835456</t>
         </is>
       </c>
       <c r="D10" s="0" t="n">
-        <v>22500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
@@ -1106,19 +1110,15 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I10" s="0" t="inlineStr">
-        <is>
-          <t>9925</t>
-        </is>
-      </c>
+          <t>Transferencia</t>
+        </is>
+      </c>
+      <c r="I10" s="0"/>
       <c r="J10" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1126,46 +1126,46 @@
         <v>0.0</v>
       </c>
       <c r="L10" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M10" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N10" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O10" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P10" s="0" t="n">
-        <v>229.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q10" s="0" t="n">
-        <v>21618.5</v>
+        <v>0.0</v>
       </c>
       <c r="R10" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V10" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W10" s="0"/>
@@ -1183,17 +1183,17 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:10:30</t>
+          <t>2026/05/18 01:01:03</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:11:16</t>
+          <t>2026/05/18 01:01:18</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>822743130440389902336</t>
+          <t>822746930752535928832</t>
         </is>
       </c>
       <c r="D11" s="0" t="n">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>6353</t>
         </is>
       </c>
       <c r="J11" s="0" t="n">
@@ -1240,32 +1240,32 @@
         <v>22500.0</v>
       </c>
       <c r="O11" s="0" t="n">
-        <v>652.5</v>
+        <v>337.5</v>
       </c>
       <c r="P11" s="0" t="n">
         <v>229.0</v>
       </c>
       <c r="Q11" s="0" t="n">
-        <v>21618.5</v>
+        <v>21933.5</v>
       </c>
       <c r="R11" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>Sasha Porteny</t>
         </is>
       </c>
       <c r="S11" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>sashaglatt@gmail.com</t>
         </is>
       </c>
       <c r="T11" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>sashaglatt@gmail.com, trietedouard@gmail.com</t>
         </is>
       </c>
       <c r="U11" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>Sasha Glatt Porteny, Edouard Triet</t>
         </is>
       </c>
       <c r="V11" s="0" t="inlineStr">
@@ -1288,17 +1288,17 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:51</t>
+          <t>2026/05/17 15:13:36</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:53</t>
+          <t>2026/05/17 15:13:38</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>822743104942704197632</t>
+          <t>822746635081215909888</t>
         </is>
       </c>
       <c r="D12" s="0" t="n">
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>1709</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="J12" s="0" t="n">
@@ -1345,37 +1345,37 @@
         <v>45000.0</v>
       </c>
       <c r="O12" s="0" t="n">
-        <v>1305.0</v>
+        <v>1530.0</v>
       </c>
       <c r="P12" s="0" t="n">
         <v>454.0</v>
       </c>
       <c r="Q12" s="0" t="n">
-        <v>43241.0</v>
+        <v>43016.0</v>
       </c>
       <c r="R12" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ</t>
+          <t>SIMON NATHAN GITTLER</t>
         </is>
       </c>
       <c r="S12" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com</t>
+          <t>simon.gitt@gmail.com</t>
         </is>
       </c>
       <c r="T12" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
+          <t>simon.gitt@gmail.com, halina@hadasa.com.mx</t>
         </is>
       </c>
       <c r="U12" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
+          <t>SIMON NATHAN GITTLER SALOMON, Halina Unikel</t>
         </is>
       </c>
       <c r="V12" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W12" s="0"/>
@@ -1393,21 +1393,21 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/17 03:20:35</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/17 03:20:37</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>822742523051869483008</t>
+          <t>822746276208009285632</t>
         </is>
       </c>
       <c r="D13" s="0" t="n">
-        <v>20500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
@@ -1421,15 +1421,19 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="I13" s="0"/>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>1009</t>
+        </is>
+      </c>
       <c r="J13" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1437,46 +1441,46 @@
         <v>0.0</v>
       </c>
       <c r="L13" s="0" t="n">
-        <v>0.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M13" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N13" s="0" t="n">
-        <v>0.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O13" s="0" t="n">
-        <v>0.0</v>
+        <v>1530.0</v>
       </c>
       <c r="P13" s="0" t="n">
-        <v>0.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q13" s="0" t="n">
-        <v>0.0</v>
+        <v>43016.0</v>
       </c>
       <c r="R13" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Mauricio Schiavon magaña</t>
         </is>
       </c>
       <c r="S13" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>mschiavon@me.com</t>
         </is>
       </c>
       <c r="T13" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>mschiavon@me.com, mschiavon@me.com</t>
         </is>
       </c>
       <c r="U13" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Mauricio Esteban Schiavon Magaña, Mauricio Esteban Schiavon Magaña</t>
         </is>
       </c>
       <c r="V13" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W13" s="0"/>
@@ -1494,21 +1498,21 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:09</t>
+          <t>2026/05/16 16:30:32</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:12</t>
+          <t>2026/05/16 23:29:12</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>822742502121738878976</t>
+          <t>822745949026787532800</t>
         </is>
       </c>
       <c r="D14" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
@@ -1522,19 +1526,15 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>spei</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
-        </is>
-      </c>
-      <c r="I14" s="0" t="inlineStr">
-        <is>
-          <t>1775</t>
-        </is>
-      </c>
+          <t>SPEI</t>
+        </is>
+      </c>
+      <c r="I14" s="0"/>
       <c r="J14" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1542,46 +1542,46 @@
         <v>0.0</v>
       </c>
       <c r="L14" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M14" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N14" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O14" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P14" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q14" s="0" t="n">
-        <v>21618.5</v>
+        <v>44546.0</v>
       </c>
       <c r="R14" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri</t>
+          <t>Miguel Ángel Garcia</t>
         </is>
       </c>
       <c r="S14" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com</t>
+          <t>miguel@garcia.mx</t>
         </is>
       </c>
       <c r="T14" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
+          <t>Miguel@garcia.mx, Paonany8@gmail.com</t>
         </is>
       </c>
       <c r="U14" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri, Isabel Fernández</t>
+          <t>Miguel Ángel Garcia, María Elena Sánche</t>
         </is>
       </c>
       <c r="V14" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W14" s="0"/>
@@ -1599,21 +1599,21 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:41</t>
+          <t>2026/05/15 17:24:50</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:43</t>
+          <t>2026/05/15 17:24:53</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>822740352219193810944</t>
+          <t>822745251580101009408</t>
         </is>
       </c>
       <c r="D15" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>3097</t>
         </is>
       </c>
       <c r="J15" s="0" t="n">
@@ -1647,41 +1647,41 @@
         <v>0.0</v>
       </c>
       <c r="L15" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M15" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N15" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O15" s="0" t="n">
-        <v>2754.0</v>
+        <v>652.5</v>
       </c>
       <c r="P15" s="0" t="n">
-        <v>814.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q15" s="0" t="n">
-        <v>77432.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R15" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres</t>
+          <t>Marihel Arias</t>
         </is>
       </c>
       <c r="S15" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com</t>
+          <t>marihel_arias@hotmail.com</t>
         </is>
       </c>
       <c r="T15" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
+          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
         </is>
       </c>
       <c r="U15" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
+          <t>Marihel Arias, Alondra Arias</t>
         </is>
       </c>
       <c r="V15" s="0" t="inlineStr">
@@ -1704,21 +1704,21 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:11</t>
+          <t>2026/05/14 21:47:03</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:12</t>
+          <t>2026/05/14 21:47:05</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>822740218587619794944</t>
+          <t>822744658783664881664</t>
         </is>
       </c>
       <c r="D16" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t>6624</t>
+          <t>1003</t>
         </is>
       </c>
       <c r="J16" s="0" t="n">
@@ -1752,46 +1752,46 @@
         <v>0.0</v>
       </c>
       <c r="L16" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M16" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N16" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O16" s="0" t="n">
-        <v>739.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P16" s="0" t="n">
-        <v>259.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q16" s="0" t="n">
-        <v>24501.5</v>
+        <v>43016.0</v>
       </c>
       <c r="R16" s="0" t="inlineStr">
         <is>
-          <t>MELB PEREZ SALDANA</t>
+          <t>FERNANDO FONSECA</t>
         </is>
       </c>
       <c r="S16" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="T16" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>fonsecaf88@gmail.com, fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="U16" s="0" t="inlineStr">
         <is>
-          <t>MELBA ASTRID PEREZ SALDAÑA</t>
+          <t>FERNANDO FONSECA, Matias fonseca</t>
         </is>
       </c>
       <c r="V16" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W16" s="0"/>
@@ -1809,21 +1809,21 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:10</t>
+          <t>2026/05/13 04:18:31</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:12</t>
+          <t>2026/05/13 04:18:33</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>822740202977192058880</t>
+          <t>822743406261352546304</t>
         </is>
       </c>
       <c r="D17" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
@@ -1842,12 +1842,12 @@
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>9925</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="J17" s="0" t="n">
@@ -1857,46 +1857,46 @@
         <v>0.0</v>
       </c>
       <c r="L17" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M17" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N17" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O17" s="0" t="n">
-        <v>652.5</v>
+        <v>433.5</v>
       </c>
       <c r="P17" s="0" t="n">
-        <v>229.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q17" s="0" t="n">
-        <v>21618.5</v>
+        <v>12185.0</v>
       </c>
       <c r="R17" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="S17" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="T17" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="U17" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="V17" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W17" s="0"/>
@@ -1914,21 +1914,21 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:20</t>
+          <t>2026/05/13 03:36:03</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:22</t>
+          <t>2026/05/13 03:36:05</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>822738944267014664192</t>
+          <t>822743384884528578560</t>
         </is>
       </c>
       <c r="D18" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -1947,12 +1947,12 @@
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t>6156</t>
+          <t>7758</t>
         </is>
       </c>
       <c r="J18" s="0" t="n">
@@ -1962,41 +1962,41 @@
         <v>0.0</v>
       </c>
       <c r="L18" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M18" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N18" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O18" s="0" t="n">
-        <v>652.5</v>
+        <v>369.75</v>
       </c>
       <c r="P18" s="0" t="n">
-        <v>229.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q18" s="0" t="n">
-        <v>21618.5</v>
+        <v>12248.75</v>
       </c>
       <c r="R18" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="S18" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="T18" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="U18" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas, Denisse Olivo</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="V18" s="0" t="inlineStr">
@@ -2019,25 +2019,25 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>2026/05/06 23:07:12</t>
+          <t>2026/05/12 21:17:39</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:05:58</t>
+          <t>2026/05/12 21:17:41</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>822738900913572839424</t>
+          <t>822743194435830431744</t>
         </is>
       </c>
       <c r="D19" s="0" t="n">
-        <v>20500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Refunded</t>
+          <t>Successful</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
@@ -2047,62 +2047,66 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
         <is>
-          <t>transferencia</t>
-        </is>
-      </c>
-      <c r="I19" s="0"/>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I19" s="0" t="inlineStr">
+        <is>
+          <t>9925</t>
+        </is>
+      </c>
       <c r="J19" s="0" t="n">
-        <v>20500.0</v>
+        <v>0.0</v>
       </c>
       <c r="K19" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L19" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M19" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N19" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O19" s="0" t="n">
-        <v>0.0</v>
+        <v>652.5</v>
       </c>
       <c r="P19" s="0" t="n">
-        <v>0.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q19" s="0" t="n">
-        <v>0.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R19" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S19" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T19" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U19" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V19" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W19" s="0"/>
@@ -2120,21 +2124,21 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:40</t>
+          <t>2026/05/12 19:10:30</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:42</t>
+          <t>2026/05/12 19:11:16</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>822735991480689651712</t>
+          <t>822743130440389902336</t>
         </is>
       </c>
       <c r="D20" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
@@ -2153,12 +2157,12 @@
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>2003</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J20" s="0" t="n">
@@ -2168,46 +2172,46 @@
         <v>0.0</v>
       </c>
       <c r="L20" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M20" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N20" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O20" s="0" t="n">
-        <v>1530.0</v>
+        <v>652.5</v>
       </c>
       <c r="P20" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q20" s="0" t="n">
-        <v>43016.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R20" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S20" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T20" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U20" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V20" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W20" s="0"/>
@@ -2225,21 +2229,21 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:35</t>
+          <t>2026/05/12 18:19:51</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:36</t>
+          <t>2026/05/12 18:19:53</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>822733043006520176640</t>
+          <t>822743104942704197632</t>
         </is>
       </c>
       <c r="D21" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
@@ -2258,12 +2262,12 @@
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t>5558</t>
+          <t>1709</t>
         </is>
       </c>
       <c r="J21" s="0" t="n">
@@ -2273,41 +2277,41 @@
         <v>0.0</v>
       </c>
       <c r="L21" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M21" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N21" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O21" s="0" t="n">
-        <v>652.5</v>
+        <v>1305.0</v>
       </c>
       <c r="P21" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q21" s="0" t="n">
-        <v>21618.5</v>
+        <v>43241.0</v>
       </c>
       <c r="R21" s="0" t="inlineStr">
         <is>
-          <t>IGNACIO PORTILLA</t>
+          <t>RAFAEL BELTRAN LOPEZ</t>
         </is>
       </c>
       <c r="S21" s="0" t="inlineStr">
         <is>
-          <t>mx.portilla@gmail.com</t>
+          <t>rbeltran1976@hotmail.com</t>
         </is>
       </c>
       <c r="T21" s="0" t="inlineStr">
         <is>
-          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
+          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
         </is>
       </c>
       <c r="U21" s="0" t="inlineStr">
         <is>
-          <t>VALERIA PORTILLA, Natalia Portilla</t>
+          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
         </is>
       </c>
       <c r="V21" s="0" t="inlineStr">
@@ -2330,21 +2334,21 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:10:30</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:11:05</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>822732983572553019392</t>
+          <t>822742523051869483008</t>
         </is>
       </c>
       <c r="D22" s="0" t="n">
-        <v>18000.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -2358,19 +2362,15 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I22" s="0" t="inlineStr">
-        <is>
-          <t>4583</t>
-        </is>
-      </c>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I22" s="0"/>
       <c r="J22" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -2378,41 +2378,41 @@
         <v>0.0</v>
       </c>
       <c r="L22" s="0" t="n">
-        <v>18000.0</v>
+        <v>0.0</v>
       </c>
       <c r="M22" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N22" s="0" t="n">
-        <v>18000.0</v>
+        <v>0.0</v>
       </c>
       <c r="O22" s="0" t="n">
-        <v>522.0</v>
+        <v>0.0</v>
       </c>
       <c r="P22" s="0" t="n">
-        <v>184.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q22" s="0" t="n">
-        <v>17294.0</v>
+        <v>0.0</v>
       </c>
       <c r="R22" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S22" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T22" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U22" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V22" s="0" t="inlineStr">
@@ -2435,21 +2435,21 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:49</t>
+          <t>2026/05/11 22:22:09</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:51</t>
+          <t>2026/05/11 22:22:12</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>822728072370714607616</t>
+          <t>822742502121738878976</t>
         </is>
       </c>
       <c r="D23" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -2468,12 +2468,12 @@
       </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t>2071</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="J23" s="0" t="n">
@@ -2483,46 +2483,46 @@
         <v>0.0</v>
       </c>
       <c r="L23" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M23" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N23" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O23" s="0" t="n">
-        <v>285.16</v>
+        <v>652.5</v>
       </c>
       <c r="P23" s="0" t="n">
-        <v>102.33</v>
+        <v>229.0</v>
       </c>
       <c r="Q23" s="0" t="n">
-        <v>9445.51</v>
+        <v>21618.5</v>
       </c>
       <c r="R23" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>Macarena Olavarri</t>
         </is>
       </c>
       <c r="S23" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>macaolavarri@gmail.com</t>
         </is>
       </c>
       <c r="T23" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
         </is>
       </c>
       <c r="U23" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>Macarena Olavarri, Isabel Fernández</t>
         </is>
       </c>
       <c r="V23" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W23" s="0"/>
@@ -2540,21 +2540,21 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:44</t>
+          <t>2026/05/08 23:10:41</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:46</t>
+          <t>2026/05/08 23:10:43</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>822728021498622136320</t>
+          <t>822740352219193810944</t>
         </is>
       </c>
       <c r="D24" s="0" t="n">
-        <v>22500.0</v>
+        <v>81000.0</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="J24" s="0" t="n">
@@ -2588,46 +2588,46 @@
         <v>0.0</v>
       </c>
       <c r="L24" s="0" t="n">
-        <v>22500.0</v>
+        <v>81000.0</v>
       </c>
       <c r="M24" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N24" s="0" t="n">
-        <v>22500.0</v>
+        <v>81000.0</v>
       </c>
       <c r="O24" s="0" t="n">
-        <v>652.5</v>
+        <v>2754.0</v>
       </c>
       <c r="P24" s="0" t="n">
-        <v>229.0</v>
+        <v>814.0</v>
       </c>
       <c r="Q24" s="0" t="n">
-        <v>21618.5</v>
+        <v>77432.0</v>
       </c>
       <c r="R24" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>Judith Escobar Torres</t>
         </is>
       </c>
       <c r="S24" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>judith.escobar@gmail.com</t>
         </is>
       </c>
       <c r="T24" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
         </is>
       </c>
       <c r="U24" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
         </is>
       </c>
       <c r="V24" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W24" s="0"/>
@@ -2645,21 +2645,21 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:01</t>
+          <t>2026/05/08 18:45:11</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:03</t>
+          <t>2026/05/08 18:45:12</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>822727454901268389888</t>
+          <t>822740218587619794944</t>
         </is>
       </c>
       <c r="D25" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -2683,7 +2683,7 @@
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>6624</t>
         </is>
       </c>
       <c r="J25" s="0" t="n">
@@ -2693,46 +2693,46 @@
         <v>0.0</v>
       </c>
       <c r="L25" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M25" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N25" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O25" s="0" t="n">
-        <v>652.5</v>
+        <v>739.5</v>
       </c>
       <c r="P25" s="0" t="n">
-        <v>229.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q25" s="0" t="n">
-        <v>21618.5</v>
+        <v>24501.5</v>
       </c>
       <c r="R25" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>MELB PEREZ SALDANA</t>
         </is>
       </c>
       <c r="S25" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="T25" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="U25" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>MELBA ASTRID PEREZ SALDAÑA</t>
         </is>
       </c>
       <c r="V25" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W25" s="0"/>
@@ -2750,17 +2750,17 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:12</t>
+          <t>2026/05/08 18:14:10</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:13</t>
+          <t>2026/05/08 18:14:12</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>822727364900010598400</t>
+          <t>822740202977192058880</t>
         </is>
       </c>
       <c r="D26" s="0" t="n">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t>7852</t>
+          <t>9925</t>
         </is>
       </c>
       <c r="J26" s="0" t="n">
@@ -2817,27 +2817,27 @@
       </c>
       <c r="R26" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S26" s="0" t="inlineStr">
         <is>
-          <t>ricardocb23@gmail.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T26" s="0" t="inlineStr">
         <is>
-          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U26" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V26" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W26" s="0"/>
@@ -2855,21 +2855,21 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:19</t>
+          <t>2026/05/07 00:33:20</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:21</t>
+          <t>2026/05/07 00:33:22</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>822726495229304659968</t>
+          <t>822738944267014664192</t>
         </is>
       </c>
       <c r="D27" s="0" t="n">
-        <v>14750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -2883,17 +2883,17 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I27" s="0" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>6156</t>
         </is>
       </c>
       <c r="J27" s="0" t="n">
@@ -2903,46 +2903,46 @@
         <v>0.0</v>
       </c>
       <c r="L27" s="0" t="n">
-        <v>14750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M27" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N27" s="0" t="n">
-        <v>14750.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O27" s="0" t="n">
-        <v>427.75</v>
+        <v>652.5</v>
       </c>
       <c r="P27" s="0" t="n">
-        <v>151.5</v>
+        <v>229.0</v>
       </c>
       <c r="Q27" s="0" t="n">
-        <v>14170.75</v>
+        <v>21618.5</v>
       </c>
       <c r="R27" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>Alejandra Serpas</t>
         </is>
       </c>
       <c r="S27" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="T27" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="U27" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>Alejandra Serpas, Denisse Olivo</t>
         </is>
       </c>
       <c r="V27" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W27" s="0"/>
@@ -2960,25 +2960,25 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:21</t>
+          <t>2026/05/06 23:07:12</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:23</t>
+          <t>2026/05/11 23:05:58</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>822725726179188305920</t>
+          <t>822738900913572839424</t>
         </is>
       </c>
       <c r="D28" s="0" t="n">
-        <v>25500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Successful</t>
+          <t>Refunded</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
@@ -2988,66 +2988,62 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I28" s="0" t="inlineStr">
-        <is>
-          <t>9962</t>
-        </is>
-      </c>
+          <t>transferencia</t>
+        </is>
+      </c>
+      <c r="I28" s="0"/>
       <c r="J28" s="0" t="n">
-        <v>0.0</v>
+        <v>20500.0</v>
       </c>
       <c r="K28" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L28" s="0" t="n">
-        <v>25500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M28" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N28" s="0" t="n">
-        <v>25500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O28" s="0" t="n">
-        <v>739.5</v>
+        <v>0.0</v>
       </c>
       <c r="P28" s="0" t="n">
-        <v>259.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q28" s="0" t="n">
-        <v>24501.5</v>
+        <v>0.0</v>
       </c>
       <c r="R28" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon Mendez</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S28" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T28" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U28" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V28" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W28" s="0"/>
@@ -3065,21 +3061,21 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:42</t>
+          <t>2026/05/02 22:46:40</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:44</t>
+          <t>2026/05/02 22:46:42</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>822724934643911520256</t>
+          <t>822735991480689651712</t>
         </is>
       </c>
       <c r="D29" s="0" t="n">
-        <v>70500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -3103,7 +3099,7 @@
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="J29" s="0" t="n">
@@ -3113,46 +3109,46 @@
         <v>0.0</v>
       </c>
       <c r="L29" s="0" t="n">
-        <v>70500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M29" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N29" s="0" t="n">
-        <v>70500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O29" s="0" t="n">
-        <v>2397.0</v>
+        <v>1530.0</v>
       </c>
       <c r="P29" s="0" t="n">
-        <v>709.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q29" s="0" t="n">
-        <v>67394.0</v>
+        <v>43016.0</v>
       </c>
       <c r="R29" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos</t>
+          <t>ALEJANDRO CANALES MORALES</t>
         </is>
       </c>
       <c r="S29" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com</t>
+          <t>alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="T29" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
+          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="U29" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
+          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
         </is>
       </c>
       <c r="V29" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W29" s="0"/>
@@ -3170,21 +3166,21 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:28</t>
+          <t>2026/04/28 21:08:35</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:30</t>
+          <t>2026/04/28 21:08:36</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>822722199504844500992</t>
+          <t>822733043006520176640</t>
         </is>
       </c>
       <c r="D30" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -3203,12 +3199,12 @@
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t>4291</t>
+          <t>5558</t>
         </is>
       </c>
       <c r="J30" s="0" t="n">
@@ -3218,41 +3214,41 @@
         <v>0.0</v>
       </c>
       <c r="L30" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M30" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N30" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O30" s="0" t="n">
-        <v>1305.0</v>
+        <v>652.5</v>
       </c>
       <c r="P30" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q30" s="0" t="n">
-        <v>43241.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R30" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza</t>
+          <t>IGNACIO PORTILLA</t>
         </is>
       </c>
       <c r="S30" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com</t>
+          <t>mx.portilla@gmail.com</t>
         </is>
       </c>
       <c r="T30" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
+          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
         </is>
       </c>
       <c r="U30" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
+          <t>VALERIA PORTILLA, Natalia Portilla</t>
         </is>
       </c>
       <c r="V30" s="0" t="inlineStr">
@@ -3275,21 +3271,21 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:45</t>
+          <t>2026/04/28 19:10:30</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:47</t>
+          <t>2026/04/28 19:11:05</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>822722120121735725056</t>
+          <t>822732983572553019392</t>
         </is>
       </c>
       <c r="D31" s="0" t="n">
-        <v>45000.0</v>
+        <v>18000.0</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
@@ -3308,12 +3304,12 @@
       </c>
       <c r="H31" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I31" s="0" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J31" s="0" t="n">
@@ -3323,46 +3319,46 @@
         <v>0.0</v>
       </c>
       <c r="L31" s="0" t="n">
-        <v>45000.0</v>
+        <v>18000.0</v>
       </c>
       <c r="M31" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N31" s="0" t="n">
-        <v>45000.0</v>
+        <v>18000.0</v>
       </c>
       <c r="O31" s="0" t="n">
-        <v>1530.0</v>
+        <v>522.0</v>
       </c>
       <c r="P31" s="0" t="n">
-        <v>454.0</v>
+        <v>184.0</v>
       </c>
       <c r="Q31" s="0" t="n">
-        <v>43016.0</v>
+        <v>17294.0</v>
       </c>
       <c r="R31" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S31" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T31" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U31" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac, Gabriela Vazquez</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V31" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W31" s="0"/>
@@ -3380,21 +3376,21 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:14</t>
+          <t>2026/04/22 00:32:49</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:16</t>
+          <t>2026/04/22 00:32:51</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>822718782367677300736</t>
+          <t>822728072370714607616</t>
         </is>
       </c>
       <c r="D32" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
@@ -3408,7 +3404,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -3418,7 +3414,7 @@
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t>7348</t>
+          <t>2071</t>
         </is>
       </c>
       <c r="J32" s="0" t="n">
@@ -3428,46 +3424,46 @@
         <v>0.0</v>
       </c>
       <c r="L32" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M32" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N32" s="0" t="n">
-        <v>45000.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O32" s="0" t="n">
-        <v>1305.0</v>
+        <v>285.16</v>
       </c>
       <c r="P32" s="0" t="n">
-        <v>454.0</v>
+        <v>102.33</v>
       </c>
       <c r="Q32" s="0" t="n">
-        <v>43241.0</v>
+        <v>9445.51</v>
       </c>
       <c r="R32" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera Lima</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="S32" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="T32" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="U32" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="V32" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W32" s="0"/>
@@ -3485,21 +3481,21 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:52</t>
+          <t>2026/04/21 22:51:44</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:54</t>
+          <t>2026/04/21 22:51:46</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>822717931075648110592</t>
+          <t>822728021498622136320</t>
         </is>
       </c>
       <c r="D33" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
@@ -3518,12 +3514,12 @@
       </c>
       <c r="H33" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J33" s="0" t="n">
@@ -3533,46 +3529,46 @@
         <v>0.0</v>
       </c>
       <c r="L33" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M33" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N33" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O33" s="0" t="n">
-        <v>1530.0</v>
+        <v>652.5</v>
       </c>
       <c r="P33" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q33" s="0" t="n">
-        <v>43016.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R33" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S33" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T33" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U33" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V33" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W33" s="0"/>
@@ -3590,21 +3586,21 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:06</t>
+          <t>2026/04/21 04:06:01</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:09</t>
+          <t>2026/04/21 04:06:03</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>822717887408069685248</t>
+          <t>822727454901268389888</t>
         </is>
       </c>
       <c r="D34" s="0" t="n">
-        <v>31500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
@@ -3623,12 +3619,12 @@
       </c>
       <c r="H34" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I34" s="0" t="inlineStr">
         <is>
-          <t>4006</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J34" s="0" t="n">
@@ -3638,46 +3634,46 @@
         <v>0.0</v>
       </c>
       <c r="L34" s="0" t="n">
-        <v>31500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M34" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N34" s="0" t="n">
-        <v>31500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O34" s="0" t="n">
-        <v>1071.0</v>
+        <v>652.5</v>
       </c>
       <c r="P34" s="0" t="n">
-        <v>319.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q34" s="0" t="n">
-        <v>30110.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R34" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S34" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T34" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U34" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago, Michelle Ralph</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V34" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W34" s="0"/>
@@ -3695,21 +3691,21 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:57</t>
+          <t>2026/04/21 01:07:12</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:59</t>
+          <t>2026/04/21 01:07:13</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>822717804781623066624</t>
+          <t>822727364900010598400</t>
         </is>
       </c>
       <c r="D35" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
@@ -3733,7 +3729,7 @@
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t>3513</t>
+          <t>7852</t>
         </is>
       </c>
       <c r="J35" s="0" t="n">
@@ -3743,46 +3739,46 @@
         <v>0.0</v>
       </c>
       <c r="L35" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M35" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N35" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O35" s="0" t="n">
-        <v>739.5</v>
+        <v>652.5</v>
       </c>
       <c r="P35" s="0" t="n">
-        <v>259.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q35" s="0" t="n">
-        <v>24501.5</v>
+        <v>21618.5</v>
       </c>
       <c r="R35" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>RICARDO CAMACHO BOFILL</t>
         </is>
       </c>
       <c r="S35" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>ricardocb23@gmail.com</t>
         </is>
       </c>
       <c r="T35" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
         </is>
       </c>
       <c r="U35" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
         </is>
       </c>
       <c r="V35" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W35" s="0"/>
@@ -3800,21 +3796,21 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:51</t>
+          <t>2026/04/19 20:19:19</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:53</t>
+          <t>2026/04/19 20:19:21</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>822717250585584762880</t>
+          <t>822726495229304659968</t>
         </is>
       </c>
       <c r="D36" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
@@ -3828,7 +3824,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>apple_pay</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -3838,7 +3834,7 @@
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="J36" s="0" t="n">
@@ -3848,46 +3844,46 @@
         <v>0.0</v>
       </c>
       <c r="L36" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="M36" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N36" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="O36" s="0" t="n">
-        <v>1530.0</v>
+        <v>427.75</v>
       </c>
       <c r="P36" s="0" t="n">
-        <v>454.0</v>
+        <v>151.5</v>
       </c>
       <c r="Q36" s="0" t="n">
-        <v>43016.0</v>
+        <v>14170.75</v>
       </c>
       <c r="R36" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="S36" s="0" t="inlineStr">
         <is>
-          <t>sofiacarrioncobian@hotmail.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="T36" s="0" t="inlineStr">
         <is>
-          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="U36" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion, Ana María Carrion</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="V36" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W36" s="0"/>
@@ -3897,6 +3893,951 @@
         </is>
       </c>
       <c r="Y36" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/18 18:51:21</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/18 18:51:23</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>822725726179188305920</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H37" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I37" s="0" t="inlineStr">
+        <is>
+          <t>9962</t>
+        </is>
+      </c>
+      <c r="J37" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K37" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L37" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="M37" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N37" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="O37" s="0" t="n">
+        <v>739.5</v>
+      </c>
+      <c r="P37" s="0" t="n">
+        <v>259.0</v>
+      </c>
+      <c r="Q37" s="0" t="n">
+        <v>24501.5</v>
+      </c>
+      <c r="R37" s="0" t="inlineStr">
+        <is>
+          <t>Jonatan Oregon Mendez</t>
+        </is>
+      </c>
+      <c r="S37" s="0" t="inlineStr">
+        <is>
+          <t>johnoregon@live.com</t>
+        </is>
+      </c>
+      <c r="T37" s="0" t="inlineStr">
+        <is>
+          <t>johnoregon@live.com</t>
+        </is>
+      </c>
+      <c r="U37" s="0" t="inlineStr">
+        <is>
+          <t>Jonatan Oregon</t>
+        </is>
+      </c>
+      <c r="V37" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W37" s="0"/>
+      <c r="X37" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y37" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/17 16:38:42</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/17 16:38:44</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>822724934643911520256</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="n">
+        <v>70500.0</v>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H38" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I38" s="0" t="inlineStr">
+        <is>
+          <t>1008</t>
+        </is>
+      </c>
+      <c r="J38" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K38" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L38" s="0" t="n">
+        <v>70500.0</v>
+      </c>
+      <c r="M38" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N38" s="0" t="n">
+        <v>70500.0</v>
+      </c>
+      <c r="O38" s="0" t="n">
+        <v>2397.0</v>
+      </c>
+      <c r="P38" s="0" t="n">
+        <v>709.0</v>
+      </c>
+      <c r="Q38" s="0" t="n">
+        <v>67394.0</v>
+      </c>
+      <c r="R38" s="0" t="inlineStr">
+        <is>
+          <t>Marcela Alvarez Campos</t>
+        </is>
+      </c>
+      <c r="S38" s="0" t="inlineStr">
+        <is>
+          <t>marcela.ac@me.com</t>
+        </is>
+      </c>
+      <c r="T38" s="0" t="inlineStr">
+        <is>
+          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
+        </is>
+      </c>
+      <c r="U38" s="0" t="inlineStr">
+        <is>
+          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
+        </is>
+      </c>
+      <c r="V38" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+        </is>
+      </c>
+      <c r="W38" s="0"/>
+      <c r="X38" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y38" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 22:04:28</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 22:04:30</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>822722199504844500992</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H39" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I39" s="0" t="inlineStr">
+        <is>
+          <t>4291</t>
+        </is>
+      </c>
+      <c r="J39" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K39" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L39" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M39" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N39" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O39" s="0" t="n">
+        <v>1305.0</v>
+      </c>
+      <c r="P39" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q39" s="0" t="n">
+        <v>43241.0</v>
+      </c>
+      <c r="R39" s="0" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="S39" s="0" t="inlineStr">
+        <is>
+          <t>mendoza.carlos.a@gmail.com</t>
+        </is>
+      </c>
+      <c r="T39" s="0" t="inlineStr">
+        <is>
+          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
+        </is>
+      </c>
+      <c r="U39" s="0" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
+        </is>
+      </c>
+      <c r="V39" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+        </is>
+      </c>
+      <c r="W39" s="0"/>
+      <c r="X39" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y39" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 19:26:45</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/13 19:26:47</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>822722120121735725056</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F40" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H40" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I40" s="0" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+      <c r="J40" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K40" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L40" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M40" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N40" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O40" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P40" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q40" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R40" s="0" t="inlineStr">
+        <is>
+          <t>Ana paula Isaac</t>
+        </is>
+      </c>
+      <c r="S40" s="0" t="inlineStr">
+        <is>
+          <t>anapauisaac@gmail.com</t>
+        </is>
+      </c>
+      <c r="T40" s="0" t="inlineStr">
+        <is>
+          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
+        </is>
+      </c>
+      <c r="U40" s="0" t="inlineStr">
+        <is>
+          <t>Ana paula Isaac, Gabriela Vazquez</t>
+        </is>
+      </c>
+      <c r="V40" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W40" s="0"/>
+      <c r="X40" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y40" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/09 04:55:14</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/09 04:55:16</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>822718782367677300736</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>apple_pay</t>
+        </is>
+      </c>
+      <c r="H41" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I41" s="0" t="inlineStr">
+        <is>
+          <t>7348</t>
+        </is>
+      </c>
+      <c r="J41" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K41" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L41" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M41" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N41" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O41" s="0" t="n">
+        <v>1305.0</v>
+      </c>
+      <c r="P41" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q41" s="0" t="n">
+        <v>43241.0</v>
+      </c>
+      <c r="R41" s="0" t="inlineStr">
+        <is>
+          <t>Francisco Javier Vera Lima</t>
+        </is>
+      </c>
+      <c r="S41" s="0" t="inlineStr">
+        <is>
+          <t>fjvera@vmodal.mx</t>
+        </is>
+      </c>
+      <c r="T41" s="0" t="inlineStr">
+        <is>
+          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+        </is>
+      </c>
+      <c r="U41" s="0" t="inlineStr">
+        <is>
+          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
+        </is>
+      </c>
+      <c r="V41" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W41" s="0"/>
+      <c r="X41" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y41" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:52</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:54</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>822717931075648110592</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H42" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I42" s="0" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="J42" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K42" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L42" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M42" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N42" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O42" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P42" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q42" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R42" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+        </is>
+      </c>
+      <c r="S42" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T42" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+        </is>
+      </c>
+      <c r="U42" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+        </is>
+      </c>
+      <c r="V42" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W42" s="0"/>
+      <c r="X42" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y42" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:06</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:09</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>822717887408069685248</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H43" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I43" s="0" t="inlineStr">
+        <is>
+          <t>4006</t>
+        </is>
+      </c>
+      <c r="J43" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K43" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L43" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="M43" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N43" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="O43" s="0" t="n">
+        <v>1071.0</v>
+      </c>
+      <c r="P43" s="0" t="n">
+        <v>319.0</v>
+      </c>
+      <c r="Q43" s="0" t="n">
+        <v>30110.0</v>
+      </c>
+      <c r="R43" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago</t>
+        </is>
+      </c>
+      <c r="S43" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com</t>
+        </is>
+      </c>
+      <c r="T43" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+        </is>
+      </c>
+      <c r="U43" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago, Michelle Ralph</t>
+        </is>
+      </c>
+      <c r="V43" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W43" s="0"/>
+      <c r="X43" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y43" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:57</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:59</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>822717804781623066624</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H44" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I44" s="0" t="inlineStr">
+        <is>
+          <t>3513</t>
+        </is>
+      </c>
+      <c r="J44" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K44" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L44" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="M44" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N44" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="O44" s="0" t="n">
+        <v>739.5</v>
+      </c>
+      <c r="P44" s="0" t="n">
+        <v>259.0</v>
+      </c>
+      <c r="Q44" s="0" t="n">
+        <v>24501.5</v>
+      </c>
+      <c r="R44" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="S44" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="T44" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="U44" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="V44" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W44" s="0"/>
+      <c r="X44" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y44" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:51</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:53</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>822717250585584762880</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F45" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G45" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H45" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I45" s="0" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="J45" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K45" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L45" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M45" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N45" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O45" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P45" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q45" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R45" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion</t>
+        </is>
+      </c>
+      <c r="S45" s="0" t="inlineStr">
+        <is>
+          <t>sofiacarrioncobian@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T45" s="0" t="inlineStr">
+        <is>
+          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+        </is>
+      </c>
+      <c r="U45" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion, Ana María Carrion</t>
+        </is>
+      </c>
+      <c r="V45" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W45" s="0"/>
+      <c r="X45" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y45" s="0" t="inlineStr">
         <is>
           <t>daniel@akampa.mx</t>
         </is>

</xml_diff>

<commit_message>
📥 WeTravel: Reporting_Payments_WeTravel-539682-1779724797.xlsx (2026-05-25)
</commit_message>
<xml_diff>
--- a/reportes/Reporting_Payments_WeTravel.xlsx
+++ b/reportes/Reporting_Payments_WeTravel.xlsx
@@ -82,7 +82,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y45"/>
+  <dimension ref="A1:Y50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="29.4" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -242,21 +242,21 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/21 17:22:39</t>
+          <t>2026/05/23 18:48:45</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>2026/05/21 17:22:42</t>
+          <t>2026/05/23 18:48:49</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>822749599136998244352</t>
+          <t>822751092026383556608</t>
         </is>
       </c>
       <c r="D2" s="0" t="n">
-        <v>9833.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
@@ -280,7 +280,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>4931</t>
         </is>
       </c>
       <c r="J2" s="0" t="n">
@@ -290,46 +290,46 @@
         <v>0.0</v>
       </c>
       <c r="L2" s="0" t="n">
-        <v>9833.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M2" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N2" s="0" t="n">
-        <v>9833.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O2" s="0" t="n">
-        <v>285.16</v>
+        <v>369.75</v>
       </c>
       <c r="P2" s="0" t="n">
-        <v>102.33</v>
+        <v>131.5</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <v>9445.51</v>
+        <v>12248.75</v>
       </c>
       <c r="R2" s="0" t="inlineStr">
         <is>
-          <t>Leah Pages</t>
+          <t>Nayvy Juarez</t>
         </is>
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t>pagesnava.leah@gmail.com</t>
+          <t>nayvyj@gmail.com</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t>Pagesnava.leah@gmail.com</t>
+          <t>nayvyj@gmail.com</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
         <is>
-          <t>Leah Pages</t>
+          <t>Nayvy Juarez Pérez</t>
         </is>
       </c>
       <c r="V2" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W2" s="0"/>
@@ -347,21 +347,21 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/20 23:14:50</t>
+          <t>2026/05/23 00:23:31</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>2026/05/20 23:14:51</t>
+          <t>2026/05/23 00:23:34</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>822749051616429613056</t>
+          <t>822750535743452508160</t>
         </is>
       </c>
       <c r="D3" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
@@ -380,12 +380,12 @@
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="J3" s="0" t="n">
@@ -395,46 +395,46 @@
         <v>0.0</v>
       </c>
       <c r="L3" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M3" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N3" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O3" s="0" t="n">
-        <v>867.0</v>
+        <v>652.5</v>
       </c>
       <c r="P3" s="0" t="n">
-        <v>259.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q3" s="0" t="n">
-        <v>24374.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R3" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Aviles</t>
+          <t>Macarena Olavarri</t>
         </is>
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t>avilo26@hotmail.com</t>
+          <t>macaolavarri@gmail.com</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t>avilo26@hotmail.com</t>
+          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Aviles</t>
+          <t>Macarena Olavarri, Isabel Fernández</t>
         </is>
       </c>
       <c r="V3" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W3" s="0"/>
@@ -452,21 +452,21 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/20 17:53:15</t>
+          <t>2026/05/22 23:07:26</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>2026/05/20 17:53:18</t>
+          <t>2026/05/22 23:07:28</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>822748889761073610752</t>
+          <t>822750497446034432000</t>
         </is>
       </c>
       <c r="D4" s="0" t="n">
-        <v>9833.0</v>
+        <v>35250.0</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
@@ -485,12 +485,12 @@
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>3493</t>
+          <t>6953</t>
         </is>
       </c>
       <c r="J4" s="0" t="n">
@@ -500,46 +500,46 @@
         <v>0.0</v>
       </c>
       <c r="L4" s="0" t="n">
-        <v>9833.0</v>
+        <v>35250.0</v>
       </c>
       <c r="M4" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N4" s="0" t="n">
-        <v>9833.0</v>
+        <v>35250.0</v>
       </c>
       <c r="O4" s="0" t="n">
-        <v>285.16</v>
+        <v>1022.25</v>
       </c>
       <c r="P4" s="0" t="n">
-        <v>102.33</v>
+        <v>356.5</v>
       </c>
       <c r="Q4" s="0" t="n">
-        <v>9445.51</v>
+        <v>33871.25</v>
       </c>
       <c r="R4" s="0" t="inlineStr">
         <is>
-          <t>Liliana Osuna Domínguez</t>
+          <t>Arturs Aleksandrovics</t>
         </is>
       </c>
       <c r="S4" s="0" t="inlineStr">
         <is>
-          <t>lilianaeod@gmail.com</t>
+          <t>aa@novacard.mx</t>
         </is>
       </c>
       <c r="T4" s="0" t="inlineStr">
         <is>
-          <t>Lilianaeod@gmail.com</t>
+          <t>Aa@novacard.mx, Aleksandrowicz@gmx.net, Aleksandrovics@gmx.net</t>
         </is>
       </c>
       <c r="U4" s="0" t="inlineStr">
         <is>
-          <t>Liliana Osuna Domínguez</t>
+          <t>Arturs Aleksandrovics, Maksimilians Aleksandrovics, Markus Aleksandrovics</t>
         </is>
       </c>
       <c r="V4" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W4" s="0"/>
@@ -557,17 +557,17 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/20 17:09:53</t>
+          <t>2026/05/22 22:57:55</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>2026/05/20 17:09:55</t>
+          <t>2026/05/23 10:58:03</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>822748867929998106624</t>
+          <t>822750492657833766912</t>
         </is>
       </c>
       <c r="D5" s="0" t="n">
@@ -575,7 +575,7 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Successful</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
@@ -585,19 +585,15 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>spei</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
-        </is>
-      </c>
-      <c r="I5" s="0" t="inlineStr">
-        <is>
-          <t>8841</t>
-        </is>
-      </c>
+          <t>SPEI</t>
+        </is>
+      </c>
+      <c r="I5" s="0"/>
       <c r="J5" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -614,37 +610,37 @@
         <v>12750.0</v>
       </c>
       <c r="O5" s="0" t="n">
-        <v>369.75</v>
+        <v>0.0</v>
       </c>
       <c r="P5" s="0" t="n">
-        <v>131.5</v>
+        <v>0.0</v>
       </c>
       <c r="Q5" s="0" t="n">
-        <v>12248.75</v>
+        <v>0.0</v>
       </c>
       <c r="R5" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>Valeria Gonzalez</t>
         </is>
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>valeriagonzalez@hotmail.com</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>valeriagonzalez@hotmail.com</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>Valeria Gonzalez</t>
         </is>
       </c>
       <c r="V5" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W5" s="0"/>
@@ -662,21 +658,21 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:10:35</t>
+          <t>2026/05/22 20:55:21</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:11:23</t>
+          <t>2026/05/22 20:55:24</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>822747479128876781568</t>
+          <t>822750430970527117312</t>
         </is>
       </c>
       <c r="D6" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
@@ -690,17 +686,17 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>apple_pay</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t>3097</t>
+          <t>7348</t>
         </is>
       </c>
       <c r="J6" s="0" t="n">
@@ -710,41 +706,41 @@
         <v>0.0</v>
       </c>
       <c r="L6" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M6" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N6" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O6" s="0" t="n">
-        <v>652.5</v>
+        <v>739.5</v>
       </c>
       <c r="P6" s="0" t="n">
-        <v>229.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q6" s="0" t="n">
-        <v>21618.5</v>
+        <v>24501.5</v>
       </c>
       <c r="R6" s="0" t="inlineStr">
         <is>
-          <t>Marihel Arias</t>
+          <t>Francisco Javier Vera Lima</t>
         </is>
       </c>
       <c r="S6" s="0" t="inlineStr">
         <is>
-          <t>marihel_arias@hotmail.com</t>
+          <t>fjvera@vmodal.mx</t>
         </is>
       </c>
       <c r="T6" s="0" t="inlineStr">
         <is>
-          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
+          <t>fjvera@vmodal.mx, fjvera@vmodal.mx, fjvera@vmodal.mx</t>
         </is>
       </c>
       <c r="U6" s="0" t="inlineStr">
         <is>
-          <t>Marihel Arias, Alondra Arias</t>
+          <t>Francisco Javier Vera, Carlos Vera, Gabriela Vera</t>
         </is>
       </c>
       <c r="V6" s="0" t="inlineStr">
@@ -767,21 +763,21 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:10:33</t>
+          <t>2026/05/21 17:22:39</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:11:20</t>
+          <t>2026/05/21 17:22:42</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>822747479118273585152</t>
+          <t>822749599136998244352</t>
         </is>
       </c>
       <c r="D7" s="0" t="n">
-        <v>12750.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
@@ -800,12 +796,12 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>1009</t>
+          <t>2500</t>
         </is>
       </c>
       <c r="J7" s="0" t="n">
@@ -815,46 +811,46 @@
         <v>0.0</v>
       </c>
       <c r="L7" s="0" t="n">
-        <v>12750.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M7" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N7" s="0" t="n">
-        <v>12750.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>433.5</v>
+        <v>285.16</v>
       </c>
       <c r="P7" s="0" t="n">
-        <v>131.5</v>
+        <v>102.33</v>
       </c>
       <c r="Q7" s="0" t="n">
-        <v>12185.0</v>
+        <v>9445.51</v>
       </c>
       <c r="R7" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Leah Pages</t>
         </is>
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>pagesnava.leah@gmail.com</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>Pagesnava.leah@gmail.com</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>Leah Pages</t>
         </is>
       </c>
       <c r="V7" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W7" s="0"/>
@@ -872,21 +868,21 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:10:32</t>
+          <t>2026/05/20 23:14:50</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:11:18</t>
+          <t>2026/05/20 23:14:51</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>822747479109650092032</t>
+          <t>822749051616429613056</t>
         </is>
       </c>
       <c r="D8" s="0" t="n">
-        <v>18000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
@@ -905,12 +901,12 @@
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>6156</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J8" s="0" t="n">
@@ -920,46 +916,46 @@
         <v>0.0</v>
       </c>
       <c r="L8" s="0" t="n">
-        <v>18000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M8" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N8" s="0" t="n">
-        <v>18000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O8" s="0" t="n">
-        <v>522.0</v>
+        <v>867.0</v>
       </c>
       <c r="P8" s="0" t="n">
-        <v>184.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q8" s="0" t="n">
-        <v>17294.0</v>
+        <v>24374.0</v>
       </c>
       <c r="R8" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas</t>
+          <t>Rodrigo Aviles</t>
         </is>
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel</t>
+          <t>avilo26@hotmail.com</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
+          <t>avilo26@hotmail.com</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas, Denisse Olivo</t>
+          <t>Rodrigo Aviles</t>
         </is>
       </c>
       <c r="V8" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W8" s="0"/>
@@ -977,21 +973,21 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:10:31</t>
+          <t>2026/05/20 17:53:15</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 19:11:14</t>
+          <t>2026/05/20 17:53:18</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>822747479096832299008</t>
+          <t>822748889761073610752</t>
         </is>
       </c>
       <c r="D9" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
@@ -1010,12 +1006,12 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>5558</t>
+          <t>3493</t>
         </is>
       </c>
       <c r="J9" s="0" t="n">
@@ -1025,46 +1021,46 @@
         <v>0.0</v>
       </c>
       <c r="L9" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M9" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N9" s="0" t="n">
-        <v>22500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O9" s="0" t="n">
-        <v>652.5</v>
+        <v>285.16</v>
       </c>
       <c r="P9" s="0" t="n">
-        <v>229.0</v>
+        <v>102.33</v>
       </c>
       <c r="Q9" s="0" t="n">
-        <v>21618.5</v>
+        <v>9445.51</v>
       </c>
       <c r="R9" s="0" t="inlineStr">
         <is>
-          <t>IGNACIO PORTILLA</t>
+          <t>Liliana Osuna Domínguez</t>
         </is>
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t>mx.portilla@gmail.com</t>
+          <t>lilianaeod@gmail.com</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
+          <t>Lilianaeod@gmail.com</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
         <is>
-          <t>VALERIA PORTILLA, Natalia Portilla</t>
+          <t>Liliana Osuna Domínguez</t>
         </is>
       </c>
       <c r="V9" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W9" s="0"/>
@@ -1082,21 +1078,21 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 16:14:03</t>
+          <t>2026/05/20 17:09:53</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 16:14:03</t>
+          <t>2026/05/20 17:09:55</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>822747390277042835456</t>
+          <t>822748867929998106624</t>
         </is>
       </c>
       <c r="D10" s="0" t="n">
-        <v>20500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
@@ -1110,15 +1106,19 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="I10" s="0"/>
+          <t>mastercard</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>8841</t>
+        </is>
+      </c>
       <c r="J10" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1126,46 +1126,46 @@
         <v>0.0</v>
       </c>
       <c r="L10" s="0" t="n">
-        <v>0.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M10" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N10" s="0" t="n">
-        <v>0.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O10" s="0" t="n">
-        <v>0.0</v>
+        <v>369.75</v>
       </c>
       <c r="P10" s="0" t="n">
-        <v>0.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q10" s="0" t="n">
-        <v>0.0</v>
+        <v>12248.75</v>
       </c>
       <c r="R10" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="V10" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W10" s="0"/>
@@ -1183,17 +1183,17 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 01:01:03</t>
+          <t>2026/05/18 19:10:35</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>2026/05/18 01:01:18</t>
+          <t>2026/05/18 19:11:23</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>822746930752535928832</t>
+          <t>822747479128876781568</t>
         </is>
       </c>
       <c r="D11" s="0" t="n">
@@ -1216,12 +1216,12 @@
       </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>6353</t>
+          <t>3097</t>
         </is>
       </c>
       <c r="J11" s="0" t="n">
@@ -1240,37 +1240,37 @@
         <v>22500.0</v>
       </c>
       <c r="O11" s="0" t="n">
-        <v>337.5</v>
+        <v>652.5</v>
       </c>
       <c r="P11" s="0" t="n">
         <v>229.0</v>
       </c>
       <c r="Q11" s="0" t="n">
-        <v>21933.5</v>
+        <v>21618.5</v>
       </c>
       <c r="R11" s="0" t="inlineStr">
         <is>
-          <t>Sasha Porteny</t>
+          <t>Marihel Arias</t>
         </is>
       </c>
       <c r="S11" s="0" t="inlineStr">
         <is>
-          <t>sashaglatt@gmail.com</t>
+          <t>marihel_arias@hotmail.com</t>
         </is>
       </c>
       <c r="T11" s="0" t="inlineStr">
         <is>
-          <t>sashaglatt@gmail.com, trietedouard@gmail.com</t>
+          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
         </is>
       </c>
       <c r="U11" s="0" t="inlineStr">
         <is>
-          <t>Sasha Glatt Porteny, Edouard Triet</t>
+          <t>Marihel Arias, Alondra Arias</t>
         </is>
       </c>
       <c r="V11" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W11" s="0"/>
@@ -1288,21 +1288,21 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 15:13:36</t>
+          <t>2026/05/18 19:10:33</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 15:13:38</t>
+          <t>2026/05/18 19:11:20</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>822746635081215909888</t>
+          <t>822747479118273585152</t>
         </is>
       </c>
       <c r="D12" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="J12" s="0" t="n">
@@ -1336,46 +1336,46 @@
         <v>0.0</v>
       </c>
       <c r="L12" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M12" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N12" s="0" t="n">
-        <v>45000.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O12" s="0" t="n">
-        <v>1530.0</v>
+        <v>433.5</v>
       </c>
       <c r="P12" s="0" t="n">
-        <v>454.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q12" s="0" t="n">
-        <v>43016.0</v>
+        <v>12185.0</v>
       </c>
       <c r="R12" s="0" t="inlineStr">
         <is>
-          <t>SIMON NATHAN GITTLER</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="S12" s="0" t="inlineStr">
         <is>
-          <t>simon.gitt@gmail.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="T12" s="0" t="inlineStr">
         <is>
-          <t>simon.gitt@gmail.com, halina@hadasa.com.mx</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="U12" s="0" t="inlineStr">
         <is>
-          <t>SIMON NATHAN GITTLER SALOMON, Halina Unikel</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="V12" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W12" s="0"/>
@@ -1393,21 +1393,21 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 03:20:35</t>
+          <t>2026/05/18 19:10:32</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>2026/05/17 03:20:37</t>
+          <t>2026/05/18 19:11:18</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>822746276208009285632</t>
+          <t>822747479109650092032</t>
         </is>
       </c>
       <c r="D13" s="0" t="n">
-        <v>45000.0</v>
+        <v>18000.0</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
@@ -1426,12 +1426,12 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I13" s="0" t="inlineStr">
         <is>
-          <t>1009</t>
+          <t>6156</t>
         </is>
       </c>
       <c r="J13" s="0" t="n">
@@ -1441,41 +1441,41 @@
         <v>0.0</v>
       </c>
       <c r="L13" s="0" t="n">
-        <v>45000.0</v>
+        <v>18000.0</v>
       </c>
       <c r="M13" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N13" s="0" t="n">
-        <v>45000.0</v>
+        <v>18000.0</v>
       </c>
       <c r="O13" s="0" t="n">
-        <v>1530.0</v>
+        <v>522.0</v>
       </c>
       <c r="P13" s="0" t="n">
-        <v>454.0</v>
+        <v>184.0</v>
       </c>
       <c r="Q13" s="0" t="n">
-        <v>43016.0</v>
+        <v>17294.0</v>
       </c>
       <c r="R13" s="0" t="inlineStr">
         <is>
-          <t>Mauricio Schiavon magaña</t>
+          <t>Alejandra Serpas</t>
         </is>
       </c>
       <c r="S13" s="0" t="inlineStr">
         <is>
-          <t>mschiavon@me.com</t>
+          <t>denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="T13" s="0" t="inlineStr">
         <is>
-          <t>mschiavon@me.com, mschiavon@me.com</t>
+          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="U13" s="0" t="inlineStr">
         <is>
-          <t>Mauricio Esteban Schiavon Magaña, Mauricio Esteban Schiavon Magaña</t>
+          <t>Alejandra Serpas, Denisse Olivo</t>
         </is>
       </c>
       <c r="V13" s="0" t="inlineStr">
@@ -1498,21 +1498,21 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/16 16:30:32</t>
+          <t>2026/05/18 19:10:31</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026/05/16 23:29:12</t>
+          <t>2026/05/18 19:11:14</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>822745949026787532800</t>
+          <t>822747479096832299008</t>
         </is>
       </c>
       <c r="D14" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
@@ -1526,15 +1526,19 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>spei</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t>SPEI</t>
-        </is>
-      </c>
-      <c r="I14" s="0"/>
+          <t>mastercard</t>
+        </is>
+      </c>
+      <c r="I14" s="0" t="inlineStr">
+        <is>
+          <t>5558</t>
+        </is>
+      </c>
       <c r="J14" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1542,46 +1546,46 @@
         <v>0.0</v>
       </c>
       <c r="L14" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M14" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N14" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O14" s="0" t="n">
-        <v>0.0</v>
+        <v>652.5</v>
       </c>
       <c r="P14" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q14" s="0" t="n">
-        <v>44546.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R14" s="0" t="inlineStr">
         <is>
-          <t>Miguel Ángel Garcia</t>
+          <t>IGNACIO PORTILLA</t>
         </is>
       </c>
       <c r="S14" s="0" t="inlineStr">
         <is>
-          <t>miguel@garcia.mx</t>
+          <t>mx.portilla@gmail.com</t>
         </is>
       </c>
       <c r="T14" s="0" t="inlineStr">
         <is>
-          <t>Miguel@garcia.mx, Paonany8@gmail.com</t>
+          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
         </is>
       </c>
       <c r="U14" s="0" t="inlineStr">
         <is>
-          <t>Miguel Ángel Garcia, María Elena Sánche</t>
+          <t>VALERIA PORTILLA, Natalia Portilla</t>
         </is>
       </c>
       <c r="V14" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W14" s="0"/>
@@ -1599,21 +1603,21 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>2026/05/15 17:24:50</t>
+          <t>2026/05/18 16:14:03</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>2026/05/15 17:24:53</t>
+          <t>2026/05/18 16:14:03</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>822745251580101009408</t>
+          <t>822747390277042835456</t>
         </is>
       </c>
       <c r="D15" s="0" t="n">
-        <v>22500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
@@ -1627,19 +1631,15 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
-        </is>
-      </c>
-      <c r="I15" s="0" t="inlineStr">
-        <is>
-          <t>3097</t>
-        </is>
-      </c>
+          <t>Transferencia</t>
+        </is>
+      </c>
+      <c r="I15" s="0"/>
       <c r="J15" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -1647,46 +1647,46 @@
         <v>0.0</v>
       </c>
       <c r="L15" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M15" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N15" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O15" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P15" s="0" t="n">
-        <v>229.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q15" s="0" t="n">
-        <v>21618.5</v>
+        <v>0.0</v>
       </c>
       <c r="R15" s="0" t="inlineStr">
         <is>
-          <t>Marihel Arias</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S15" s="0" t="inlineStr">
         <is>
-          <t>marihel_arias@hotmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T15" s="0" t="inlineStr">
         <is>
-          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U15" s="0" t="inlineStr">
         <is>
-          <t>Marihel Arias, Alondra Arias</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V15" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W15" s="0"/>
@@ -1704,21 +1704,21 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>2026/05/14 21:47:03</t>
+          <t>2026/05/18 01:01:03</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>2026/05/14 21:47:05</t>
+          <t>2026/05/18 01:01:18</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>822744658783664881664</t>
+          <t>822746930752535928832</t>
         </is>
       </c>
       <c r="D16" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>6353</t>
         </is>
       </c>
       <c r="J16" s="0" t="n">
@@ -1752,46 +1752,46 @@
         <v>0.0</v>
       </c>
       <c r="L16" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M16" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N16" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O16" s="0" t="n">
-        <v>1530.0</v>
+        <v>337.5</v>
       </c>
       <c r="P16" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q16" s="0" t="n">
-        <v>43016.0</v>
+        <v>21933.5</v>
       </c>
       <c r="R16" s="0" t="inlineStr">
         <is>
-          <t>FERNANDO FONSECA</t>
+          <t>Sasha Porteny</t>
         </is>
       </c>
       <c r="S16" s="0" t="inlineStr">
         <is>
-          <t>fonsecaf88@gmail.com</t>
+          <t>sashaglatt@gmail.com</t>
         </is>
       </c>
       <c r="T16" s="0" t="inlineStr">
         <is>
-          <t>fonsecaf88@gmail.com, fonsecaf88@gmail.com</t>
+          <t>sashaglatt@gmail.com, trietedouard@gmail.com</t>
         </is>
       </c>
       <c r="U16" s="0" t="inlineStr">
         <is>
-          <t>FERNANDO FONSECA, Matias fonseca</t>
+          <t>Sasha Glatt Porteny, Edouard Triet</t>
         </is>
       </c>
       <c r="V16" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W16" s="0"/>
@@ -1809,21 +1809,21 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:31</t>
+          <t>2026/05/17 15:13:36</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 04:18:33</t>
+          <t>2026/05/17 15:13:38</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>822743406261352546304</t>
+          <t>822746635081215909888</t>
         </is>
       </c>
       <c r="D17" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>1009</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="J17" s="0" t="n">
@@ -1857,46 +1857,46 @@
         <v>0.0</v>
       </c>
       <c r="L17" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M17" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N17" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O17" s="0" t="n">
-        <v>433.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P17" s="0" t="n">
-        <v>131.5</v>
+        <v>454.0</v>
       </c>
       <c r="Q17" s="0" t="n">
-        <v>12185.0</v>
+        <v>43016.0</v>
       </c>
       <c r="R17" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>SIMON NATHAN GITTLER</t>
         </is>
       </c>
       <c r="S17" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>simon.gitt@gmail.com</t>
         </is>
       </c>
       <c r="T17" s="0" t="inlineStr">
         <is>
-          <t>roenecoiz@gmail.com</t>
+          <t>simon.gitt@gmail.com, halina@hadasa.com.mx</t>
         </is>
       </c>
       <c r="U17" s="0" t="inlineStr">
         <is>
-          <t>Rodrigo Enecoiz</t>
+          <t>SIMON NATHAN GITTLER SALOMON, Halina Unikel</t>
         </is>
       </c>
       <c r="V17" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W17" s="0"/>
@@ -1914,21 +1914,21 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:03</t>
+          <t>2026/05/17 03:20:35</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>2026/05/13 03:36:05</t>
+          <t>2026/05/17 03:20:37</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>822743384884528578560</t>
+          <t>822746276208009285632</t>
         </is>
       </c>
       <c r="D18" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -1947,12 +1947,12 @@
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t>7758</t>
+          <t>1009</t>
         </is>
       </c>
       <c r="J18" s="0" t="n">
@@ -1962,41 +1962,41 @@
         <v>0.0</v>
       </c>
       <c r="L18" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M18" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N18" s="0" t="n">
-        <v>12750.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O18" s="0" t="n">
-        <v>369.75</v>
+        <v>1530.0</v>
       </c>
       <c r="P18" s="0" t="n">
-        <v>131.5</v>
+        <v>454.0</v>
       </c>
       <c r="Q18" s="0" t="n">
-        <v>12248.75</v>
+        <v>43016.0</v>
       </c>
       <c r="R18" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>Mauricio Schiavon magaña</t>
         </is>
       </c>
       <c r="S18" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>mschiavon@me.com</t>
         </is>
       </c>
       <c r="T18" s="0" t="inlineStr">
         <is>
-          <t>tanyagza@gmail.com</t>
+          <t>mschiavon@me.com, mschiavon@me.com</t>
         </is>
       </c>
       <c r="U18" s="0" t="inlineStr">
         <is>
-          <t>Tanya Garza</t>
+          <t>Mauricio Esteban Schiavon Magaña, Mauricio Esteban Schiavon Magaña</t>
         </is>
       </c>
       <c r="V18" s="0" t="inlineStr">
@@ -2019,21 +2019,21 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:39</t>
+          <t>2026/05/16 16:30:32</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 21:17:41</t>
+          <t>2026/05/16 23:29:12</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>822743194435830431744</t>
+          <t>822745949026787532800</t>
         </is>
       </c>
       <c r="D19" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
@@ -2047,19 +2047,15 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>spei</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I19" s="0" t="inlineStr">
-        <is>
-          <t>9925</t>
-        </is>
-      </c>
+          <t>SPEI</t>
+        </is>
+      </c>
+      <c r="I19" s="0"/>
       <c r="J19" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -2067,46 +2063,46 @@
         <v>0.0</v>
       </c>
       <c r="L19" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M19" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N19" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O19" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P19" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q19" s="0" t="n">
-        <v>21618.5</v>
+        <v>44546.0</v>
       </c>
       <c r="R19" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>Miguel Ángel Garcia</t>
         </is>
       </c>
       <c r="S19" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>miguel@garcia.mx</t>
         </is>
       </c>
       <c r="T19" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>Miguel@garcia.mx, Paonany8@gmail.com</t>
         </is>
       </c>
       <c r="U19" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>Miguel Ángel Garcia, María Elena Sánche</t>
         </is>
       </c>
       <c r="V19" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W19" s="0"/>
@@ -2124,17 +2120,17 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:10:30</t>
+          <t>2026/05/15 17:24:50</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 19:11:16</t>
+          <t>2026/05/15 17:24:53</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>822743130440389902336</t>
+          <t>822745251580101009408</t>
         </is>
       </c>
       <c r="D20" s="0" t="n">
@@ -2157,12 +2153,12 @@
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>3097</t>
         </is>
       </c>
       <c r="J20" s="0" t="n">
@@ -2191,27 +2187,27 @@
       </c>
       <c r="R20" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>Marihel Arias</t>
         </is>
       </c>
       <c r="S20" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>marihel_arias@hotmail.com</t>
         </is>
       </c>
       <c r="T20" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>marihel_arias@hotmail.com, lizbethariasglez@gmail.com</t>
         </is>
       </c>
       <c r="U20" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>Marihel Arias, Alondra Arias</t>
         </is>
       </c>
       <c r="V20" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W20" s="0"/>
@@ -2229,17 +2225,17 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:51</t>
+          <t>2026/05/14 21:47:03</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>2026/05/12 18:19:53</t>
+          <t>2026/05/14 21:47:05</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>822743104942704197632</t>
+          <t>822744658783664881664</t>
         </is>
       </c>
       <c r="D21" s="0" t="n">
@@ -2262,12 +2258,12 @@
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t>1709</t>
+          <t>1003</t>
         </is>
       </c>
       <c r="J21" s="0" t="n">
@@ -2286,37 +2282,37 @@
         <v>45000.0</v>
       </c>
       <c r="O21" s="0" t="n">
-        <v>1305.0</v>
+        <v>1530.0</v>
       </c>
       <c r="P21" s="0" t="n">
         <v>454.0</v>
       </c>
       <c r="Q21" s="0" t="n">
-        <v>43241.0</v>
+        <v>43016.0</v>
       </c>
       <c r="R21" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ</t>
+          <t>FERNANDO FONSECA</t>
         </is>
       </c>
       <c r="S21" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com</t>
+          <t>fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="T21" s="0" t="inlineStr">
         <is>
-          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
+          <t>fonsecaf88@gmail.com, fonsecaf88@gmail.com</t>
         </is>
       </c>
       <c r="U21" s="0" t="inlineStr">
         <is>
-          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
+          <t>FERNANDO FONSECA, Matias fonseca</t>
         </is>
       </c>
       <c r="V21" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W21" s="0"/>
@@ -2334,21 +2330,21 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/13 04:18:31</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:03:44</t>
+          <t>2026/05/13 04:18:33</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>822742523051869483008</t>
+          <t>822743406261352546304</t>
         </is>
       </c>
       <c r="D22" s="0" t="n">
-        <v>20500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -2362,15 +2358,19 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="I22" s="0"/>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I22" s="0" t="inlineStr">
+        <is>
+          <t>1009</t>
+        </is>
+      </c>
       <c r="J22" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -2378,41 +2378,41 @@
         <v>0.0</v>
       </c>
       <c r="L22" s="0" t="n">
-        <v>0.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M22" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N22" s="0" t="n">
-        <v>0.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O22" s="0" t="n">
-        <v>0.0</v>
+        <v>433.5</v>
       </c>
       <c r="P22" s="0" t="n">
-        <v>0.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q22" s="0" t="n">
-        <v>0.0</v>
+        <v>12185.0</v>
       </c>
       <c r="R22" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="S22" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="T22" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>roenecoiz@gmail.com</t>
         </is>
       </c>
       <c r="U22" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Rodrigo Enecoiz</t>
         </is>
       </c>
       <c r="V22" s="0" t="inlineStr">
@@ -2435,21 +2435,21 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:09</t>
+          <t>2026/05/13 03:36:03</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 22:22:12</t>
+          <t>2026/05/13 03:36:05</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>822742502121738878976</t>
+          <t>822743384884528578560</t>
         </is>
       </c>
       <c r="D23" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -2468,12 +2468,12 @@
       </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t>1775</t>
+          <t>7758</t>
         </is>
       </c>
       <c r="J23" s="0" t="n">
@@ -2483,46 +2483,46 @@
         <v>0.0</v>
       </c>
       <c r="L23" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="M23" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N23" s="0" t="n">
-        <v>22500.0</v>
+        <v>12750.0</v>
       </c>
       <c r="O23" s="0" t="n">
-        <v>652.5</v>
+        <v>369.75</v>
       </c>
       <c r="P23" s="0" t="n">
-        <v>229.0</v>
+        <v>131.5</v>
       </c>
       <c r="Q23" s="0" t="n">
-        <v>21618.5</v>
+        <v>12248.75</v>
       </c>
       <c r="R23" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="S23" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="T23" s="0" t="inlineStr">
         <is>
-          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
+          <t>tanyagza@gmail.com</t>
         </is>
       </c>
       <c r="U23" s="0" t="inlineStr">
         <is>
-          <t>Macarena Olavarri, Isabel Fernández</t>
+          <t>Tanya Garza</t>
         </is>
       </c>
       <c r="V23" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W23" s="0"/>
@@ -2540,21 +2540,21 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:41</t>
+          <t>2026/05/12 21:17:39</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 23:10:43</t>
+          <t>2026/05/12 21:17:41</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>822740352219193810944</t>
+          <t>822743194435830431744</t>
         </is>
       </c>
       <c r="D24" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>9925</t>
         </is>
       </c>
       <c r="J24" s="0" t="n">
@@ -2588,46 +2588,46 @@
         <v>0.0</v>
       </c>
       <c r="L24" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M24" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N24" s="0" t="n">
-        <v>81000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O24" s="0" t="n">
-        <v>2754.0</v>
+        <v>652.5</v>
       </c>
       <c r="P24" s="0" t="n">
-        <v>814.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q24" s="0" t="n">
-        <v>77432.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R24" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S24" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T24" s="0" t="inlineStr">
         <is>
-          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U24" s="0" t="inlineStr">
         <is>
-          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V24" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W24" s="0"/>
@@ -2645,21 +2645,21 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:11</t>
+          <t>2026/05/12 19:10:30</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:45:12</t>
+          <t>2026/05/12 19:11:16</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>822740218587619794944</t>
+          <t>822743130440389902336</t>
         </is>
       </c>
       <c r="D25" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -2683,7 +2683,7 @@
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>6624</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J25" s="0" t="n">
@@ -2693,46 +2693,46 @@
         <v>0.0</v>
       </c>
       <c r="L25" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M25" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N25" s="0" t="n">
-        <v>25500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O25" s="0" t="n">
-        <v>739.5</v>
+        <v>652.5</v>
       </c>
       <c r="P25" s="0" t="n">
-        <v>259.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q25" s="0" t="n">
-        <v>24501.5</v>
+        <v>21618.5</v>
       </c>
       <c r="R25" s="0" t="inlineStr">
         <is>
-          <t>MELB PEREZ SALDANA</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S25" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T25" s="0" t="inlineStr">
         <is>
-          <t>asistente@corporativojamia.com</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U25" s="0" t="inlineStr">
         <is>
-          <t>MELBA ASTRID PEREZ SALDAÑA</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V25" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W25" s="0"/>
@@ -2750,21 +2750,21 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:10</t>
+          <t>2026/05/12 18:19:51</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>2026/05/08 18:14:12</t>
+          <t>2026/05/12 18:19:53</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>822740202977192058880</t>
+          <t>822743104942704197632</t>
         </is>
       </c>
       <c r="D26" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t>9925</t>
+          <t>1709</t>
         </is>
       </c>
       <c r="J26" s="0" t="n">
@@ -2798,46 +2798,46 @@
         <v>0.0</v>
       </c>
       <c r="L26" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M26" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N26" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O26" s="0" t="n">
-        <v>652.5</v>
+        <v>1305.0</v>
       </c>
       <c r="P26" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q26" s="0" t="n">
-        <v>21618.5</v>
+        <v>43241.0</v>
       </c>
       <c r="R26" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores</t>
+          <t>RAFAEL BELTRAN LOPEZ</t>
         </is>
       </c>
       <c r="S26" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com</t>
+          <t>rbeltran1976@hotmail.com</t>
         </is>
       </c>
       <c r="T26" s="0" t="inlineStr">
         <is>
-          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
+          <t>rbeltran1976@hotmail.com, macasanchez77@hotmail.com</t>
         </is>
       </c>
       <c r="U26" s="0" t="inlineStr">
         <is>
-          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
+          <t>RAFAEL BELTRAN LOPEZ, Margarita Sanchez Rios</t>
         </is>
       </c>
       <c r="V26" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W26" s="0"/>
@@ -2855,21 +2855,21 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:20</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>2026/05/07 00:33:22</t>
+          <t>2026/05/11 23:03:44</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>822738944267014664192</t>
+          <t>822742523051869483008</t>
         </is>
       </c>
       <c r="D27" s="0" t="n">
-        <v>22500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -2883,19 +2883,15 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
-        </is>
-      </c>
-      <c r="I27" s="0" t="inlineStr">
-        <is>
-          <t>6156</t>
-        </is>
-      </c>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I27" s="0"/>
       <c r="J27" s="0" t="n">
         <v>0.0</v>
       </c>
@@ -2903,46 +2899,46 @@
         <v>0.0</v>
       </c>
       <c r="L27" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M27" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N27" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O27" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P27" s="0" t="n">
-        <v>229.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q27" s="0" t="n">
-        <v>21618.5</v>
+        <v>0.0</v>
       </c>
       <c r="R27" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S27" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T27" s="0" t="inlineStr">
         <is>
-          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U27" s="0" t="inlineStr">
         <is>
-          <t>Alejandra Serpas, Denisse Olivo</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V27" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W27" s="0"/>
@@ -2960,25 +2956,25 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>2026/05/06 23:07:12</t>
+          <t>2026/05/11 22:22:09</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>2026/05/11 23:05:58</t>
+          <t>2026/05/11 22:22:12</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>822738900913572839424</t>
+          <t>822742502121738878976</t>
         </is>
       </c>
       <c r="D28" s="0" t="n">
-        <v>20500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Refunded</t>
+          <t>Successful</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
@@ -2988,62 +2984,66 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>External</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t>transferencia</t>
-        </is>
-      </c>
-      <c r="I28" s="0"/>
+          <t>mastercard</t>
+        </is>
+      </c>
+      <c r="I28" s="0" t="inlineStr">
+        <is>
+          <t>1775</t>
+        </is>
+      </c>
       <c r="J28" s="0" t="n">
-        <v>20500.0</v>
+        <v>0.0</v>
       </c>
       <c r="K28" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L28" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M28" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N28" s="0" t="n">
-        <v>0.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O28" s="0" t="n">
-        <v>0.0</v>
+        <v>652.5</v>
       </c>
       <c r="P28" s="0" t="n">
-        <v>0.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q28" s="0" t="n">
-        <v>0.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R28" s="0" t="inlineStr">
         <is>
-          <t>María Patricia García Kern</t>
+          <t>Macarena Olavarri</t>
         </is>
       </c>
       <c r="S28" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com</t>
+          <t>macaolavarri@gmail.com</t>
         </is>
       </c>
       <c r="T28" s="0" t="inlineStr">
         <is>
-          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
+          <t>macaolavarri@gmail.com, isafer31@gmail.com</t>
         </is>
       </c>
       <c r="U28" s="0" t="inlineStr">
         <is>
-          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
+          <t>Macarena Olavarri, Isabel Fernández</t>
         </is>
       </c>
       <c r="V28" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W28" s="0"/>
@@ -3061,21 +3061,21 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:40</t>
+          <t>2026/05/08 23:10:41</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>2026/05/02 22:46:42</t>
+          <t>2026/05/08 23:10:43</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>822735991480689651712</t>
+          <t>822740352219193810944</t>
         </is>
       </c>
       <c r="D29" s="0" t="n">
-        <v>45000.0</v>
+        <v>81000.0</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t>2003</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="J29" s="0" t="n">
@@ -3109,41 +3109,41 @@
         <v>0.0</v>
       </c>
       <c r="L29" s="0" t="n">
-        <v>45000.0</v>
+        <v>81000.0</v>
       </c>
       <c r="M29" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N29" s="0" t="n">
-        <v>45000.0</v>
+        <v>81000.0</v>
       </c>
       <c r="O29" s="0" t="n">
-        <v>1530.0</v>
+        <v>2754.0</v>
       </c>
       <c r="P29" s="0" t="n">
-        <v>454.0</v>
+        <v>814.0</v>
       </c>
       <c r="Q29" s="0" t="n">
-        <v>43016.0</v>
+        <v>77432.0</v>
       </c>
       <c r="R29" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES</t>
+          <t>Judith Escobar Torres</t>
         </is>
       </c>
       <c r="S29" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com</t>
+          <t>judith.escobar@gmail.com</t>
         </is>
       </c>
       <c r="T29" s="0" t="inlineStr">
         <is>
-          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
+          <t>judith.escobar@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com, fernando.ruizgalindo@gmail.com</t>
         </is>
       </c>
       <c r="U29" s="0" t="inlineStr">
         <is>
-          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
+          <t>Judith Escobar Torres, Fernando Ruiz Galindo Drucker, Leonardo Ruiz Galindo Escobar, Alexa Ruiz Galindo Escobar</t>
         </is>
       </c>
       <c r="V29" s="0" t="inlineStr">
@@ -3166,21 +3166,21 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:35</t>
+          <t>2026/05/08 18:45:11</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 21:08:36</t>
+          <t>2026/05/08 18:45:12</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>822733043006520176640</t>
+          <t>822740218587619794944</t>
         </is>
       </c>
       <c r="D30" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -3199,12 +3199,12 @@
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t>mastercard</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t>5558</t>
+          <t>6624</t>
         </is>
       </c>
       <c r="J30" s="0" t="n">
@@ -3214,41 +3214,41 @@
         <v>0.0</v>
       </c>
       <c r="L30" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M30" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N30" s="0" t="n">
-        <v>22500.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O30" s="0" t="n">
-        <v>652.5</v>
+        <v>739.5</v>
       </c>
       <c r="P30" s="0" t="n">
-        <v>229.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q30" s="0" t="n">
-        <v>21618.5</v>
+        <v>24501.5</v>
       </c>
       <c r="R30" s="0" t="inlineStr">
         <is>
-          <t>IGNACIO PORTILLA</t>
+          <t>MELB PEREZ SALDANA</t>
         </is>
       </c>
       <c r="S30" s="0" t="inlineStr">
         <is>
-          <t>mx.portilla@gmail.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="T30" s="0" t="inlineStr">
         <is>
-          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
+          <t>asistente@corporativojamia.com</t>
         </is>
       </c>
       <c r="U30" s="0" t="inlineStr">
         <is>
-          <t>VALERIA PORTILLA, Natalia Portilla</t>
+          <t>MELBA ASTRID PEREZ SALDAÑA</t>
         </is>
       </c>
       <c r="V30" s="0" t="inlineStr">
@@ -3271,21 +3271,21 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:10:30</t>
+          <t>2026/05/08 18:14:10</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>2026/04/28 19:11:05</t>
+          <t>2026/05/08 18:14:12</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>822732983572553019392</t>
+          <t>822740202977192058880</t>
         </is>
       </c>
       <c r="D31" s="0" t="n">
-        <v>18000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="I31" s="0" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>9925</t>
         </is>
       </c>
       <c r="J31" s="0" t="n">
@@ -3319,46 +3319,46 @@
         <v>0.0</v>
       </c>
       <c r="L31" s="0" t="n">
-        <v>18000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M31" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N31" s="0" t="n">
-        <v>18000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O31" s="0" t="n">
-        <v>522.0</v>
+        <v>652.5</v>
       </c>
       <c r="P31" s="0" t="n">
-        <v>184.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q31" s="0" t="n">
-        <v>17294.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R31" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>Alexis Navarro Flores</t>
         </is>
       </c>
       <c r="S31" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>alexisnf09@hotmail.com</t>
         </is>
       </c>
       <c r="T31" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>alexisnf09@hotmail.com, hansfernandovll@gmail.com</t>
         </is>
       </c>
       <c r="U31" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>Alexis Navarro Flores, Hans del Valle Manzano</t>
         </is>
       </c>
       <c r="V31" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W31" s="0"/>
@@ -3376,21 +3376,21 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:49</t>
+          <t>2026/05/07 00:33:20</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>2026/04/22 00:32:51</t>
+          <t>2026/05/07 00:33:22</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>822728072370714607616</t>
+          <t>822738944267014664192</t>
         </is>
       </c>
       <c r="D32" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
@@ -3409,12 +3409,12 @@
       </c>
       <c r="H32" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t>2071</t>
+          <t>6156</t>
         </is>
       </c>
       <c r="J32" s="0" t="n">
@@ -3424,46 +3424,46 @@
         <v>0.0</v>
       </c>
       <c r="L32" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M32" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N32" s="0" t="n">
-        <v>9833.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O32" s="0" t="n">
-        <v>285.16</v>
+        <v>652.5</v>
       </c>
       <c r="P32" s="0" t="n">
-        <v>102.33</v>
+        <v>229.0</v>
       </c>
       <c r="Q32" s="0" t="n">
-        <v>9445.51</v>
+        <v>21618.5</v>
       </c>
       <c r="R32" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>Alejandra Serpas</t>
         </is>
       </c>
       <c r="S32" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="T32" s="0" t="inlineStr">
         <is>
-          <t>daniabahena@gmail.com</t>
+          <t>denisse.olivo@fora.travel, denisse.olivo@fora.travel</t>
         </is>
       </c>
       <c r="U32" s="0" t="inlineStr">
         <is>
-          <t>Dania Bahena</t>
+          <t>Alejandra Serpas, Denisse Olivo</t>
         </is>
       </c>
       <c r="V32" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W32" s="0"/>
@@ -3481,25 +3481,25 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:44</t>
+          <t>2026/05/06 23:07:12</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 22:51:46</t>
+          <t>2026/05/11 23:05:58</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>822728021498622136320</t>
+          <t>822738900913572839424</t>
         </is>
       </c>
       <c r="D33" s="0" t="n">
-        <v>22500.0</v>
+        <v>20500.0</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Successful</t>
+          <t>Refunded</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
@@ -3509,61 +3509,57 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>External</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
-        </is>
-      </c>
-      <c r="I33" s="0" t="inlineStr">
-        <is>
-          <t>4583</t>
-        </is>
-      </c>
+          <t>transferencia</t>
+        </is>
+      </c>
+      <c r="I33" s="0"/>
       <c r="J33" s="0" t="n">
-        <v>0.0</v>
+        <v>20500.0</v>
       </c>
       <c r="K33" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="L33" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="M33" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N33" s="0" t="n">
-        <v>22500.0</v>
+        <v>0.0</v>
       </c>
       <c r="O33" s="0" t="n">
-        <v>652.5</v>
+        <v>0.0</v>
       </c>
       <c r="P33" s="0" t="n">
-        <v>229.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q33" s="0" t="n">
-        <v>21618.5</v>
+        <v>0.0</v>
       </c>
       <c r="R33" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON</t>
+          <t>María Patricia García Kern</t>
         </is>
       </c>
       <c r="S33" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com</t>
+          <t>patricia.garcia@viajeslegrand.com</t>
         </is>
       </c>
       <c r="T33" s="0" t="inlineStr">
         <is>
-          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
+          <t>patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com, patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled), patricia.garcia@viajeslegrand.com (Canceled)</t>
         </is>
       </c>
       <c r="U33" s="0" t="inlineStr">
         <is>
-          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
+          <t>Maria Patricia Garcia, Maria Patricia Garcia, María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled), María Patricia García Kern (Canceled)</t>
         </is>
       </c>
       <c r="V33" s="0" t="inlineStr">
@@ -3586,21 +3582,21 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:01</t>
+          <t>2026/05/02 22:46:40</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 04:06:03</t>
+          <t>2026/05/02 22:46:42</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>822727454901268389888</t>
+          <t>822735991480689651712</t>
         </is>
       </c>
       <c r="D34" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
@@ -3619,12 +3615,12 @@
       </c>
       <c r="H34" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I34" s="0" t="inlineStr">
         <is>
-          <t>7580</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="J34" s="0" t="n">
@@ -3634,46 +3630,46 @@
         <v>0.0</v>
       </c>
       <c r="L34" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M34" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N34" s="0" t="n">
-        <v>22500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O34" s="0" t="n">
-        <v>652.5</v>
+        <v>1530.0</v>
       </c>
       <c r="P34" s="0" t="n">
-        <v>229.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q34" s="0" t="n">
-        <v>21618.5</v>
+        <v>43016.0</v>
       </c>
       <c r="R34" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya</t>
+          <t>ALEJANDRO CANALES MORALES</t>
         </is>
       </c>
       <c r="S34" s="0" t="inlineStr">
         <is>
-          <t>dan.rios.an.182@gmail.com</t>
+          <t>alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="T34" s="0" t="inlineStr">
         <is>
-          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
+          <t>alejandro.canales.morales@gmail.com, alejandro.canales.morales@gmail.com</t>
         </is>
       </c>
       <c r="U34" s="0" t="inlineStr">
         <is>
-          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
+          <t>ALEJANDRO CANALES MORALES, Ampelio Canales Zaragoza</t>
         </is>
       </c>
       <c r="V34" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W34" s="0"/>
@@ -3691,17 +3687,17 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:12</t>
+          <t>2026/04/28 21:08:35</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>2026/04/21 01:07:13</t>
+          <t>2026/04/28 21:08:36</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>822727364900010598400</t>
+          <t>822733043006520176640</t>
         </is>
       </c>
       <c r="D35" s="0" t="n">
@@ -3724,12 +3720,12 @@
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>mastercard</t>
         </is>
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t>7852</t>
+          <t>5558</t>
         </is>
       </c>
       <c r="J35" s="0" t="n">
@@ -3758,22 +3754,22 @@
       </c>
       <c r="R35" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL</t>
+          <t>IGNACIO PORTILLA</t>
         </is>
       </c>
       <c r="S35" s="0" t="inlineStr">
         <is>
-          <t>ricardocb23@gmail.com</t>
+          <t>mx.portilla@gmail.com</t>
         </is>
       </c>
       <c r="T35" s="0" t="inlineStr">
         <is>
-          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
+          <t>valeriaportilla@icloud.com, nataliaportilla@icloud.com</t>
         </is>
       </c>
       <c r="U35" s="0" t="inlineStr">
         <is>
-          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
+          <t>VALERIA PORTILLA, Natalia Portilla</t>
         </is>
       </c>
       <c r="V35" s="0" t="inlineStr">
@@ -3796,21 +3792,21 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:19</t>
+          <t>2026/04/28 19:10:30</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>2026/04/19 20:19:21</t>
+          <t>2026/04/28 19:11:05</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>822726495229304659968</t>
+          <t>822732983572553019392</t>
         </is>
       </c>
       <c r="D36" s="0" t="n">
-        <v>14750.0</v>
+        <v>18000.0</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
@@ -3824,17 +3820,17 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>apple_pay</t>
+          <t>card</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J36" s="0" t="n">
@@ -3844,46 +3840,46 @@
         <v>0.0</v>
       </c>
       <c r="L36" s="0" t="n">
-        <v>14750.0</v>
+        <v>18000.0</v>
       </c>
       <c r="M36" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N36" s="0" t="n">
-        <v>14750.0</v>
+        <v>18000.0</v>
       </c>
       <c r="O36" s="0" t="n">
-        <v>427.75</v>
+        <v>522.0</v>
       </c>
       <c r="P36" s="0" t="n">
-        <v>151.5</v>
+        <v>184.0</v>
       </c>
       <c r="Q36" s="0" t="n">
-        <v>14170.75</v>
+        <v>17294.0</v>
       </c>
       <c r="R36" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S36" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T36" s="0" t="inlineStr">
         <is>
-          <t>nataly_victoria16@yahoo.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U36" s="0" t="inlineStr">
         <is>
-          <t>Victoria Medina</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V36" s="0" t="inlineStr">
         <is>
-          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W36" s="0"/>
@@ -3901,21 +3897,21 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:21</t>
+          <t>2026/04/22 00:32:49</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>2026/04/18 18:51:23</t>
+          <t>2026/04/22 00:32:51</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>822725726179188305920</t>
+          <t>822728072370714607616</t>
         </is>
       </c>
       <c r="D37" s="0" t="n">
-        <v>25500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
@@ -3939,7 +3935,7 @@
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t>9962</t>
+          <t>2071</t>
         </is>
       </c>
       <c r="J37" s="0" t="n">
@@ -3949,46 +3945,46 @@
         <v>0.0</v>
       </c>
       <c r="L37" s="0" t="n">
-        <v>25500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="M37" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N37" s="0" t="n">
-        <v>25500.0</v>
+        <v>9833.0</v>
       </c>
       <c r="O37" s="0" t="n">
-        <v>739.5</v>
+        <v>285.16</v>
       </c>
       <c r="P37" s="0" t="n">
-        <v>259.0</v>
+        <v>102.33</v>
       </c>
       <c r="Q37" s="0" t="n">
-        <v>24501.5</v>
+        <v>9445.51</v>
       </c>
       <c r="R37" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon Mendez</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="S37" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="T37" s="0" t="inlineStr">
         <is>
-          <t>johnoregon@live.com</t>
+          <t>daniabahena@gmail.com</t>
         </is>
       </c>
       <c r="U37" s="0" t="inlineStr">
         <is>
-          <t>Jonatan Oregon</t>
+          <t>Dania Bahena</t>
         </is>
       </c>
       <c r="V37" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W37" s="0"/>
@@ -4006,21 +4002,21 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:42</t>
+          <t>2026/04/21 22:51:44</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>2026/04/17 16:38:44</t>
+          <t>2026/04/21 22:51:46</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>822724934643911520256</t>
+          <t>822728021498622136320</t>
         </is>
       </c>
       <c r="D38" s="0" t="n">
-        <v>70500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
@@ -4039,12 +4035,12 @@
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="J38" s="0" t="n">
@@ -4054,41 +4050,41 @@
         <v>0.0</v>
       </c>
       <c r="L38" s="0" t="n">
-        <v>70500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M38" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N38" s="0" t="n">
-        <v>70500.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O38" s="0" t="n">
-        <v>2397.0</v>
+        <v>652.5</v>
       </c>
       <c r="P38" s="0" t="n">
-        <v>709.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q38" s="0" t="n">
-        <v>67394.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R38" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos</t>
+          <t>MARIA DE MONTSERRAT CERON</t>
         </is>
       </c>
       <c r="S38" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com</t>
+          <t>mdmtramites@gmail.com</t>
         </is>
       </c>
       <c r="T38" s="0" t="inlineStr">
         <is>
-          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
+          <t>mdmtramites@gmail.com, carla.ceron@yahoo.com.mx</t>
         </is>
       </c>
       <c r="U38" s="0" t="inlineStr">
         <is>
-          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
+          <t>MARIA DE MONTSERRAT CERON, CARLA CERON</t>
         </is>
       </c>
       <c r="V38" s="0" t="inlineStr">
@@ -4111,21 +4107,21 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:28</t>
+          <t>2026/04/21 04:06:01</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 22:04:30</t>
+          <t>2026/04/21 04:06:03</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>822722199504844500992</t>
+          <t>822727454901268389888</t>
         </is>
       </c>
       <c r="D39" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
@@ -4149,7 +4145,7 @@
       </c>
       <c r="I39" s="0" t="inlineStr">
         <is>
-          <t>4291</t>
+          <t>7580</t>
         </is>
       </c>
       <c r="J39" s="0" t="n">
@@ -4159,46 +4155,46 @@
         <v>0.0</v>
       </c>
       <c r="L39" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M39" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N39" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O39" s="0" t="n">
-        <v>1305.0</v>
+        <v>652.5</v>
       </c>
       <c r="P39" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q39" s="0" t="n">
-        <v>43241.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R39" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza</t>
+          <t>Daniel Alberto Ríos Anaya</t>
         </is>
       </c>
       <c r="S39" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com</t>
+          <t>dan.rios.an.182@gmail.com</t>
         </is>
       </c>
       <c r="T39" s="0" t="inlineStr">
         <is>
-          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
+          <t>Dan.rios.an.182@gmail.com, mel.araiza@hotmail.com</t>
         </is>
       </c>
       <c r="U39" s="0" t="inlineStr">
         <is>
-          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
+          <t>Daniel Alberto Ríos Anaya, Melissa Araiza</t>
         </is>
       </c>
       <c r="V39" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
         </is>
       </c>
       <c r="W39" s="0"/>
@@ -4216,21 +4212,21 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:45</t>
+          <t>2026/04/21 01:07:12</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>2026/04/13 19:26:47</t>
+          <t>2026/04/21 01:07:13</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>822722120121735725056</t>
+          <t>822727364900010598400</t>
         </is>
       </c>
       <c r="D40" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
@@ -4249,12 +4245,12 @@
       </c>
       <c r="H40" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I40" s="0" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>7852</t>
         </is>
       </c>
       <c r="J40" s="0" t="n">
@@ -4264,46 +4260,46 @@
         <v>0.0</v>
       </c>
       <c r="L40" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="M40" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N40" s="0" t="n">
-        <v>45000.0</v>
+        <v>22500.0</v>
       </c>
       <c r="O40" s="0" t="n">
-        <v>1530.0</v>
+        <v>652.5</v>
       </c>
       <c r="P40" s="0" t="n">
-        <v>454.0</v>
+        <v>229.0</v>
       </c>
       <c r="Q40" s="0" t="n">
-        <v>43016.0</v>
+        <v>21618.5</v>
       </c>
       <c r="R40" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac</t>
+          <t>RICARDO CAMACHO BOFILL</t>
         </is>
       </c>
       <c r="S40" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com</t>
+          <t>ricardocb23@gmail.com</t>
         </is>
       </c>
       <c r="T40" s="0" t="inlineStr">
         <is>
-          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
+          <t>Ricardocb23@gmail.com, danielapages07@gmail.com</t>
         </is>
       </c>
       <c r="U40" s="0" t="inlineStr">
         <is>
-          <t>Ana paula Isaac, Gabriela Vazquez</t>
+          <t>RICARDO CAMACHO BOFILL, Daniela Pages Salgado</t>
         </is>
       </c>
       <c r="V40" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W40" s="0"/>
@@ -4321,21 +4317,21 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:14</t>
+          <t>2026/04/19 20:19:19</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>2026/04/09 04:55:16</t>
+          <t>2026/04/19 20:19:21</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>822718782367677300736</t>
+          <t>822726495229304659968</t>
         </is>
       </c>
       <c r="D41" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
@@ -4354,12 +4350,12 @@
       </c>
       <c r="H41" s="0" t="inlineStr">
         <is>
-          <t>visa</t>
+          <t>amex</t>
         </is>
       </c>
       <c r="I41" s="0" t="inlineStr">
         <is>
-          <t>7348</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="J41" s="0" t="n">
@@ -4369,46 +4365,46 @@
         <v>0.0</v>
       </c>
       <c r="L41" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="M41" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N41" s="0" t="n">
-        <v>45000.0</v>
+        <v>14750.0</v>
       </c>
       <c r="O41" s="0" t="n">
-        <v>1305.0</v>
+        <v>427.75</v>
       </c>
       <c r="P41" s="0" t="n">
-        <v>454.0</v>
+        <v>151.5</v>
       </c>
       <c r="Q41" s="0" t="n">
-        <v>43241.0</v>
+        <v>14170.75</v>
       </c>
       <c r="R41" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera Lima</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="S41" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="T41" s="0" t="inlineStr">
         <is>
-          <t>fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+          <t>nataly_victoria16@yahoo.com</t>
         </is>
       </c>
       <c r="U41" s="0" t="inlineStr">
         <is>
-          <t>Francisco Javier Vera, Maria Fernanda Osorio Chavez</t>
+          <t>Victoria Medina</t>
         </is>
       </c>
       <c r="V41" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>Osom People - Play Is Sacred | Yucatan Jungle Camp (1 - 4 oct 2026)</t>
         </is>
       </c>
       <c r="W41" s="0"/>
@@ -4426,21 +4422,21 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:52</t>
+          <t>2026/04/18 18:51:21</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>2026/04/08 00:43:54</t>
+          <t>2026/04/18 18:51:23</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>822717931075648110592</t>
+          <t>822725726179188305920</t>
         </is>
       </c>
       <c r="D42" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
@@ -4459,12 +4455,12 @@
       </c>
       <c r="H42" s="0" t="inlineStr">
         <is>
-          <t>amex</t>
+          <t>visa</t>
         </is>
       </c>
       <c r="I42" s="0" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>9962</t>
         </is>
       </c>
       <c r="J42" s="0" t="n">
@@ -4474,46 +4470,46 @@
         <v>0.0</v>
       </c>
       <c r="L42" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="M42" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N42" s="0" t="n">
-        <v>45000.0</v>
+        <v>25500.0</v>
       </c>
       <c r="O42" s="0" t="n">
-        <v>1530.0</v>
+        <v>739.5</v>
       </c>
       <c r="P42" s="0" t="n">
-        <v>454.0</v>
+        <v>259.0</v>
       </c>
       <c r="Q42" s="0" t="n">
-        <v>43016.0</v>
+        <v>24501.5</v>
       </c>
       <c r="R42" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+          <t>Jonatan Oregon Mendez</t>
         </is>
       </c>
       <c r="S42" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="T42" s="0" t="inlineStr">
         <is>
-          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+          <t>johnoregon@live.com</t>
         </is>
       </c>
       <c r="U42" s="0" t="inlineStr">
         <is>
-          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+          <t>Jonatan Oregon</t>
         </is>
       </c>
       <c r="V42" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
         </is>
       </c>
       <c r="W42" s="0"/>
@@ -4531,21 +4527,21 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:06</t>
+          <t>2026/04/17 16:38:42</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 23:17:09</t>
+          <t>2026/04/17 16:38:44</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>822717887408069685248</t>
+          <t>822724934643911520256</t>
         </is>
       </c>
       <c r="D43" s="0" t="n">
-        <v>31500.0</v>
+        <v>70500.0</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
@@ -4569,7 +4565,7 @@
       </c>
       <c r="I43" s="0" t="inlineStr">
         <is>
-          <t>4006</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J43" s="0" t="n">
@@ -4579,46 +4575,46 @@
         <v>0.0</v>
       </c>
       <c r="L43" s="0" t="n">
-        <v>31500.0</v>
+        <v>70500.0</v>
       </c>
       <c r="M43" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N43" s="0" t="n">
-        <v>31500.0</v>
+        <v>70500.0</v>
       </c>
       <c r="O43" s="0" t="n">
-        <v>1071.0</v>
+        <v>2397.0</v>
       </c>
       <c r="P43" s="0" t="n">
-        <v>319.0</v>
+        <v>709.0</v>
       </c>
       <c r="Q43" s="0" t="n">
-        <v>30110.0</v>
+        <v>67394.0</v>
       </c>
       <c r="R43" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago</t>
+          <t>Marcela Alvarez Campos</t>
         </is>
       </c>
       <c r="S43" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com</t>
+          <t>marcela.ac@me.com</t>
         </is>
       </c>
       <c r="T43" s="0" t="inlineStr">
         <is>
-          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+          <t>marcela.ac@me.com, marcela.ac@me.com, marcela.ac@me.com</t>
         </is>
       </c>
       <c r="U43" s="0" t="inlineStr">
         <is>
-          <t>Eduardo Zago, Michelle Ralph</t>
+          <t>Marcela Alvarez Campos, Natalia Germenos Alvarez, Inés Germenos Alvarez</t>
         </is>
       </c>
       <c r="V43" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W43" s="0"/>
@@ -4636,21 +4632,21 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:57</t>
+          <t>2026/04/13 22:04:28</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 20:32:59</t>
+          <t>2026/04/13 22:04:30</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>822717804781623066624</t>
+          <t>822722199504844500992</t>
         </is>
       </c>
       <c r="D44" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
@@ -4674,7 +4670,7 @@
       </c>
       <c r="I44" s="0" t="inlineStr">
         <is>
-          <t>3513</t>
+          <t>4291</t>
         </is>
       </c>
       <c r="J44" s="0" t="n">
@@ -4684,46 +4680,46 @@
         <v>0.0</v>
       </c>
       <c r="L44" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="M44" s="0" t="n">
         <v>0.0</v>
       </c>
       <c r="N44" s="0" t="n">
-        <v>25500.0</v>
+        <v>45000.0</v>
       </c>
       <c r="O44" s="0" t="n">
-        <v>739.5</v>
+        <v>1305.0</v>
       </c>
       <c r="P44" s="0" t="n">
-        <v>259.0</v>
+        <v>454.0</v>
       </c>
       <c r="Q44" s="0" t="n">
-        <v>24501.5</v>
+        <v>43241.0</v>
       </c>
       <c r="R44" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>Carlos Mendoza</t>
         </is>
       </c>
       <c r="S44" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>mendoza.carlos.a@gmail.com</t>
         </is>
       </c>
       <c r="T44" s="0" t="inlineStr">
         <is>
-          <t>mateeomateeo@gmail.com</t>
+          <t>mendoza.carlos.a@gmail.com, elena.toral.o@gmail.com</t>
         </is>
       </c>
       <c r="U44" s="0" t="inlineStr">
         <is>
-          <t>Ana Maria Mateo Reyes</t>
+          <t>Carlos Mendoza, Maria Elena Ortal Ortega</t>
         </is>
       </c>
       <c r="V44" s="0" t="inlineStr">
         <is>
-          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+          <t>La Ventana Expedition Camp (28 mayo -31 mayo 2026)</t>
         </is>
       </c>
       <c r="W44" s="0"/>
@@ -4741,17 +4737,17 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:51</t>
+          <t>2026/04/13 19:26:45</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>2026/04/07 02:11:53</t>
+          <t>2026/04/13 19:26:47</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>822717250585584762880</t>
+          <t>822722120121735725056</t>
         </is>
       </c>
       <c r="D45" s="0" t="n">
@@ -4779,7 +4775,7 @@
       </c>
       <c r="I45" s="0" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="J45" s="0" t="n">
@@ -4808,22 +4804,22 @@
       </c>
       <c r="R45" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion</t>
+          <t>Ana paula Isaac</t>
         </is>
       </c>
       <c r="S45" s="0" t="inlineStr">
         <is>
-          <t>sofiacarrioncobian@hotmail.com</t>
+          <t>anapauisaac@gmail.com</t>
         </is>
       </c>
       <c r="T45" s="0" t="inlineStr">
         <is>
-          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+          <t>anapauisaac@gmail.com, gabriela@kahlio.com</t>
         </is>
       </c>
       <c r="U45" s="0" t="inlineStr">
         <is>
-          <t>Sofia Carrion, Ana María Carrion</t>
+          <t>Ana paula Isaac, Gabriela Vazquez</t>
         </is>
       </c>
       <c r="V45" s="0" t="inlineStr">
@@ -4838,6 +4834,531 @@
         </is>
       </c>
       <c r="Y45" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/09 04:55:14</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/09 04:55:16</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>822718782367677300736</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F46" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G46" s="0" t="inlineStr">
+        <is>
+          <t>apple_pay</t>
+        </is>
+      </c>
+      <c r="H46" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I46" s="0" t="inlineStr">
+        <is>
+          <t>7348</t>
+        </is>
+      </c>
+      <c r="J46" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K46" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L46" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M46" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N46" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O46" s="0" t="n">
+        <v>1305.0</v>
+      </c>
+      <c r="P46" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q46" s="0" t="n">
+        <v>43241.0</v>
+      </c>
+      <c r="R46" s="0" t="inlineStr">
+        <is>
+          <t>Francisco Javier Vera Lima</t>
+        </is>
+      </c>
+      <c r="S46" s="0" t="inlineStr">
+        <is>
+          <t>fjvera@vmodal.mx</t>
+        </is>
+      </c>
+      <c r="T46" s="0" t="inlineStr">
+        <is>
+          <t>fjvera@vmodal.mx, fjvera@vmodal.mx, fjvera@vmodal.mx</t>
+        </is>
+      </c>
+      <c r="U46" s="0" t="inlineStr">
+        <is>
+          <t>Francisco Javier Vera, Carlos Vera, Gabriela Vera</t>
+        </is>
+      </c>
+      <c r="V46" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W46" s="0"/>
+      <c r="X46" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y46" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:52</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/08 00:43:54</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>822717931075648110592</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F47" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G47" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H47" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I47" s="0" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="J47" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K47" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L47" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M47" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N47" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O47" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P47" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q47" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R47" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO RODRIGUEZ QUIROZ</t>
+        </is>
+      </c>
+      <c r="S47" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T47" s="0" t="inlineStr">
+        <is>
+          <t>mardoqueorq@hotmail.com, Lorerosa@hotmail.com</t>
+        </is>
+      </c>
+      <c r="U47" s="0" t="inlineStr">
+        <is>
+          <t>MARDOQUEO Rodriguez, Lorena Rodriguez</t>
+        </is>
+      </c>
+      <c r="V47" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W47" s="0"/>
+      <c r="X47" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y47" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:06</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 23:17:09</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>822717887408069685248</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F48" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G48" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H48" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I48" s="0" t="inlineStr">
+        <is>
+          <t>4006</t>
+        </is>
+      </c>
+      <c r="J48" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K48" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L48" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="M48" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N48" s="0" t="n">
+        <v>31500.0</v>
+      </c>
+      <c r="O48" s="0" t="n">
+        <v>1071.0</v>
+      </c>
+      <c r="P48" s="0" t="n">
+        <v>319.0</v>
+      </c>
+      <c r="Q48" s="0" t="n">
+        <v>30110.0</v>
+      </c>
+      <c r="R48" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago</t>
+        </is>
+      </c>
+      <c r="S48" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com</t>
+        </is>
+      </c>
+      <c r="T48" s="0" t="inlineStr">
+        <is>
+          <t>eddiezago500@gmail.com, michralph1@gmail.com</t>
+        </is>
+      </c>
+      <c r="U48" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Zago, Michelle Ralph</t>
+        </is>
+      </c>
+      <c r="V48" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W48" s="0"/>
+      <c r="X48" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y48" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:57</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 20:32:59</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>822717804781623066624</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F49" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G49" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H49" s="0" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="I49" s="0" t="inlineStr">
+        <is>
+          <t>3513</t>
+        </is>
+      </c>
+      <c r="J49" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K49" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L49" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="M49" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N49" s="0" t="n">
+        <v>25500.0</v>
+      </c>
+      <c r="O49" s="0" t="n">
+        <v>739.5</v>
+      </c>
+      <c r="P49" s="0" t="n">
+        <v>259.0</v>
+      </c>
+      <c r="Q49" s="0" t="n">
+        <v>24501.5</v>
+      </c>
+      <c r="R49" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="S49" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="T49" s="0" t="inlineStr">
+        <is>
+          <t>mateeomateeo@gmail.com</t>
+        </is>
+      </c>
+      <c r="U49" s="0" t="inlineStr">
+        <is>
+          <t>Ana Maria Mateo Reyes</t>
+        </is>
+      </c>
+      <c r="V49" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (4 junio - 7 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W49" s="0"/>
+      <c r="X49" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y49" s="0" t="inlineStr">
+        <is>
+          <t>daniel@akampa.mx</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:51</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>2026/04/07 02:11:53</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>822717250585584762880</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="E50" s="0" t="inlineStr">
+        <is>
+          <t>Successful</t>
+        </is>
+      </c>
+      <c r="F50" s="0" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="G50" s="0" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H50" s="0" t="inlineStr">
+        <is>
+          <t>amex</t>
+        </is>
+      </c>
+      <c r="I50" s="0" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="J50" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K50" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L50" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="M50" s="0" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N50" s="0" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="O50" s="0" t="n">
+        <v>1530.0</v>
+      </c>
+      <c r="P50" s="0" t="n">
+        <v>454.0</v>
+      </c>
+      <c r="Q50" s="0" t="n">
+        <v>43016.0</v>
+      </c>
+      <c r="R50" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion</t>
+        </is>
+      </c>
+      <c r="S50" s="0" t="inlineStr">
+        <is>
+          <t>sofiacarrioncobian@hotmail.com</t>
+        </is>
+      </c>
+      <c r="T50" s="0" t="inlineStr">
+        <is>
+          <t>Sofiacarrioncobian@hotmail.com, Anamaria.carcob@gmail.com</t>
+        </is>
+      </c>
+      <c r="U50" s="0" t="inlineStr">
+        <is>
+          <t>Sofia Carrion, Ana María Carrion</t>
+        </is>
+      </c>
+      <c r="V50" s="0" t="inlineStr">
+        <is>
+          <t>La Ventana Expedition Camp (11 junio - 14 junio 2026)</t>
+        </is>
+      </c>
+      <c r="W50" s="0"/>
+      <c r="X50" s="0" t="inlineStr">
+        <is>
+          <t>Akampa</t>
+        </is>
+      </c>
+      <c r="Y50" s="0" t="inlineStr">
         <is>
           <t>daniel@akampa.mx</t>
         </is>

</xml_diff>